<commit_message>
Improve ArchIvory editorial workbook workflow
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/archivory-editorial/ArchIvory Editorial Workbook.xlsx
+++ b/outputs/archivory-editorial/ArchIvory Editorial Workbook.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Placements" sheetId="1" r:id="Rb497896396ec40e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content" sheetId="2" r:id="R254823be89494ef6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="3" r:id="Rca64618e21334040"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timelines" sheetId="4" r:id="Refd42bd4033144b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rooms" sheetId="5" r:id="Rfb2de58daa3c49e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slots" sheetId="6" r:id="R4141fb30fd9a407b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection" sheetId="7" r:id="Rcd34d11aaf5b466c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="R267053c941224fec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Placements" sheetId="1" r:id="R59f823f6830344ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content" sheetId="2" r:id="Rad978ebcbde54700"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="3" r:id="R0a2ab727074e4c55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timelines" sheetId="4" r:id="Ref700006386f427b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rooms" sheetId="5" r:id="R2d53f8f3db174a8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slots" sheetId="6" r:id="R62f8395dd30b46e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection" sheetId="7" r:id="R509ed4a287c54002"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="R3996e973189646a2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -162,11 +162,32 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="1">
+  <x:dxfs count="4">
     <x:dxf>
       <x:fill>
         <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFFE2A8"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFF4B4B4"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFF4B4B4"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFF4B4B4"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -175,17 +196,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PlacementsTable" displayName="PlacementsTable" ref="A1:I63" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="9">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PlacementsTable" displayName="PlacementsTable" ref="A1:K63" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="11">
     <x:tableColumn id="1" name="placement_id"/>
     <x:tableColumn id="2" name="slot_id"/>
     <x:tableColumn id="3" name="content_id"/>
     <x:tableColumn id="4" name="content_type"/>
     <x:tableColumn id="5" name="sort_order"/>
     <x:tableColumn id="6" name="published"/>
-    <x:tableColumn id="7" name="Room (automatic)"/>
-    <x:tableColumn id="8" name="Location (automatic)"/>
-    <x:tableColumn id="9" name="Content title (automatic)"/>
+    <x:tableColumn id="7" name="Room ID (automatic)"/>
+    <x:tableColumn id="8" name="Room name (automatic)"/>
+    <x:tableColumn id="9" name="Location (automatic)"/>
+    <x:tableColumn id="10" name="Supported type (automatic)"/>
+    <x:tableColumn id="11" name="Capacity (automatic)"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -506,6 +529,8 @@
     <x:col min="7" max="7" width="40" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="40" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="40" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="40" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="40" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
@@ -528,13 +553,19 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="G1" s="10" t="str">
-        <x:v>Room (automatic)</x:v>
+        <x:v>Room ID (automatic)</x:v>
       </x:c>
       <x:c r="H1" s="10" t="str">
+        <x:v>Room name (automatic)</x:v>
+      </x:c>
+      <x:c r="I1" s="10" t="str">
         <x:v>Location (automatic)</x:v>
       </x:c>
-      <x:c r="I1" s="10" t="str">
-        <x:v>Content title (automatic)</x:v>
+      <x:c r="J1" s="10" t="str">
+        <x:v>Supported type (automatic)</x:v>
+      </x:c>
+      <x:c r="K1" s="10" t="str">
+        <x:v>Capacity (automatic)</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
@@ -561,12 +592,20 @@
         <x:v>gallery</x:v>
       </x:c>
       <x:c r="H2" s="15" t="str">
+        <x:f>IF(G2="","",IFNA(VLOOKUP(G2,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Gallery</x:v>
+      </x:c>
+      <x:c r="I2" s="15" t="str">
         <x:f>IF(B2="","",IFNA(VLOOKUP(B2,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Gallery introduction</x:v>
       </x:c>
-      <x:c r="I2" s="15" t="str">
-        <x:f>IF(C2="","Choose content",IF(D2="timeline",IFNA(VLOOKUP(C2,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C2,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Gallery Intro</x:v>
+      <x:c r="J2" s="15" t="str">
+        <x:f>IF(B2="","",IFNA(VLOOKUP(B2,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="K2" s="15" t="n">
+        <x:f>IF(B2="","",IFNA(VLOOKUP(B2,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
@@ -593,12 +632,20 @@
         <x:v>conservation_lab</x:v>
       </x:c>
       <x:c r="H3" s="15" t="str">
+        <x:f>IF(G3="","",IFNA(VLOOKUP(G3,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Conservation Lab</x:v>
+      </x:c>
+      <x:c r="I3" s="15" t="str">
         <x:f>IF(B3="","",IFNA(VLOOKUP(B3,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Conservation Lab introduction</x:v>
       </x:c>
-      <x:c r="I3" s="15" t="str">
-        <x:f>IF(C3="","Choose content",IF(D3="timeline",IFNA(VLOOKUP(C3,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C3,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Conservation Lab Intro</x:v>
+      <x:c r="J3" s="15" t="str">
+        <x:f>IF(B3="","",IFNA(VLOOKUP(B3,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="K3" s="15" t="n">
+        <x:f>IF(B3="","",IFNA(VLOOKUP(B3,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
@@ -625,12 +672,20 @@
         <x:v>vestibule</x:v>
       </x:c>
       <x:c r="H4" s="15" t="str">
+        <x:f>IF(G4="","",IFNA(VLOOKUP(G4,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Vestibule</x:v>
+      </x:c>
+      <x:c r="I4" s="15" t="str">
         <x:f>IF(B4="","",IFNA(VLOOKUP(B4,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Welcome and check-in</x:v>
       </x:c>
-      <x:c r="I4" s="15" t="str">
-        <x:f>IF(C4="","Choose content",IF(D4="timeline",IFNA(VLOOKUP(C4,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C4,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Welcome to ArchIvory</x:v>
+      <x:c r="J4" s="15" t="str">
+        <x:f>IF(B4="","",IFNA(VLOOKUP(B4,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="K4" s="15" t="n">
+        <x:f>IF(B4="","",IFNA(VLOOKUP(B4,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
@@ -657,12 +712,20 @@
         <x:v>gallery</x:v>
       </x:c>
       <x:c r="H5" s="15" t="str">
+        <x:f>IF(G5="","",IFNA(VLOOKUP(G5,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Gallery</x:v>
+      </x:c>
+      <x:c r="I5" s="15" t="str">
         <x:f>IF(B5="","",IFNA(VLOOKUP(B5,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Near left-wall relief</x:v>
       </x:c>
-      <x:c r="I5" s="15" t="str">
-        <x:f>IF(C5="","Choose content",IF(D5="timeline",IFNA(VLOOKUP(C5,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C5,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Illustrated relief — identity unverified</x:v>
+      <x:c r="J5" s="15" t="str">
+        <x:f>IF(B5="","",IFNA(VLOOKUP(B5,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K5" s="15" t="n">
+        <x:f>IF(B5="","",IFNA(VLOOKUP(B5,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
@@ -689,12 +752,20 @@
         <x:v>gallery</x:v>
       </x:c>
       <x:c r="H6" s="15" t="str">
+        <x:f>IF(G6="","",IFNA(VLOOKUP(G6,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Gallery</x:v>
+      </x:c>
+      <x:c r="I6" s="15" t="str">
         <x:f>IF(B6="","",IFNA(VLOOKUP(B6,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Near left-wall relief</x:v>
       </x:c>
-      <x:c r="I6" s="15" t="str">
-        <x:f>IF(C6="","Choose content",IF(D6="timeline",IFNA(VLOOKUP(C6,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C6,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Susanna and the Elders</x:v>
+      <x:c r="J6" s="15" t="str">
+        <x:f>IF(B6="","",IFNA(VLOOKUP(B6,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K6" s="15" t="n">
+        <x:f>IF(B6="","",IFNA(VLOOKUP(B6,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
@@ -721,12 +792,20 @@
         <x:v>gallery</x:v>
       </x:c>
       <x:c r="H7" s="15" t="str">
+        <x:f>IF(G7="","",IFNA(VLOOKUP(G7,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Gallery</x:v>
+      </x:c>
+      <x:c r="I7" s="15" t="str">
         <x:f>IF(B7="","",IFNA(VLOOKUP(B7,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Far left-wall relief</x:v>
       </x:c>
-      <x:c r="I7" s="15" t="str">
-        <x:f>IF(C7="","Choose content",IF(D7="timeline",IFNA(VLOOKUP(C7,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C7,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Illustrated relief — identity unverified</x:v>
+      <x:c r="J7" s="15" t="str">
+        <x:f>IF(B7="","",IFNA(VLOOKUP(B7,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K7" s="15" t="n">
+        <x:f>IF(B7="","",IFNA(VLOOKUP(B7,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
@@ -753,12 +832,20 @@
         <x:v>gallery</x:v>
       </x:c>
       <x:c r="H8" s="15" t="str">
+        <x:f>IF(G8="","",IFNA(VLOOKUP(G8,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Gallery</x:v>
+      </x:c>
+      <x:c r="I8" s="15" t="str">
         <x:f>IF(B8="","",IFNA(VLOOKUP(B8,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Far left-wall relief</x:v>
       </x:c>
-      <x:c r="I8" s="15" t="str">
-        <x:f>IF(C8="","Choose content",IF(D8="timeline",IFNA(VLOOKUP(C8,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C8,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Barberini Ivory</x:v>
+      <x:c r="J8" s="15" t="str">
+        <x:f>IF(B8="","",IFNA(VLOOKUP(B8,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K8" s="15" t="n">
+        <x:f>IF(B8="","",IFNA(VLOOKUP(B8,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
@@ -785,12 +872,20 @@
         <x:v>gallery</x:v>
       </x:c>
       <x:c r="H9" s="15" t="str">
+        <x:f>IF(G9="","",IFNA(VLOOKUP(G9,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Gallery</x:v>
+      </x:c>
+      <x:c r="I9" s="15" t="str">
         <x:f>IF(B9="","",IFNA(VLOOKUP(B9,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Front glass case</x:v>
       </x:c>
-      <x:c r="I9" s="15" t="str">
-        <x:f>IF(C9="","Choose content",IF(D9="timeline",IFNA(VLOOKUP(C9,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C9,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Illustrated folding fan</x:v>
+      <x:c r="J9" s="15" t="str">
+        <x:f>IF(B9="","",IFNA(VLOOKUP(B9,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K9" s="15" t="n">
+        <x:f>IF(B9="","",IFNA(VLOOKUP(B9,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
@@ -817,12 +912,20 @@
         <x:v>gallery</x:v>
       </x:c>
       <x:c r="H10" s="15" t="str">
+        <x:f>IF(G10="","",IFNA(VLOOKUP(G10,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Gallery</x:v>
+      </x:c>
+      <x:c r="I10" s="15" t="str">
         <x:f>IF(B10="","",IFNA(VLOOKUP(B10,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Small rear-wall frame</x:v>
       </x:c>
-      <x:c r="I10" s="15" t="str">
-        <x:f>IF(C10="","Choose content",IF(D10="timeline",IFNA(VLOOKUP(C10,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C10,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Roman Wall Sconce</x:v>
+      <x:c r="J10" s="15" t="str">
+        <x:f>IF(B10="","",IFNA(VLOOKUP(B10,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="K10" s="15" t="n">
+        <x:f>IF(B10="","",IFNA(VLOOKUP(B10,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
@@ -849,12 +952,20 @@
         <x:v>conservation_lab</x:v>
       </x:c>
       <x:c r="H11" s="15" t="str">
+        <x:f>IF(G11="","",IFNA(VLOOKUP(G11,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Conservation Lab</x:v>
+      </x:c>
+      <x:c r="I11" s="15" t="str">
         <x:f>IF(B11="","",IFNA(VLOOKUP(B11,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Central ivories collection</x:v>
       </x:c>
-      <x:c r="I11" s="15" t="str">
-        <x:f>IF(C11="","Choose content",IF(D11="timeline",IFNA(VLOOKUP(C11,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C11,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>IU Eskenazi Museum Ivories</x:v>
+      <x:c r="J11" s="15" t="str">
+        <x:f>IF(B11="","",IFNA(VLOOKUP(B11,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K11" s="15" t="n">
+        <x:f>IF(B11="","",IFNA(VLOOKUP(B11,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="34" customHeight="1">
@@ -881,12 +992,20 @@
         <x:v>conservation_lab</x:v>
       </x:c>
       <x:c r="H12" s="15" t="str">
+        <x:f>IF(G12="","",IFNA(VLOOKUP(G12,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Conservation Lab</x:v>
+      </x:c>
+      <x:c r="I12" s="15" t="str">
         <x:f>IF(B12="","",IFNA(VLOOKUP(B12,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Ivory Through the Ages</x:v>
       </x:c>
-      <x:c r="I12" s="15" t="str">
-        <x:f>IF(C12="","Choose content",IF(D12="timeline",IFNA(VLOOKUP(C12,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C12,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Conservation Lab</x:v>
+      <x:c r="J12" s="15" t="str">
+        <x:f>IF(B12="","",IFNA(VLOOKUP(B12,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>timeline</x:v>
+      </x:c>
+      <x:c r="K12" s="15" t="n">
+        <x:f>IF(B12="","",IFNA(VLOOKUP(B12,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="34" customHeight="1">
@@ -913,12 +1032,20 @@
         <x:v>conservation_lab</x:v>
       </x:c>
       <x:c r="H13" s="15" t="str">
+        <x:f>IF(G13="","",IFNA(VLOOKUP(G13,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Conservation Lab</x:v>
+      </x:c>
+      <x:c r="I13" s="15" t="str">
         <x:f>IF(B13="","",IFNA(VLOOKUP(B13,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Rear analysis workbench</x:v>
       </x:c>
-      <x:c r="I13" s="15" t="str">
-        <x:f>IF(C13="","Choose content",IF(D13="timeline",IFNA(VLOOKUP(C13,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C13,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Analysis workbench</x:v>
+      <x:c r="J13" s="15" t="str">
+        <x:f>IF(B13="","",IFNA(VLOOKUP(B13,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="K13" s="15" t="n">
+        <x:f>IF(B13="","",IFNA(VLOOKUP(B13,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="34" customHeight="1">
@@ -945,12 +1072,20 @@
         <x:v>historical_society</x:v>
       </x:c>
       <x:c r="H14" s="15" t="str">
+        <x:f>IF(G14="","",IFNA(VLOOKUP(G14,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Historical Society</x:v>
+      </x:c>
+      <x:c r="I14" s="15" t="str">
         <x:f>IF(B14="","",IFNA(VLOOKUP(B14,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Local Lives</x:v>
       </x:c>
-      <x:c r="I14" s="15" t="str">
-        <x:f>IF(C14="","Choose content",IF(D14="timeline",IFNA(VLOOKUP(C14,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C14,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Historical Society</x:v>
+      <x:c r="J14" s="15" t="str">
+        <x:f>IF(B14="","",IFNA(VLOOKUP(B14,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>timeline</x:v>
+      </x:c>
+      <x:c r="K14" s="15" t="n">
+        <x:f>IF(B14="","",IFNA(VLOOKUP(B14,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="34" customHeight="1">
@@ -977,12 +1112,20 @@
         <x:v>historical_society</x:v>
       </x:c>
       <x:c r="H15" s="15" t="str">
+        <x:f>IF(G15="","",IFNA(VLOOKUP(G15,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Historical Society</x:v>
+      </x:c>
+      <x:c r="I15" s="15" t="str">
         <x:f>IF(B15="","",IFNA(VLOOKUP(B15,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Piano</x:v>
       </x:c>
-      <x:c r="I15" s="15" t="str">
-        <x:f>IF(C15="","Choose content",IF(D15="timeline",IFNA(VLOOKUP(C15,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C15,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Piano</x:v>
+      <x:c r="J15" s="15" t="str">
+        <x:f>IF(B15="","",IFNA(VLOOKUP(B15,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="K15" s="15" t="n">
+        <x:f>IF(B15="","",IFNA(VLOOKUP(B15,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="34" customHeight="1">
@@ -1009,12 +1152,20 @@
         <x:v>historical_society</x:v>
       </x:c>
       <x:c r="H16" s="15" t="str">
+        <x:f>IF(G16="","",IFNA(VLOOKUP(G16,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Historical Society</x:v>
+      </x:c>
+      <x:c r="I16" s="15" t="str">
         <x:f>IF(B16="","",IFNA(VLOOKUP(B16,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Billiards table</x:v>
       </x:c>
-      <x:c r="I16" s="15" t="str">
-        <x:f>IF(C16="","Choose content",IF(D16="timeline",IFNA(VLOOKUP(C16,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C16,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Billiards table</x:v>
+      <x:c r="J16" s="15" t="str">
+        <x:f>IF(B16="","",IFNA(VLOOKUP(B16,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="K16" s="15" t="n">
+        <x:f>IF(B16="","",IFNA(VLOOKUP(B16,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="34" customHeight="1">
@@ -1041,12 +1192,20 @@
         <x:v>attic</x:v>
       </x:c>
       <x:c r="H17" s="15" t="str">
+        <x:f>IF(G17="","",IFNA(VLOOKUP(G17,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Attic</x:v>
+      </x:c>
+      <x:c r="I17" s="15" t="str">
         <x:f>IF(B17="","",IFNA(VLOOKUP(B17,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Family Traces</x:v>
       </x:c>
-      <x:c r="I17" s="15" t="str">
-        <x:f>IF(C17="","Choose content",IF(D17="timeline",IFNA(VLOOKUP(C17,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C17,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Attic</x:v>
+      <x:c r="J17" s="15" t="str">
+        <x:f>IF(B17="","",IFNA(VLOOKUP(B17,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>timeline</x:v>
+      </x:c>
+      <x:c r="K17" s="15" t="n">
+        <x:f>IF(B17="","",IFNA(VLOOKUP(B17,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="34" customHeight="1">
@@ -1073,12 +1232,20 @@
         <x:v>natural_history</x:v>
       </x:c>
       <x:c r="H18" s="15" t="str">
+        <x:f>IF(G18="","",IFNA(VLOOKUP(G18,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Natural History Museum</x:v>
+      </x:c>
+      <x:c r="I18" s="15" t="str">
         <x:f>IF(B18="","",IFNA(VLOOKUP(B18,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Tusk specimen</x:v>
       </x:c>
-      <x:c r="I18" s="15" t="str">
-        <x:f>IF(C18="","Choose content",IF(D18="timeline",IFNA(VLOOKUP(C18,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C18,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Elephant tusk</x:v>
+      <x:c r="J18" s="15" t="str">
+        <x:f>IF(B18="","",IFNA(VLOOKUP(B18,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="K18" s="15" t="n">
+        <x:f>IF(B18="","",IFNA(VLOOKUP(B18,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="34" customHeight="1">
@@ -1105,12 +1272,20 @@
         <x:v>natural_history</x:v>
       </x:c>
       <x:c r="H19" s="15" t="str">
+        <x:f>IF(G19="","",IFNA(VLOOKUP(G19,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Natural History Museum</x:v>
+      </x:c>
+      <x:c r="I19" s="15" t="str">
         <x:f>IF(B19="","",IFNA(VLOOKUP(B19,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Specimen label</x:v>
       </x:c>
-      <x:c r="I19" s="15" t="str">
-        <x:f>IF(C19="","Choose content",IF(D19="timeline",IFNA(VLOOKUP(C19,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C19,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Elephant tusk</x:v>
+      <x:c r="J19" s="15" t="str">
+        <x:f>IF(B19="","",IFNA(VLOOKUP(B19,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="K19" s="15" t="n">
+        <x:f>IF(B19="","",IFNA(VLOOKUP(B19,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="34" customHeight="1">
@@ -1137,12 +1312,20 @@
         <x:v>natural_history</x:v>
       </x:c>
       <x:c r="H20" s="15" t="str">
+        <x:f>IF(G20="","",IFNA(VLOOKUP(G20,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Natural History Museum</x:v>
+      </x:c>
+      <x:c r="I20" s="15" t="str">
         <x:f>IF(B20="","",IFNA(VLOOKUP(B20,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Elephant interpretation panel</x:v>
       </x:c>
-      <x:c r="I20" s="15" t="str">
-        <x:f>IF(C20="","Choose content",IF(D20="timeline",IFNA(VLOOKUP(C20,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C20,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Natural History Intro</x:v>
+      <x:c r="J20" s="15" t="str">
+        <x:f>IF(B20="","",IFNA(VLOOKUP(B20,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="K20" s="15" t="n">
+        <x:f>IF(B20="","",IFNA(VLOOKUP(B20,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="34" customHeight="1">
@@ -1169,12 +1352,20 @@
         <x:v>natural_history</x:v>
       </x:c>
       <x:c r="H21" s="15" t="str">
+        <x:f>IF(G21="","",IFNA(VLOOKUP(G21,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Natural History Museum</x:v>
+      </x:c>
+      <x:c r="I21" s="15" t="str">
         <x:f>IF(B21="","",IFNA(VLOOKUP(B21,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Wall map</x:v>
       </x:c>
-      <x:c r="I21" s="15" t="str">
-        <x:f>IF(C21="","Choose content",IF(D21="timeline",IFNA(VLOOKUP(C21,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C21,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>World map</x:v>
+      <x:c r="J21" s="15" t="str">
+        <x:f>IF(B21="","",IFNA(VLOOKUP(B21,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="K21" s="15" t="n">
+        <x:f>IF(B21="","",IFNA(VLOOKUP(B21,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="34" customHeight="1">
@@ -1201,12 +1392,20 @@
         <x:v>natural_history</x:v>
       </x:c>
       <x:c r="H22" s="15" t="str">
+        <x:f>IF(G22="","",IFNA(VLOOKUP(G22,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Natural History Museum</x:v>
+      </x:c>
+      <x:c r="I22" s="15" t="str">
         <x:f>IF(B22="","",IFNA(VLOOKUP(B22,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Deep-time explorer</x:v>
       </x:c>
-      <x:c r="I22" s="15" t="str">
-        <x:f>IF(C22="","Choose content",IF(D22="timeline",IFNA(VLOOKUP(C22,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C22,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Deep-time explorer</x:v>
+      <x:c r="J22" s="15" t="str">
+        <x:f>IF(B22="","",IFNA(VLOOKUP(B22,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="K22" s="15" t="n">
+        <x:f>IF(B22="","",IFNA(VLOOKUP(B22,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="34" customHeight="1">
@@ -1233,12 +1432,20 @@
         <x:v>natural_history</x:v>
       </x:c>
       <x:c r="H23" s="15" t="str">
+        <x:f>IF(G23="","",IFNA(VLOOKUP(G23,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Natural History Museum</x:v>
+      </x:c>
+      <x:c r="I23" s="15" t="str">
         <x:f>IF(B23="","",IFNA(VLOOKUP(B23,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Habitation map within explorer</x:v>
       </x:c>
-      <x:c r="I23" s="15" t="str">
-        <x:f>IF(C23="","Choose content",IF(D23="timeline",IFNA(VLOOKUP(C23,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C23,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Habitation map</x:v>
+      <x:c r="J23" s="15" t="str">
+        <x:f>IF(B23="","",IFNA(VLOOKUP(B23,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="K23" s="15" t="n">
+        <x:f>IF(B23="","",IFNA(VLOOKUP(B23,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="34" customHeight="1">
@@ -1265,12 +1472,20 @@
         <x:v>natural_history</x:v>
       </x:c>
       <x:c r="H24" s="15" t="str">
+        <x:f>IF(G24="","",IFNA(VLOOKUP(G24,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Natural History Museum</x:v>
+      </x:c>
+      <x:c r="I24" s="15" t="str">
         <x:f>IF(B24="","",IFNA(VLOOKUP(B24,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Arrange the evidence</x:v>
       </x:c>
-      <x:c r="I24" s="15" t="str">
-        <x:f>IF(C24="","Choose content",IF(D24="timeline",IFNA(VLOOKUP(C24,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C24,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Natural History Museum</x:v>
+      <x:c r="J24" s="15" t="str">
+        <x:f>IF(B24="","",IFNA(VLOOKUP(B24,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>timeline</x:v>
+      </x:c>
+      <x:c r="K24" s="15" t="n">
+        <x:f>IF(B24="","",IFNA(VLOOKUP(B24,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="34" customHeight="1">
@@ -1297,12 +1512,20 @@
         <x:v>natural_history</x:v>
       </x:c>
       <x:c r="H25" s="15" t="str">
+        <x:f>IF(G25="","",IFNA(VLOOKUP(G25,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Natural History Museum</x:v>
+      </x:c>
+      <x:c r="I25" s="15" t="str">
         <x:f>IF(B25="","",IFNA(VLOOKUP(B25,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Ivory inquiry</x:v>
       </x:c>
-      <x:c r="I25" s="15" t="str">
-        <x:f>IF(C25="","Choose content",IF(D25="timeline",IFNA(VLOOKUP(C25,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C25,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Ivory Inquiry Terminal</x:v>
+      <x:c r="J25" s="15" t="str">
+        <x:f>IF(B25="","",IFNA(VLOOKUP(B25,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="K25" s="15" t="n">
+        <x:f>IF(B25="","",IFNA(VLOOKUP(B25,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="34" customHeight="1">
@@ -1329,12 +1552,20 @@
         <x:v>conservators_office</x:v>
       </x:c>
       <x:c r="H26" s="15" t="str">
+        <x:f>IF(G26="","",IFNA(VLOOKUP(G26,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Conservator's Office</x:v>
+      </x:c>
+      <x:c r="I26" s="15" t="str">
         <x:f>IF(B26="","",IFNA(VLOOKUP(B26,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Desk terminal</x:v>
       </x:c>
-      <x:c r="I26" s="15" t="str">
-        <x:f>IF(C26="","Choose content",IF(D26="timeline",IFNA(VLOOKUP(C26,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C26,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Curation terminal</x:v>
+      <x:c r="J26" s="15" t="str">
+        <x:f>IF(B26="","",IFNA(VLOOKUP(B26,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="K26" s="15" t="n">
+        <x:f>IF(B26="","",IFNA(VLOOKUP(B26,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="34" customHeight="1">
@@ -1361,12 +1592,20 @@
         <x:v>conservators_office</x:v>
       </x:c>
       <x:c r="H27" s="15" t="str">
+        <x:f>IF(G27="","",IFNA(VLOOKUP(G27,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Conservator's Office</x:v>
+      </x:c>
+      <x:c r="I27" s="15" t="str">
         <x:f>IF(B27="","",IFNA(VLOOKUP(B27,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Elephant wall panel</x:v>
       </x:c>
-      <x:c r="I27" s="15" t="str">
-        <x:f>IF(C27="","Choose content",IF(D27="timeline",IFNA(VLOOKUP(C27,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C27,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Conservators Office Intro</x:v>
+      <x:c r="J27" s="15" t="str">
+        <x:f>IF(B27="","",IFNA(VLOOKUP(B27,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="K27" s="15" t="n">
+        <x:f>IF(B27="","",IFNA(VLOOKUP(B27,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="34" customHeight="1">
@@ -1393,12 +1632,20 @@
         <x:v>lab</x:v>
       </x:c>
       <x:c r="H28" s="15" t="str">
+        <x:f>IF(G28="","",IFNA(VLOOKUP(G28,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Lab</x:v>
+      </x:c>
+      <x:c r="I28" s="15" t="str">
         <x:f>IF(B28="","",IFNA(VLOOKUP(B28,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Attic access context</x:v>
       </x:c>
-      <x:c r="I28" s="15" t="str">
-        <x:f>IF(C28="","Choose content",IF(D28="timeline",IFNA(VLOOKUP(C28,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C28,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Attic investigations</x:v>
+      <x:c r="J28" s="15" t="str">
+        <x:f>IF(B28="","",IFNA(VLOOKUP(B28,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="K28" s="15" t="n">
+        <x:f>IF(B28="","",IFNA(VLOOKUP(B28,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="34" customHeight="1">
@@ -1423,12 +1670,20 @@
         <x:v>historical_society</x:v>
       </x:c>
       <x:c r="H29" s="15" t="str">
+        <x:f>IF(G29="","",IFNA(VLOOKUP(G29,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Historical Society</x:v>
+      </x:c>
+      <x:c r="I29" s="15" t="str">
         <x:f>IF(B29="","",IFNA(VLOOKUP(B29,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Historical Society introduction</x:v>
       </x:c>
-      <x:c r="I29" s="15" t="str">
-        <x:f>IF(C29="","Choose content",IF(D29="timeline",IFNA(VLOOKUP(C29,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C29,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J29" s="15" t="str">
+        <x:f>IF(B29="","",IFNA(VLOOKUP(B29,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="K29" s="15" t="n">
+        <x:f>IF(B29="","",IFNA(VLOOKUP(B29,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="34" customHeight="1">
@@ -1453,12 +1708,20 @@
         <x:v>attic</x:v>
       </x:c>
       <x:c r="H30" s="15" t="str">
+        <x:f>IF(G30="","",IFNA(VLOOKUP(G30,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Attic</x:v>
+      </x:c>
+      <x:c r="I30" s="15" t="str">
         <x:f>IF(B30="","",IFNA(VLOOKUP(B30,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Attic introduction</x:v>
       </x:c>
-      <x:c r="I30" s="15" t="str">
-        <x:f>IF(C30="","Choose content",IF(D30="timeline",IFNA(VLOOKUP(C30,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C30,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J30" s="15" t="str">
+        <x:f>IF(B30="","",IFNA(VLOOKUP(B30,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="K30" s="15" t="n">
+        <x:f>IF(B30="","",IFNA(VLOOKUP(B30,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="34" customHeight="1">
@@ -1483,12 +1746,20 @@
         <x:v>natural_history</x:v>
       </x:c>
       <x:c r="H31" s="15" t="str">
+        <x:f>IF(G31="","",IFNA(VLOOKUP(G31,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Natural History Museum</x:v>
+      </x:c>
+      <x:c r="I31" s="15" t="str">
         <x:f>IF(B31="","",IFNA(VLOOKUP(B31,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Natural History Museum introduction</x:v>
       </x:c>
-      <x:c r="I31" s="15" t="str">
-        <x:f>IF(C31="","Choose content",IF(D31="timeline",IFNA(VLOOKUP(C31,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C31,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J31" s="15" t="str">
+        <x:f>IF(B31="","",IFNA(VLOOKUP(B31,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="K31" s="15" t="n">
+        <x:f>IF(B31="","",IFNA(VLOOKUP(B31,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="34" customHeight="1">
@@ -1513,12 +1784,20 @@
         <x:v>conservators_office</x:v>
       </x:c>
       <x:c r="H32" s="15" t="str">
+        <x:f>IF(G32="","",IFNA(VLOOKUP(G32,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Conservator's Office</x:v>
+      </x:c>
+      <x:c r="I32" s="15" t="str">
         <x:f>IF(B32="","",IFNA(VLOOKUP(B32,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Conservator's Office introduction</x:v>
       </x:c>
-      <x:c r="I32" s="15" t="str">
-        <x:f>IF(C32="","Choose content",IF(D32="timeline",IFNA(VLOOKUP(C32,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C32,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J32" s="15" t="str">
+        <x:f>IF(B32="","",IFNA(VLOOKUP(B32,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="K32" s="15" t="n">
+        <x:f>IF(B32="","",IFNA(VLOOKUP(B32,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="34" customHeight="1">
@@ -1543,12 +1822,20 @@
         <x:v>lab</x:v>
       </x:c>
       <x:c r="H33" s="15" t="str">
+        <x:f>IF(G33="","",IFNA(VLOOKUP(G33,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Lab</x:v>
+      </x:c>
+      <x:c r="I33" s="15" t="str">
         <x:f>IF(B33="","",IFNA(VLOOKUP(B33,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Lab introduction</x:v>
       </x:c>
-      <x:c r="I33" s="15" t="str">
-        <x:f>IF(C33="","Choose content",IF(D33="timeline",IFNA(VLOOKUP(C33,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C33,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J33" s="15" t="str">
+        <x:f>IF(B33="","",IFNA(VLOOKUP(B33,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="K33" s="15" t="n">
+        <x:f>IF(B33="","",IFNA(VLOOKUP(B33,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="34" customHeight="1">
@@ -1573,12 +1860,20 @@
         <x:v>gallery</x:v>
       </x:c>
       <x:c r="H34" s="15" t="str">
+        <x:f>IF(G34="","",IFNA(VLOOKUP(G34,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Gallery</x:v>
+      </x:c>
+      <x:c r="I34" s="15" t="str">
         <x:f>IF(B34="","",IFNA(VLOOKUP(B34,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Rear round display</x:v>
       </x:c>
-      <x:c r="I34" s="15" t="str">
-        <x:f>IF(C34="","Choose content",IF(D34="timeline",IFNA(VLOOKUP(C34,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C34,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J34" s="15" t="str">
+        <x:f>IF(B34="","",IFNA(VLOOKUP(B34,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K34" s="15" t="n">
+        <x:f>IF(B34="","",IFNA(VLOOKUP(B34,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="34" customHeight="1">
@@ -1603,12 +1898,20 @@
         <x:v>historical_society</x:v>
       </x:c>
       <x:c r="H35" s="15" t="str">
+        <x:f>IF(G35="","",IFNA(VLOOKUP(G35,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Historical Society</x:v>
+      </x:c>
+      <x:c r="I35" s="15" t="str">
         <x:f>IF(B35="","",IFNA(VLOOKUP(B35,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Window-side case</x:v>
       </x:c>
-      <x:c r="I35" s="15" t="str">
-        <x:f>IF(C35="","Choose content",IF(D35="timeline",IFNA(VLOOKUP(C35,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C35,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J35" s="15" t="str">
+        <x:f>IF(B35="","",IFNA(VLOOKUP(B35,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K35" s="15" t="n">
+        <x:f>IF(B35="","",IFNA(VLOOKUP(B35,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="34" customHeight="1">
@@ -1633,12 +1936,20 @@
         <x:v>historical_society</x:v>
       </x:c>
       <x:c r="H36" s="15" t="str">
+        <x:f>IF(G36="","",IFNA(VLOOKUP(G36,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Historical Society</x:v>
+      </x:c>
+      <x:c r="I36" s="15" t="str">
         <x:f>IF(B36="","",IFNA(VLOOKUP(B36,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Foreground-right case</x:v>
       </x:c>
-      <x:c r="I36" s="15" t="str">
-        <x:f>IF(C36="","Choose content",IF(D36="timeline",IFNA(VLOOKUP(C36,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C36,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J36" s="15" t="str">
+        <x:f>IF(B36="","",IFNA(VLOOKUP(B36,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K36" s="15" t="n">
+        <x:f>IF(B36="","",IFNA(VLOOKUP(B36,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="34" customHeight="1">
@@ -1663,12 +1974,20 @@
         <x:v>attic</x:v>
       </x:c>
       <x:c r="H37" s="15" t="str">
+        <x:f>IF(G37="","",IFNA(VLOOKUP(G37,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Attic</x:v>
+      </x:c>
+      <x:c r="I37" s="15" t="str">
         <x:f>IF(B37="","",IFNA(VLOOKUP(B37,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Left open trunk</x:v>
       </x:c>
-      <x:c r="I37" s="15" t="str">
-        <x:f>IF(C37="","Choose content",IF(D37="timeline",IFNA(VLOOKUP(C37,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C37,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J37" s="15" t="str">
+        <x:f>IF(B37="","",IFNA(VLOOKUP(B37,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K37" s="15" t="n">
+        <x:f>IF(B37="","",IFNA(VLOOKUP(B37,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="34" customHeight="1">
@@ -1693,12 +2012,20 @@
         <x:v>attic</x:v>
       </x:c>
       <x:c r="H38" s="15" t="str">
+        <x:f>IF(G38="","",IFNA(VLOOKUP(G38,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Attic</x:v>
+      </x:c>
+      <x:c r="I38" s="15" t="str">
         <x:f>IF(B38="","",IFNA(VLOOKUP(B38,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Right open trunk</x:v>
       </x:c>
-      <x:c r="I38" s="15" t="str">
-        <x:f>IF(C38="","Choose content",IF(D38="timeline",IFNA(VLOOKUP(C38,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C38,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J38" s="15" t="str">
+        <x:f>IF(B38="","",IFNA(VLOOKUP(B38,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K38" s="15" t="n">
+        <x:f>IF(B38="","",IFNA(VLOOKUP(B38,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="34" customHeight="1">
@@ -1723,12 +2050,20 @@
         <x:v>attic</x:v>
       </x:c>
       <x:c r="H39" s="15" t="str">
+        <x:f>IF(G39="","",IFNA(VLOOKUP(G39,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Attic</x:v>
+      </x:c>
+      <x:c r="I39" s="15" t="str">
         <x:f>IF(B39="","",IFNA(VLOOKUP(B39,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Shelving</x:v>
       </x:c>
-      <x:c r="I39" s="15" t="str">
-        <x:f>IF(C39="","Choose content",IF(D39="timeline",IFNA(VLOOKUP(C39,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C39,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J39" s="15" t="str">
+        <x:f>IF(B39="","",IFNA(VLOOKUP(B39,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K39" s="15" t="n">
+        <x:f>IF(B39="","",IFNA(VLOOKUP(B39,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="34" customHeight="1">
@@ -1753,12 +2088,20 @@
         <x:v>attic</x:v>
       </x:c>
       <x:c r="H40" s="15" t="str">
+        <x:f>IF(G40="","",IFNA(VLOOKUP(G40,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Attic</x:v>
+      </x:c>
+      <x:c r="I40" s="15" t="str">
         <x:f>IF(B40="","",IFNA(VLOOKUP(B40,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Research table</x:v>
       </x:c>
-      <x:c r="I40" s="15" t="str">
-        <x:f>IF(C40="","Choose content",IF(D40="timeline",IFNA(VLOOKUP(C40,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C40,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J40" s="15" t="str">
+        <x:f>IF(B40="","",IFNA(VLOOKUP(B40,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K40" s="15" t="n">
+        <x:f>IF(B40="","",IFNA(VLOOKUP(B40,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="34" customHeight="1">
@@ -1783,12 +2126,20 @@
         <x:v>natural_history</x:v>
       </x:c>
       <x:c r="H41" s="15" t="str">
+        <x:f>IF(G41="","",IFNA(VLOOKUP(G41,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Natural History Museum</x:v>
+      </x:c>
+      <x:c r="I41" s="15" t="str">
         <x:f>IF(B41="","",IFNA(VLOOKUP(B41,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Central recessed panel</x:v>
       </x:c>
-      <x:c r="I41" s="15" t="str">
-        <x:f>IF(C41="","Choose content",IF(D41="timeline",IFNA(VLOOKUP(C41,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C41,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J41" s="15" t="str">
+        <x:f>IF(B41="","",IFNA(VLOOKUP(B41,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K41" s="15" t="n">
+        <x:f>IF(B41="","",IFNA(VLOOKUP(B41,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="34" customHeight="1">
@@ -1813,12 +2164,20 @@
         <x:v>conservators_office</x:v>
       </x:c>
       <x:c r="H42" s="15" t="str">
+        <x:f>IF(G42="","",IFNA(VLOOKUP(G42,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Conservator's Office</x:v>
+      </x:c>
+      <x:c r="I42" s="15" t="str">
         <x:f>IF(B42="","",IFNA(VLOOKUP(B42,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Left shelving</x:v>
       </x:c>
-      <x:c r="I42" s="15" t="str">
-        <x:f>IF(C42="","Choose content",IF(D42="timeline",IFNA(VLOOKUP(C42,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C42,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J42" s="15" t="str">
+        <x:f>IF(B42="","",IFNA(VLOOKUP(B42,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K42" s="15" t="n">
+        <x:f>IF(B42="","",IFNA(VLOOKUP(B42,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="34" customHeight="1">
@@ -1843,12 +2202,20 @@
         <x:v>conservators_office</x:v>
       </x:c>
       <x:c r="H43" s="15" t="str">
+        <x:f>IF(G43="","",IFNA(VLOOKUP(G43,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Conservator's Office</x:v>
+      </x:c>
+      <x:c r="I43" s="15" t="str">
         <x:f>IF(B43="","",IFNA(VLOOKUP(B43,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Rear shelving</x:v>
       </x:c>
-      <x:c r="I43" s="15" t="str">
-        <x:f>IF(C43="","Choose content",IF(D43="timeline",IFNA(VLOOKUP(C43,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C43,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J43" s="15" t="str">
+        <x:f>IF(B43="","",IFNA(VLOOKUP(B43,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K43" s="15" t="n">
+        <x:f>IF(B43="","",IFNA(VLOOKUP(B43,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="34" customHeight="1">
@@ -1873,12 +2240,20 @@
         <x:v>conservators_office</x:v>
       </x:c>
       <x:c r="H44" s="15" t="str">
+        <x:f>IF(G44="","",IFNA(VLOOKUP(G44,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Conservator's Office</x:v>
+      </x:c>
+      <x:c r="I44" s="15" t="str">
         <x:f>IF(B44="","",IFNA(VLOOKUP(B44,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Right shelving</x:v>
       </x:c>
-      <x:c r="I44" s="15" t="str">
-        <x:f>IF(C44="","Choose content",IF(D44="timeline",IFNA(VLOOKUP(C44,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C44,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J44" s="15" t="str">
+        <x:f>IF(B44="","",IFNA(VLOOKUP(B44,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K44" s="15" t="n">
+        <x:f>IF(B44="","",IFNA(VLOOKUP(B44,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="34" customHeight="1">
@@ -1903,12 +2278,20 @@
         <x:v>lab</x:v>
       </x:c>
       <x:c r="H45" s="15" t="str">
+        <x:f>IF(G45="","",IFNA(VLOOKUP(G45,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Lab</x:v>
+      </x:c>
+      <x:c r="I45" s="15" t="str">
         <x:f>IF(B45="","",IFNA(VLOOKUP(B45,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Analysis bench</x:v>
       </x:c>
-      <x:c r="I45" s="15" t="str">
-        <x:f>IF(C45="","Choose content",IF(D45="timeline",IFNA(VLOOKUP(C45,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C45,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J45" s="15" t="str">
+        <x:f>IF(B45="","",IFNA(VLOOKUP(B45,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K45" s="15" t="n">
+        <x:f>IF(B45="","",IFNA(VLOOKUP(B45,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="34" customHeight="1">
@@ -1933,12 +2316,20 @@
         <x:v>lab</x:v>
       </x:c>
       <x:c r="H46" s="15" t="str">
+        <x:f>IF(G46="","",IFNA(VLOOKUP(G46,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Lab</x:v>
+      </x:c>
+      <x:c r="I46" s="15" t="str">
         <x:f>IF(B46="","",IFNA(VLOOKUP(B46,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Equipment</x:v>
       </x:c>
-      <x:c r="I46" s="15" t="str">
-        <x:f>IF(C46="","Choose content",IF(D46="timeline",IFNA(VLOOKUP(C46,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C46,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J46" s="15" t="str">
+        <x:f>IF(B46="","",IFNA(VLOOKUP(B46,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K46" s="15" t="n">
+        <x:f>IF(B46="","",IFNA(VLOOKUP(B46,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="34" customHeight="1">
@@ -1963,12 +2354,20 @@
         <x:v>lab</x:v>
       </x:c>
       <x:c r="H47" s="15" t="str">
+        <x:f>IF(G47="","",IFNA(VLOOKUP(G47,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Lab</x:v>
+      </x:c>
+      <x:c r="I47" s="15" t="str">
         <x:f>IF(B47="","",IFNA(VLOOKUP(B47,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Left cabinet</x:v>
       </x:c>
-      <x:c r="I47" s="15" t="str">
-        <x:f>IF(C47="","Choose content",IF(D47="timeline",IFNA(VLOOKUP(C47,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C47,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J47" s="15" t="str">
+        <x:f>IF(B47="","",IFNA(VLOOKUP(B47,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K47" s="15" t="n">
+        <x:f>IF(B47="","",IFNA(VLOOKUP(B47,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="34" customHeight="1">
@@ -1993,12 +2392,20 @@
         <x:v>lab</x:v>
       </x:c>
       <x:c r="H48" s="15" t="str">
+        <x:f>IF(G48="","",IFNA(VLOOKUP(G48,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Lab</x:v>
+      </x:c>
+      <x:c r="I48" s="15" t="str">
         <x:f>IF(B48="","",IFNA(VLOOKUP(B48,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
         <x:v>Right cabinet</x:v>
       </x:c>
-      <x:c r="I48" s="15" t="str">
-        <x:f>IF(C48="","Choose content",IF(D48="timeline",IFNA(VLOOKUP(C48,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C48,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J48" s="15" t="str">
+        <x:f>IF(B48="","",IFNA(VLOOKUP(B48,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K48" s="15" t="n">
+        <x:f>IF(B48="","",IFNA(VLOOKUP(B48,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="32" customHeight="1">
@@ -2012,11 +2419,16 @@
         <x:f>IF(B49="","",IFNA(VLOOKUP(B49,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
       </x:c>
       <x:c r="H49" s="15" t="str">
+        <x:f>IF(G49="","",IFNA(VLOOKUP(G49,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I49" s="15" t="str">
         <x:f>IF(B49="","",IFNA(VLOOKUP(B49,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
       </x:c>
-      <x:c r="I49" s="15" t="str">
-        <x:f>IF(C49="","Choose content",IF(D49="timeline",IFNA(VLOOKUP(C49,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C49,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J49" s="15" t="str">
+        <x:f>IF(B49="","",IFNA(VLOOKUP(B49,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K49" s="15" t="str">
+        <x:f>IF(B49="","",IFNA(VLOOKUP(B49,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
       </x:c>
     </x:row>
     <x:row r="50" ht="32" customHeight="1">
@@ -2030,11 +2442,16 @@
         <x:f>IF(B50="","",IFNA(VLOOKUP(B50,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
       </x:c>
       <x:c r="H50" s="15" t="str">
+        <x:f>IF(G50="","",IFNA(VLOOKUP(G50,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I50" s="15" t="str">
         <x:f>IF(B50="","",IFNA(VLOOKUP(B50,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
       </x:c>
-      <x:c r="I50" s="15" t="str">
-        <x:f>IF(C50="","Choose content",IF(D50="timeline",IFNA(VLOOKUP(C50,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C50,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J50" s="15" t="str">
+        <x:f>IF(B50="","",IFNA(VLOOKUP(B50,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K50" s="15" t="str">
+        <x:f>IF(B50="","",IFNA(VLOOKUP(B50,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
       </x:c>
     </x:row>
     <x:row r="51" ht="32" customHeight="1">
@@ -2048,11 +2465,16 @@
         <x:f>IF(B51="","",IFNA(VLOOKUP(B51,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
       </x:c>
       <x:c r="H51" s="15" t="str">
+        <x:f>IF(G51="","",IFNA(VLOOKUP(G51,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I51" s="15" t="str">
         <x:f>IF(B51="","",IFNA(VLOOKUP(B51,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
       </x:c>
-      <x:c r="I51" s="15" t="str">
-        <x:f>IF(C51="","Choose content",IF(D51="timeline",IFNA(VLOOKUP(C51,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C51,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J51" s="15" t="str">
+        <x:f>IF(B51="","",IFNA(VLOOKUP(B51,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K51" s="15" t="str">
+        <x:f>IF(B51="","",IFNA(VLOOKUP(B51,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
       </x:c>
     </x:row>
     <x:row r="52" ht="32" customHeight="1">
@@ -2066,11 +2488,16 @@
         <x:f>IF(B52="","",IFNA(VLOOKUP(B52,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
       </x:c>
       <x:c r="H52" s="15" t="str">
+        <x:f>IF(G52="","",IFNA(VLOOKUP(G52,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I52" s="15" t="str">
         <x:f>IF(B52="","",IFNA(VLOOKUP(B52,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
       </x:c>
-      <x:c r="I52" s="15" t="str">
-        <x:f>IF(C52="","Choose content",IF(D52="timeline",IFNA(VLOOKUP(C52,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C52,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J52" s="15" t="str">
+        <x:f>IF(B52="","",IFNA(VLOOKUP(B52,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K52" s="15" t="str">
+        <x:f>IF(B52="","",IFNA(VLOOKUP(B52,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
       </x:c>
     </x:row>
     <x:row r="53" ht="32" customHeight="1">
@@ -2084,11 +2511,16 @@
         <x:f>IF(B53="","",IFNA(VLOOKUP(B53,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
       </x:c>
       <x:c r="H53" s="15" t="str">
+        <x:f>IF(G53="","",IFNA(VLOOKUP(G53,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I53" s="15" t="str">
         <x:f>IF(B53="","",IFNA(VLOOKUP(B53,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
       </x:c>
-      <x:c r="I53" s="15" t="str">
-        <x:f>IF(C53="","Choose content",IF(D53="timeline",IFNA(VLOOKUP(C53,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C53,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J53" s="15" t="str">
+        <x:f>IF(B53="","",IFNA(VLOOKUP(B53,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K53" s="15" t="str">
+        <x:f>IF(B53="","",IFNA(VLOOKUP(B53,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
       </x:c>
     </x:row>
     <x:row r="54" ht="32" customHeight="1">
@@ -2102,11 +2534,16 @@
         <x:f>IF(B54="","",IFNA(VLOOKUP(B54,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
       </x:c>
       <x:c r="H54" s="15" t="str">
+        <x:f>IF(G54="","",IFNA(VLOOKUP(G54,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I54" s="15" t="str">
         <x:f>IF(B54="","",IFNA(VLOOKUP(B54,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
       </x:c>
-      <x:c r="I54" s="15" t="str">
-        <x:f>IF(C54="","Choose content",IF(D54="timeline",IFNA(VLOOKUP(C54,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C54,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J54" s="15" t="str">
+        <x:f>IF(B54="","",IFNA(VLOOKUP(B54,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K54" s="15" t="str">
+        <x:f>IF(B54="","",IFNA(VLOOKUP(B54,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
       </x:c>
     </x:row>
     <x:row r="55" ht="32" customHeight="1">
@@ -2120,11 +2557,16 @@
         <x:f>IF(B55="","",IFNA(VLOOKUP(B55,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
       </x:c>
       <x:c r="H55" s="15" t="str">
+        <x:f>IF(G55="","",IFNA(VLOOKUP(G55,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I55" s="15" t="str">
         <x:f>IF(B55="","",IFNA(VLOOKUP(B55,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
       </x:c>
-      <x:c r="I55" s="15" t="str">
-        <x:f>IF(C55="","Choose content",IF(D55="timeline",IFNA(VLOOKUP(C55,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C55,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J55" s="15" t="str">
+        <x:f>IF(B55="","",IFNA(VLOOKUP(B55,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K55" s="15" t="str">
+        <x:f>IF(B55="","",IFNA(VLOOKUP(B55,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
       </x:c>
     </x:row>
     <x:row r="56" ht="32" customHeight="1">
@@ -2138,11 +2580,16 @@
         <x:f>IF(B56="","",IFNA(VLOOKUP(B56,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
       </x:c>
       <x:c r="H56" s="15" t="str">
+        <x:f>IF(G56="","",IFNA(VLOOKUP(G56,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I56" s="15" t="str">
         <x:f>IF(B56="","",IFNA(VLOOKUP(B56,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
       </x:c>
-      <x:c r="I56" s="15" t="str">
-        <x:f>IF(C56="","Choose content",IF(D56="timeline",IFNA(VLOOKUP(C56,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C56,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J56" s="15" t="str">
+        <x:f>IF(B56="","",IFNA(VLOOKUP(B56,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K56" s="15" t="str">
+        <x:f>IF(B56="","",IFNA(VLOOKUP(B56,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
       </x:c>
     </x:row>
     <x:row r="57" ht="32" customHeight="1">
@@ -2156,11 +2603,16 @@
         <x:f>IF(B57="","",IFNA(VLOOKUP(B57,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
       </x:c>
       <x:c r="H57" s="15" t="str">
+        <x:f>IF(G57="","",IFNA(VLOOKUP(G57,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I57" s="15" t="str">
         <x:f>IF(B57="","",IFNA(VLOOKUP(B57,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
       </x:c>
-      <x:c r="I57" s="15" t="str">
-        <x:f>IF(C57="","Choose content",IF(D57="timeline",IFNA(VLOOKUP(C57,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C57,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J57" s="15" t="str">
+        <x:f>IF(B57="","",IFNA(VLOOKUP(B57,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K57" s="15" t="str">
+        <x:f>IF(B57="","",IFNA(VLOOKUP(B57,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
       </x:c>
     </x:row>
     <x:row r="58" ht="32" customHeight="1">
@@ -2174,11 +2626,16 @@
         <x:f>IF(B58="","",IFNA(VLOOKUP(B58,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
       </x:c>
       <x:c r="H58" s="15" t="str">
+        <x:f>IF(G58="","",IFNA(VLOOKUP(G58,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I58" s="15" t="str">
         <x:f>IF(B58="","",IFNA(VLOOKUP(B58,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
       </x:c>
-      <x:c r="I58" s="15" t="str">
-        <x:f>IF(C58="","Choose content",IF(D58="timeline",IFNA(VLOOKUP(C58,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C58,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J58" s="15" t="str">
+        <x:f>IF(B58="","",IFNA(VLOOKUP(B58,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K58" s="15" t="str">
+        <x:f>IF(B58="","",IFNA(VLOOKUP(B58,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
       </x:c>
     </x:row>
     <x:row r="59" ht="32" customHeight="1">
@@ -2192,11 +2649,16 @@
         <x:f>IF(B59="","",IFNA(VLOOKUP(B59,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
       </x:c>
       <x:c r="H59" s="15" t="str">
+        <x:f>IF(G59="","",IFNA(VLOOKUP(G59,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I59" s="15" t="str">
         <x:f>IF(B59="","",IFNA(VLOOKUP(B59,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
       </x:c>
-      <x:c r="I59" s="15" t="str">
-        <x:f>IF(C59="","Choose content",IF(D59="timeline",IFNA(VLOOKUP(C59,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C59,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J59" s="15" t="str">
+        <x:f>IF(B59="","",IFNA(VLOOKUP(B59,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K59" s="15" t="str">
+        <x:f>IF(B59="","",IFNA(VLOOKUP(B59,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
       </x:c>
     </x:row>
     <x:row r="60" ht="32" customHeight="1">
@@ -2210,11 +2672,16 @@
         <x:f>IF(B60="","",IFNA(VLOOKUP(B60,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
       </x:c>
       <x:c r="H60" s="15" t="str">
+        <x:f>IF(G60="","",IFNA(VLOOKUP(G60,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I60" s="15" t="str">
         <x:f>IF(B60="","",IFNA(VLOOKUP(B60,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
       </x:c>
-      <x:c r="I60" s="15" t="str">
-        <x:f>IF(C60="","Choose content",IF(D60="timeline",IFNA(VLOOKUP(C60,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C60,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J60" s="15" t="str">
+        <x:f>IF(B60="","",IFNA(VLOOKUP(B60,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K60" s="15" t="str">
+        <x:f>IF(B60="","",IFNA(VLOOKUP(B60,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
       </x:c>
     </x:row>
     <x:row r="61" ht="32" customHeight="1">
@@ -2228,11 +2695,16 @@
         <x:f>IF(B61="","",IFNA(VLOOKUP(B61,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
       </x:c>
       <x:c r="H61" s="15" t="str">
+        <x:f>IF(G61="","",IFNA(VLOOKUP(G61,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I61" s="15" t="str">
         <x:f>IF(B61="","",IFNA(VLOOKUP(B61,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
       </x:c>
-      <x:c r="I61" s="15" t="str">
-        <x:f>IF(C61="","Choose content",IF(D61="timeline",IFNA(VLOOKUP(C61,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C61,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J61" s="15" t="str">
+        <x:f>IF(B61="","",IFNA(VLOOKUP(B61,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K61" s="15" t="str">
+        <x:f>IF(B61="","",IFNA(VLOOKUP(B61,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
       </x:c>
     </x:row>
     <x:row r="62" ht="32" customHeight="1">
@@ -2246,11 +2718,16 @@
         <x:f>IF(B62="","",IFNA(VLOOKUP(B62,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
       </x:c>
       <x:c r="H62" s="15" t="str">
+        <x:f>IF(G62="","",IFNA(VLOOKUP(G62,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I62" s="15" t="str">
         <x:f>IF(B62="","",IFNA(VLOOKUP(B62,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
       </x:c>
-      <x:c r="I62" s="15" t="str">
-        <x:f>IF(C62="","Choose content",IF(D62="timeline",IFNA(VLOOKUP(C62,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C62,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J62" s="15" t="str">
+        <x:f>IF(B62="","",IFNA(VLOOKUP(B62,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K62" s="15" t="str">
+        <x:f>IF(B62="","",IFNA(VLOOKUP(B62,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
       </x:c>
     </x:row>
     <x:row r="63" ht="32" customHeight="1">
@@ -2264,17 +2741,37 @@
         <x:f>IF(B63="","",IFNA(VLOOKUP(B63,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
       </x:c>
       <x:c r="H63" s="15" t="str">
+        <x:f>IF(G63="","",IFNA(VLOOKUP(G63,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I63" s="15" t="str">
         <x:f>IF(B63="","",IFNA(VLOOKUP(B63,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
       </x:c>
-      <x:c r="I63" s="15" t="str">
-        <x:f>IF(C63="","Choose content",IF(D63="timeline",IFNA(VLOOKUP(C63,Timelines!$A$2:$D$501,3,FALSE),"Unknown timeline"),IFNA(VLOOKUP(C63,Content!$A$2:$B$501,2,FALSE),"Unknown content")))</x:f>
-        <x:v>Choose content</x:v>
+      <x:c r="J63" s="15" t="str">
+        <x:f>IF(B63="","",IFNA(VLOOKUP(B63,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K63" s="15" t="str">
+        <x:f>IF(B63="","",IFNA(VLOOKUP(B63,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="C2:C63">
     <x:cfRule type="expression" dxfId="0" priority="1">
       <x:formula>AND($A2&lt;&gt;"",$C2="")</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="B2:B63">
+    <x:cfRule type="expression" dxfId="1" priority="2">
+      <x:formula>AND($A2&lt;&gt;"",$B2&lt;&gt;"",COUNTIF(Slots!$A$2:$A$501,$B2)=0)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="F2:F63">
+    <x:cfRule type="expression" dxfId="2" priority="3">
+      <x:formula>AND($A2&lt;&gt;"",$F2="true",COUNTIFS($B$2:$B$501,$B2,$E$2:$E$501,$E2,$F$2:$F$501,"true")&gt;1)</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="E2:E63">
+    <x:cfRule type="expression" dxfId="3" priority="4">
+      <x:formula>AND($A2&lt;&gt;"",$F2="true",$E2&lt;&gt;"",COUNTIFS($B$2:$B$501,$B2,$E$2:$E$501,$E2,$F$2:$F$501,"true")&gt;1)</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:dataValidations count="4">
@@ -2293,7 +2790,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdde5a1abd8384241"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78624cb1c2764277"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2933,7 +3430,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa52e63debfe484c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9379bceb19c4c21"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3587,7 +4084,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79516145e6f2461b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf9bebe83d294814"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3827,7 +4324,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R289302938c334979"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6801667bfe04040"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4107,7 +4604,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe2791391a494097"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2290de5f75e0478b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5657,7 +6154,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R856341d2c27840c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd87d6064648a4f23"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6197,7 +6694,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6f8543bba544415"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d30ece90c094d11"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6223,185 +6720,225 @@
     </x:row>
     <x:row r="2" ht="58" customHeight="1">
       <x:c r="A2" s="24" t="str">
-        <x:v>1. Add material</x:v>
+        <x:v>1. Start here</x:v>
       </x:c>
       <x:c r="B2" s="24" t="str">
-        <x:v>Content: give each item a stable content_id. Fill title, description, image and citation. New ordinary items use detail and a blank adapter.</x:v>
+        <x:v>Use this Guide, then work in Content, Placements, Timelines, and Events. Pale amber cells are editable; gray cells are references or calculated context. Do not rename sheets or header rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="58" customHeight="1">
       <x:c r="A3" s="24" t="str">
-        <x:v>2. Choose a location</x:v>
+        <x:v>2. Add material</x:v>
       </x:c>
       <x:c r="B3" s="24" t="str">
-        <x:v>Placements: select slot_id, then content_id. Room and location names appear automatically. Slots lists every prepared access point.</x:v>
+        <x:v>Content: create a new stable content_id only for a new record. Title, description, and content_type are required. Image and citation are optional but recommended for research.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="58" customHeight="1">
       <x:c r="A4" s="24" t="str">
-        <x:v>3. Set presentation</x:v>
+        <x:v>3. Choose a location</x:v>
       </x:c>
       <x:c r="B4" s="24" t="str">
-        <x:v>content_type must match the item. Use sort_order to order items in a collection. Set published to true when ready.</x:v>
+        <x:v>Placements: choose a slot_id from the dropdown. The workbook fills Room ID, Room name, Location, Supported type, and Capacity automatically. Do not type a room separately: the slot defines the room.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="58" customHeight="1">
       <x:c r="A5" s="24" t="str">
-        <x:v>Empty locations</x:v>
+        <x:v>4. Assign content</x:v>
       </x:c>
       <x:c r="B5" s="24" t="str">
-        <x:v>Pre-filled draft rows have no content and published=false. They do not create website records until you assign content.</x:v>
+        <x:v>Choose content_id from the dropdown after selecting content_type. A timeline placement uses Timelines; other placements use Content. Keep placement_id unique.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="58" customHeight="1">
       <x:c r="A6" s="24" t="str">
-        <x:v>Same item in two rooms</x:v>
+        <x:v>5. Set presentation</x:v>
       </x:c>
       <x:c r="B6" s="24" t="str">
-        <x:v>Add a second placement with a new placement_id and the same content_id. Do not duplicate the material record.</x:v>
+        <x:v>content_type must match the item and slot. Use sort_order 1, 2, 3... for multiple records in one collection location. Do not reuse the same active sort order or content in one slot.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="58" customHeight="1">
       <x:c r="A7" s="24" t="str">
-        <x:v>Timeline editing</x:v>
+        <x:v>6. Publish clearly</x:v>
       </x:c>
       <x:c r="B7" s="24" t="str">
-        <x:v>Timelines contains introductions and success text. Events contains dated items. Equal sortKey values accept either order. displayedDate remains text.</x:v>
+        <x:v>published=true makes the placement visible on the site; published=false keeps it hidden. An empty unpublished draft row is a workbook prompt, not a site record.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="58" customHeight="1">
       <x:c r="A8" s="24" t="str">
-        <x:v>Existing collection</x:v>
+        <x:v>Empty locations</x:v>
       </x:c>
       <x:c r="B8" s="24" t="str">
-        <x:v>Collection is the original museum metadata. ChineseUVIvoryCollection draws its description from this sheet. Preserve its exact objectid.</x:v>
+        <x:v>Pre-filled draft rows have no content and published=false. They do not create website records until you assign content.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="58" customHeight="1">
       <x:c r="A9" s="24" t="str">
-        <x:v>Existing adapters</x:v>
+        <x:v>Same item in two rooms</x:v>
       </x:c>
       <x:c r="B9" s="24" t="str">
-        <x:v>Gray adapter fields preserve existing dialogs and tools. Their built-in text is still in room pages. Content text changes affect ordinary blank-adapter items; legacy dialog copy needs a separate migration.</x:v>
+        <x:v>Add a second placement with a new placement_id and the same content_id. Do not duplicate the material record.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="58" customHeight="1">
       <x:c r="A10" s="24" t="str">
-        <x:v>Prepared locations</x:v>
+        <x:v>Timeline editing</x:v>
       </x:c>
       <x:c r="B10" s="24" t="str">
-        <x:v>Rooms and Slots describe existing artwork. Keep IDs, anchors, routes and assets stable. New physical locations require matching geometry.</x:v>
+        <x:v>Timelines contains the activity introduction and success text. Events contains at least two events per timeline. sortKey is numeric ordering; displayedDate is visitor-facing text. Equal sortKey values intentionally accept either order.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="58" customHeight="1">
       <x:c r="A11" s="24" t="str">
-        <x:v>Images</x:v>
+        <x:v>Existing collection</x:v>
       </x:c>
       <x:c r="B11" s="24" t="str">
-        <x:v>Enter a website path such as /assets/img/example.jpg or an HTTPS image URL. Typing a local file path does not upload an image.</x:v>
+        <x:v>Collection is the original museum metadata. ChineseUVIvoryCollection draws its description from this sheet. Preserve its exact objectid.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="58" customHeight="1">
       <x:c r="A12" s="24" t="str">
-        <x:v>Colors</x:v>
+        <x:v>Existing adapters</x:v>
       </x:c>
       <x:c r="B12" s="24" t="str">
-        <x:v>Pale amber: editorial inputs. Gray: reference or calculated values. Dark amber: an empty content assignment.</x:v>
+        <x:v>Gray adapter fields preserve existing dialogs and tools. Their built-in text is still in room pages. Content text changes affect ordinary blank-adapter items; legacy dialog copy needs a separate migration.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="58" customHeight="1">
       <x:c r="A13" s="24" t="str">
-        <x:v>Preserve structure</x:v>
+        <x:v>Prepared locations</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
-        <x:v>Keep sheet names and the original header row. Add records in the tables. Never reuse an existing ID for a different record.</x:v>
+        <x:v>Slots lists all 45 validated access points with a human-readable editor_label, room, capacity, type, physical notes, and anchor reference. Keep IDs, anchors, routes, and assets stable. New physical locations require matching geometry and are outside this workbook workflow.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="58" customHeight="1">
       <x:c r="A14" s="24" t="str">
-        <x:v>Draft material</x:v>
+        <x:v>Images</x:v>
       </x:c>
       <x:c r="B14" s="24" t="str">
-        <x:v>Existing teaching examples and placeholder notices are carried over unchanged. Your team supplies replacements.</x:v>
+        <x:v>Use a site path such as /assets/img/example.jpg or an HTTPS image URL. In the shared Teams workflow, enter a simple PNG/JPG filename and upload that file to the adjacent Images folder. A local computer path does not upload an image.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="58" customHeight="1">
       <x:c r="A15" s="24" t="str">
-        <x:v>Import process</x:v>
+        <x:v>Citations and links</x:v>
       </x:c>
       <x:c r="B15" s="24" t="str">
-        <x:v>Run the check command described in README.md. Apply writes the website CSVs with a backup. Rebuild and inspect locally before any publishing.</x:v>
+        <x:v>Use citation for a source or credit, not private notes. Use HTTPS or a repository/site path where appropriate. Check that the citation supports the wording before publishing.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="58" customHeight="1">
       <x:c r="A16" s="24" t="str">
-        <x:v>Sharing</x:v>
+        <x:v>Warnings</x:v>
       </x:c>
       <x:c r="B16" s="24" t="str">
-        <x:v>Share this .xlsx in Excel or a shared drive. Return the edited .xlsx for validation and import. The site does not read the workbook live.</x:v>
+        <x:v>Red cells indicate a likely invalid or conflicting entry. Run workbook.py check before sharing the workbook; it rejects unknown slots, duplicate IDs, incompatible types, missing required values, disabled targets, duplicate active ordering, and broken timeline references.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="58" customHeight="1">
       <x:c r="A17" s="24" t="str">
-        <x:v>Source snapshots</x:v>
+        <x:v>Colors</x:v>
       </x:c>
       <x:c r="B17" s="24" t="str">
-        <x:v>The hashes below prevent importing over source data changed after this workbook was created. Do not edit these cells.</x:v>
+        <x:v>Pale amber: editorial inputs. Gray: reference or calculated values. Dark amber: an empty content assignment.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="58" customHeight="1">
       <x:c r="A18" s="24" t="str">
-        <x:v>_data/placements.csv</x:v>
+        <x:v>Preserve structure</x:v>
       </x:c>
       <x:c r="B18" s="24" t="str">
-        <x:v>087a2f718b5ee1c6783cafeb30f16a5ad934822d66ecf6c0484d19156f86b918</x:v>
+        <x:v>Keep sheet names and the original header row. Add records in the tables. Never reuse an existing ID for a different record.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="58" customHeight="1">
       <x:c r="A19" s="24" t="str">
-        <x:v>_data/room_content.csv</x:v>
+        <x:v>Draft material</x:v>
       </x:c>
       <x:c r="B19" s="24" t="str">
-        <x:v>c859709397870b691cca329d6d1ec56fb9dc756d035b2636081111dc46ecebf6</x:v>
+        <x:v>Existing teaching examples and placeholder notices are carried over unchanged. Your team supplies replacements.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="58" customHeight="1">
       <x:c r="A20" s="24" t="str">
-        <x:v>_data/timeline_events.csv</x:v>
+        <x:v>Import process</x:v>
       </x:c>
       <x:c r="B20" s="24" t="str">
-        <x:v>6d440f2d8e35129dc48ee25acadc58e8491ea7bfea2e6b250ab9c792731c031e</x:v>
+        <x:v>Run the check command described in README.md. Apply writes the website CSVs with a backup. Rebuild and inspect locally before any publishing.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="58" customHeight="1">
       <x:c r="A21" s="24" t="str">
-        <x:v>_data/room_timelines.csv</x:v>
+        <x:v>Sharing</x:v>
       </x:c>
       <x:c r="B21" s="24" t="str">
-        <x:v>5b177dd4ed184a477cf576a2a6b5d86871b8f2332f353c70e0177ebaff2a68c0</x:v>
+        <x:v>Share this .xlsx in Excel or a shared drive. Return the edited .xlsx for validation and import. The site does not read the workbook live.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="58" customHeight="1">
       <x:c r="A22" s="24" t="str">
-        <x:v>_data/rooms.csv</x:v>
+        <x:v>Source snapshots</x:v>
       </x:c>
       <x:c r="B22" s="24" t="str">
-        <x:v>9de7372fc7eff45ffcb4fb71f0686068f46e8401632faa59971ffb9e42c15fb5</x:v>
+        <x:v>The hashes below prevent importing over source data changed after this workbook was created. Do not edit these cells.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="58" customHeight="1">
       <x:c r="A23" s="24" t="str">
-        <x:v>_data/exhibit_slots.csv</x:v>
+        <x:v>_data/placements.csv</x:v>
       </x:c>
       <x:c r="B23" s="24" t="str">
-        <x:v>d3e4333d6d7ec2dd97f99009148754df2099538d822c07f0c6d7f0bb2e0270ac</x:v>
+        <x:v>087a2f718b5ee1c6783cafeb30f16a5ad934822d66ecf6c0484d19156f86b918</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="58" customHeight="1">
       <x:c r="A24" s="24" t="str">
+        <x:v>_data/room_content.csv</x:v>
+      </x:c>
+      <x:c r="B24" s="24" t="str">
+        <x:v>c859709397870b691cca329d6d1ec56fb9dc756d035b2636081111dc46ecebf6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="58" customHeight="1">
+      <x:c r="A25" s="24" t="str">
+        <x:v>_data/timeline_events.csv</x:v>
+      </x:c>
+      <x:c r="B25" s="24" t="str">
+        <x:v>6d440f2d8e35129dc48ee25acadc58e8491ea7bfea2e6b250ab9c792731c031e</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="58" customHeight="1">
+      <x:c r="A26" s="24" t="str">
+        <x:v>_data/room_timelines.csv</x:v>
+      </x:c>
+      <x:c r="B26" s="24" t="str">
+        <x:v>5b177dd4ed184a477cf576a2a6b5d86871b8f2332f353c70e0177ebaff2a68c0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="58" customHeight="1">
+      <x:c r="A27" s="24" t="str">
+        <x:v>_data/rooms.csv</x:v>
+      </x:c>
+      <x:c r="B27" s="24" t="str">
+        <x:v>9de7372fc7eff45ffcb4fb71f0686068f46e8401632faa59971ffb9e42c15fb5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="58" customHeight="1">
+      <x:c r="A28" s="24" t="str">
+        <x:v>_data/exhibit_slots.csv</x:v>
+      </x:c>
+      <x:c r="B28" s="24" t="str">
+        <x:v>d3e4333d6d7ec2dd97f99009148754df2099538d822c07f0c6d7f0bb2e0270ac</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="58" customHeight="1">
+      <x:c r="A29" s="24" t="str">
         <x:v>_data/demo-metadata.csv</x:v>
       </x:c>
-      <x:c r="B24" s="24" t="str">
+      <x:c r="B29" s="24" t="str">
         <x:v>4b52545ce188c6aadc29a35bfe23c0c935ab202baaa080c7a0dee9fa4257b543</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Add curator-submitted Geib Flute media and placement
Imports the curator's Geib Flute image and editorial content via the shared OneDrive workbook pipeline: publishes a new placement in the gallery_wall_01 slot, adds the corresponding editorial content record, and copies the approved image into assets/img/editorial/. Also excludes local pre-import CSV backups (docs/room-restoration/editorial-backups/) from version control, since they are maintainer-local recovery artifacts.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/archivory-editorial/ArchIvory Editorial Workbook.xlsx
+++ b/outputs/archivory-editorial/ArchIvory Editorial Workbook.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Placements" sheetId="1" r:id="Re014c254b705446a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content" sheetId="2" r:id="R42f894b349ea4c2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="3" r:id="R1fc49a2437e74b94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timelines" sheetId="4" r:id="Re1f14be3f0994c5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rooms" sheetId="5" r:id="Rd27092c3917c4ebc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slots" sheetId="6" r:id="R5ebe49cfc1924a4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection" sheetId="7" r:id="R96365c5efe0f4dbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="Re9684f59b0454efc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Placements" sheetId="1" r:id="Rf9fb81c59d2d442d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content" sheetId="2" r:id="Rbe706e17fb9a417d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="3" r:id="R15f8978f1cfe421b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timelines" sheetId="4" r:id="Rabbebed5e7af4dd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rooms" sheetId="5" r:id="Re21abc23a4584d29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slots" sheetId="6" r:id="R0dd33f77310d47ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection" sheetId="7" r:id="Rde3aeb45d1ed4b63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="Rfbb2d1e9fb5940e2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -196,7 +196,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PlacementsTable" displayName="PlacementsTable" ref="A1:K63" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PlacementsTable" displayName="PlacementsTable" ref="A1:K44" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="placement_id"/>
     <x:tableColumn id="2" name="slot_id"/>
@@ -215,7 +215,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ContentTable" displayName="ContentTable" ref="A1:G41" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ContentTable" displayName="ContentTable" ref="A1:G42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="content_id"/>
     <x:tableColumn id="2" name="title"/>
@@ -705,7 +705,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F5" s="12" t="str">
-        <x:v>true</x:v>
+        <x:v>false</x:v>
       </x:c>
       <x:c r="G5" s="15" t="str">
         <x:f>IF(B5="","",IFERROR(VLOOKUP(B5,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
@@ -1650,12 +1650,14 @@
     </x:row>
     <x:row r="29" ht="34" customHeight="1">
       <x:c r="A29" s="12" t="str">
-        <x:v>draft_historical_society_intro</x:v>
+        <x:v>geib-flute</x:v>
       </x:c>
       <x:c r="B29" s="12" t="str">
-        <x:v>historical_society_intro</x:v>
-      </x:c>
-      <x:c r="C29" s="12" t="str"/>
+        <x:v>gallery_wall_01</x:v>
+      </x:c>
+      <x:c r="C29" s="12" t="str">
+        <x:v>geib-flute</x:v>
+      </x:c>
       <x:c r="D29" s="12" t="str">
         <x:v>detail</x:v>
       </x:c>
@@ -1663,1113 +1665,391 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F29" s="12" t="str">
-        <x:v>false</x:v>
+        <x:v>true</x:v>
       </x:c>
       <x:c r="G29" s="15" t="str">
         <x:f>IF(B29="","",IFERROR(VLOOKUP(B29,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>historical_society</x:v>
+        <x:v>gallery</x:v>
       </x:c>
       <x:c r="H29" s="15" t="str">
         <x:f>IF(G29="","",IFERROR(VLOOKUP(G29,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Historical Society</x:v>
+        <x:v>Gallery</x:v>
       </x:c>
       <x:c r="I29" s="15" t="str">
         <x:f>IF(B29="","",IFERROR(VLOOKUP(B29,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Historical Society introduction</x:v>
+        <x:v>Near left-wall relief</x:v>
       </x:c>
       <x:c r="J29" s="15" t="str">
         <x:f>IF(B29="","",IFERROR(VLOOKUP(B29,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>detail</x:v>
+        <x:v>collection</x:v>
       </x:c>
       <x:c r="K29" s="15" t="n">
         <x:f>IF(B29="","",IFERROR(VLOOKUP(B29,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="34" customHeight="1">
-      <x:c r="A30" s="12" t="str">
-        <x:v>draft_attic_intro</x:v>
-      </x:c>
-      <x:c r="B30" s="12" t="str">
-        <x:v>attic_intro</x:v>
-      </x:c>
-      <x:c r="C30" s="12" t="str"/>
-      <x:c r="D30" s="12" t="str">
-        <x:v>detail</x:v>
-      </x:c>
-      <x:c r="E30" s="13" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F30" s="12" t="str">
-        <x:v>false</x:v>
-      </x:c>
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="32" customHeight="1">
+      <x:c r="A30" s="12"/>
+      <x:c r="B30" s="12"/>
+      <x:c r="C30" s="12"/>
+      <x:c r="D30" s="12"/>
+      <x:c r="E30" s="13"/>
+      <x:c r="F30" s="12"/>
       <x:c r="G30" s="15" t="str">
         <x:f>IF(B30="","",IFERROR(VLOOKUP(B30,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>attic</x:v>
       </x:c>
       <x:c r="H30" s="15" t="str">
         <x:f>IF(G30="","",IFERROR(VLOOKUP(G30,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Attic</x:v>
       </x:c>
       <x:c r="I30" s="15" t="str">
         <x:f>IF(B30="","",IFERROR(VLOOKUP(B30,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Attic introduction</x:v>
       </x:c>
       <x:c r="J30" s="15" t="str">
         <x:f>IF(B30="","",IFERROR(VLOOKUP(B30,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>detail</x:v>
-      </x:c>
-      <x:c r="K30" s="15" t="n">
+      </x:c>
+      <x:c r="K30" s="15" t="str">
         <x:f>IF(B30="","",IFERROR(VLOOKUP(B30,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="34" customHeight="1">
-      <x:c r="A31" s="12" t="str">
-        <x:v>draft_natural_history_intro</x:v>
-      </x:c>
-      <x:c r="B31" s="12" t="str">
-        <x:v>natural_history_intro</x:v>
-      </x:c>
-      <x:c r="C31" s="12" t="str"/>
-      <x:c r="D31" s="12" t="str">
-        <x:v>detail</x:v>
-      </x:c>
-      <x:c r="E31" s="13" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F31" s="12" t="str">
-        <x:v>false</x:v>
-      </x:c>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="32" customHeight="1">
+      <x:c r="A31" s="12"/>
+      <x:c r="B31" s="12"/>
+      <x:c r="C31" s="12"/>
+      <x:c r="D31" s="12"/>
+      <x:c r="E31" s="13"/>
+      <x:c r="F31" s="12"/>
       <x:c r="G31" s="15" t="str">
         <x:f>IF(B31="","",IFERROR(VLOOKUP(B31,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>natural_history</x:v>
       </x:c>
       <x:c r="H31" s="15" t="str">
         <x:f>IF(G31="","",IFERROR(VLOOKUP(G31,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Natural History Museum</x:v>
       </x:c>
       <x:c r="I31" s="15" t="str">
         <x:f>IF(B31="","",IFERROR(VLOOKUP(B31,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Natural History Museum introduction</x:v>
       </x:c>
       <x:c r="J31" s="15" t="str">
         <x:f>IF(B31="","",IFERROR(VLOOKUP(B31,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>detail</x:v>
-      </x:c>
-      <x:c r="K31" s="15" t="n">
+      </x:c>
+      <x:c r="K31" s="15" t="str">
         <x:f>IF(B31="","",IFERROR(VLOOKUP(B31,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="34" customHeight="1">
-      <x:c r="A32" s="12" t="str">
-        <x:v>draft_conservators_office_intro</x:v>
-      </x:c>
-      <x:c r="B32" s="12" t="str">
-        <x:v>conservators_office_intro</x:v>
-      </x:c>
-      <x:c r="C32" s="12" t="str"/>
-      <x:c r="D32" s="12" t="str">
-        <x:v>detail</x:v>
-      </x:c>
-      <x:c r="E32" s="13" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F32" s="12" t="str">
-        <x:v>false</x:v>
-      </x:c>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="32" customHeight="1">
+      <x:c r="A32" s="12"/>
+      <x:c r="B32" s="12"/>
+      <x:c r="C32" s="12"/>
+      <x:c r="D32" s="12"/>
+      <x:c r="E32" s="13"/>
+      <x:c r="F32" s="12"/>
       <x:c r="G32" s="15" t="str">
         <x:f>IF(B32="","",IFERROR(VLOOKUP(B32,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>conservators_office</x:v>
       </x:c>
       <x:c r="H32" s="15" t="str">
         <x:f>IF(G32="","",IFERROR(VLOOKUP(G32,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Conservator's Office</x:v>
       </x:c>
       <x:c r="I32" s="15" t="str">
         <x:f>IF(B32="","",IFERROR(VLOOKUP(B32,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Conservator's Office introduction</x:v>
       </x:c>
       <x:c r="J32" s="15" t="str">
         <x:f>IF(B32="","",IFERROR(VLOOKUP(B32,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>detail</x:v>
-      </x:c>
-      <x:c r="K32" s="15" t="n">
+      </x:c>
+      <x:c r="K32" s="15" t="str">
         <x:f>IF(B32="","",IFERROR(VLOOKUP(B32,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="34" customHeight="1">
-      <x:c r="A33" s="12" t="str">
-        <x:v>draft_lab_intro</x:v>
-      </x:c>
-      <x:c r="B33" s="12" t="str">
-        <x:v>lab_intro</x:v>
-      </x:c>
-      <x:c r="C33" s="12" t="str"/>
-      <x:c r="D33" s="12" t="str">
-        <x:v>detail</x:v>
-      </x:c>
-      <x:c r="E33" s="13" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F33" s="12" t="str">
-        <x:v>false</x:v>
-      </x:c>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="32" customHeight="1">
+      <x:c r="A33" s="12"/>
+      <x:c r="B33" s="12"/>
+      <x:c r="C33" s="12"/>
+      <x:c r="D33" s="12"/>
+      <x:c r="E33" s="13"/>
+      <x:c r="F33" s="12"/>
       <x:c r="G33" s="15" t="str">
         <x:f>IF(B33="","",IFERROR(VLOOKUP(B33,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>lab</x:v>
       </x:c>
       <x:c r="H33" s="15" t="str">
         <x:f>IF(G33="","",IFERROR(VLOOKUP(G33,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Lab</x:v>
       </x:c>
       <x:c r="I33" s="15" t="str">
         <x:f>IF(B33="","",IFERROR(VLOOKUP(B33,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Lab introduction</x:v>
       </x:c>
       <x:c r="J33" s="15" t="str">
         <x:f>IF(B33="","",IFERROR(VLOOKUP(B33,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>detail</x:v>
-      </x:c>
-      <x:c r="K33" s="15" t="n">
+      </x:c>
+      <x:c r="K33" s="15" t="str">
         <x:f>IF(B33="","",IFERROR(VLOOKUP(B33,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="34" customHeight="1">
-      <x:c r="A34" s="12" t="str">
-        <x:v>draft_gallery_case_02</x:v>
-      </x:c>
-      <x:c r="B34" s="12" t="str">
-        <x:v>gallery_case_02</x:v>
-      </x:c>
-      <x:c r="C34" s="12" t="str"/>
-      <x:c r="D34" s="12" t="str">
-        <x:v>detail</x:v>
-      </x:c>
-      <x:c r="E34" s="13" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F34" s="12" t="str">
-        <x:v>false</x:v>
-      </x:c>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="32" customHeight="1">
+      <x:c r="A34" s="12"/>
+      <x:c r="B34" s="12"/>
+      <x:c r="C34" s="12"/>
+      <x:c r="D34" s="12"/>
+      <x:c r="E34" s="13"/>
+      <x:c r="F34" s="12"/>
       <x:c r="G34" s="15" t="str">
         <x:f>IF(B34="","",IFERROR(VLOOKUP(B34,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>gallery</x:v>
       </x:c>
       <x:c r="H34" s="15" t="str">
         <x:f>IF(G34="","",IFERROR(VLOOKUP(G34,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Gallery</x:v>
       </x:c>
       <x:c r="I34" s="15" t="str">
         <x:f>IF(B34="","",IFERROR(VLOOKUP(B34,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Rear round display</x:v>
       </x:c>
       <x:c r="J34" s="15" t="str">
         <x:f>IF(B34="","",IFERROR(VLOOKUP(B34,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>collection</x:v>
-      </x:c>
-      <x:c r="K34" s="15" t="n">
+      </x:c>
+      <x:c r="K34" s="15" t="str">
         <x:f>IF(B34="","",IFERROR(VLOOKUP(B34,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="34" customHeight="1">
-      <x:c r="A35" s="12" t="str">
-        <x:v>draft_historical_society_case_01</x:v>
-      </x:c>
-      <x:c r="B35" s="12" t="str">
-        <x:v>historical_society_case_01</x:v>
-      </x:c>
-      <x:c r="C35" s="12" t="str"/>
-      <x:c r="D35" s="12" t="str">
-        <x:v>detail</x:v>
-      </x:c>
-      <x:c r="E35" s="13" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F35" s="12" t="str">
-        <x:v>false</x:v>
-      </x:c>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="32" customHeight="1">
+      <x:c r="A35" s="12"/>
+      <x:c r="B35" s="12"/>
+      <x:c r="C35" s="12"/>
+      <x:c r="D35" s="12"/>
+      <x:c r="E35" s="13"/>
+      <x:c r="F35" s="12"/>
       <x:c r="G35" s="15" t="str">
         <x:f>IF(B35="","",IFERROR(VLOOKUP(B35,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>historical_society</x:v>
       </x:c>
       <x:c r="H35" s="15" t="str">
         <x:f>IF(G35="","",IFERROR(VLOOKUP(G35,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Historical Society</x:v>
       </x:c>
       <x:c r="I35" s="15" t="str">
         <x:f>IF(B35="","",IFERROR(VLOOKUP(B35,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Window-side case</x:v>
       </x:c>
       <x:c r="J35" s="15" t="str">
         <x:f>IF(B35="","",IFERROR(VLOOKUP(B35,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>collection</x:v>
-      </x:c>
-      <x:c r="K35" s="15" t="n">
+      </x:c>
+      <x:c r="K35" s="15" t="str">
         <x:f>IF(B35="","",IFERROR(VLOOKUP(B35,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="34" customHeight="1">
-      <x:c r="A36" s="12" t="str">
-        <x:v>draft_historical_society_case_02</x:v>
-      </x:c>
-      <x:c r="B36" s="12" t="str">
-        <x:v>historical_society_case_02</x:v>
-      </x:c>
-      <x:c r="C36" s="12" t="str"/>
-      <x:c r="D36" s="12" t="str">
-        <x:v>detail</x:v>
-      </x:c>
-      <x:c r="E36" s="13" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F36" s="12" t="str">
-        <x:v>false</x:v>
-      </x:c>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="32" customHeight="1">
+      <x:c r="A36" s="12"/>
+      <x:c r="B36" s="12"/>
+      <x:c r="C36" s="12"/>
+      <x:c r="D36" s="12"/>
+      <x:c r="E36" s="13"/>
+      <x:c r="F36" s="12"/>
       <x:c r="G36" s="15" t="str">
         <x:f>IF(B36="","",IFERROR(VLOOKUP(B36,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>historical_society</x:v>
       </x:c>
       <x:c r="H36" s="15" t="str">
         <x:f>IF(G36="","",IFERROR(VLOOKUP(G36,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Historical Society</x:v>
       </x:c>
       <x:c r="I36" s="15" t="str">
         <x:f>IF(B36="","",IFERROR(VLOOKUP(B36,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Foreground-right case</x:v>
       </x:c>
       <x:c r="J36" s="15" t="str">
         <x:f>IF(B36="","",IFERROR(VLOOKUP(B36,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>collection</x:v>
-      </x:c>
-      <x:c r="K36" s="15" t="n">
+      </x:c>
+      <x:c r="K36" s="15" t="str">
         <x:f>IF(B36="","",IFERROR(VLOOKUP(B36,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="34" customHeight="1">
-      <x:c r="A37" s="12" t="str">
-        <x:v>draft_attic_trunk_01</x:v>
-      </x:c>
-      <x:c r="B37" s="12" t="str">
-        <x:v>attic_trunk_01</x:v>
-      </x:c>
-      <x:c r="C37" s="12" t="str"/>
-      <x:c r="D37" s="12" t="str">
-        <x:v>detail</x:v>
-      </x:c>
-      <x:c r="E37" s="13" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F37" s="12" t="str">
-        <x:v>false</x:v>
-      </x:c>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="32" customHeight="1">
+      <x:c r="A37" s="12"/>
+      <x:c r="B37" s="12"/>
+      <x:c r="C37" s="12"/>
+      <x:c r="D37" s="12"/>
+      <x:c r="E37" s="13"/>
+      <x:c r="F37" s="12"/>
       <x:c r="G37" s="15" t="str">
         <x:f>IF(B37="","",IFERROR(VLOOKUP(B37,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>attic</x:v>
       </x:c>
       <x:c r="H37" s="15" t="str">
         <x:f>IF(G37="","",IFERROR(VLOOKUP(G37,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Attic</x:v>
       </x:c>
       <x:c r="I37" s="15" t="str">
         <x:f>IF(B37="","",IFERROR(VLOOKUP(B37,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Left open trunk</x:v>
       </x:c>
       <x:c r="J37" s="15" t="str">
         <x:f>IF(B37="","",IFERROR(VLOOKUP(B37,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>collection</x:v>
-      </x:c>
-      <x:c r="K37" s="15" t="n">
+      </x:c>
+      <x:c r="K37" s="15" t="str">
         <x:f>IF(B37="","",IFERROR(VLOOKUP(B37,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="34" customHeight="1">
-      <x:c r="A38" s="12" t="str">
-        <x:v>draft_attic_trunk_02</x:v>
-      </x:c>
-      <x:c r="B38" s="12" t="str">
-        <x:v>attic_trunk_02</x:v>
-      </x:c>
-      <x:c r="C38" s="12" t="str"/>
-      <x:c r="D38" s="12" t="str">
-        <x:v>detail</x:v>
-      </x:c>
-      <x:c r="E38" s="13" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F38" s="12" t="str">
-        <x:v>false</x:v>
-      </x:c>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="32" customHeight="1">
+      <x:c r="A38" s="12"/>
+      <x:c r="B38" s="12"/>
+      <x:c r="C38" s="12"/>
+      <x:c r="D38" s="12"/>
+      <x:c r="E38" s="13"/>
+      <x:c r="F38" s="12"/>
       <x:c r="G38" s="15" t="str">
         <x:f>IF(B38="","",IFERROR(VLOOKUP(B38,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>attic</x:v>
       </x:c>
       <x:c r="H38" s="15" t="str">
         <x:f>IF(G38="","",IFERROR(VLOOKUP(G38,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Attic</x:v>
       </x:c>
       <x:c r="I38" s="15" t="str">
         <x:f>IF(B38="","",IFERROR(VLOOKUP(B38,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Right open trunk</x:v>
       </x:c>
       <x:c r="J38" s="15" t="str">
         <x:f>IF(B38="","",IFERROR(VLOOKUP(B38,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>collection</x:v>
-      </x:c>
-      <x:c r="K38" s="15" t="n">
+      </x:c>
+      <x:c r="K38" s="15" t="str">
         <x:f>IF(B38="","",IFERROR(VLOOKUP(B38,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="34" customHeight="1">
-      <x:c r="A39" s="12" t="str">
-        <x:v>draft_attic_shelves_01</x:v>
-      </x:c>
-      <x:c r="B39" s="12" t="str">
-        <x:v>attic_shelves_01</x:v>
-      </x:c>
-      <x:c r="C39" s="12" t="str"/>
-      <x:c r="D39" s="12" t="str">
-        <x:v>detail</x:v>
-      </x:c>
-      <x:c r="E39" s="13" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F39" s="12" t="str">
-        <x:v>false</x:v>
-      </x:c>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="32" customHeight="1">
+      <x:c r="A39" s="12"/>
+      <x:c r="B39" s="12"/>
+      <x:c r="C39" s="12"/>
+      <x:c r="D39" s="12"/>
+      <x:c r="E39" s="13"/>
+      <x:c r="F39" s="12"/>
       <x:c r="G39" s="15" t="str">
         <x:f>IF(B39="","",IFERROR(VLOOKUP(B39,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>attic</x:v>
       </x:c>
       <x:c r="H39" s="15" t="str">
         <x:f>IF(G39="","",IFERROR(VLOOKUP(G39,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Attic</x:v>
       </x:c>
       <x:c r="I39" s="15" t="str">
         <x:f>IF(B39="","",IFERROR(VLOOKUP(B39,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Shelving</x:v>
       </x:c>
       <x:c r="J39" s="15" t="str">
         <x:f>IF(B39="","",IFERROR(VLOOKUP(B39,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>collection</x:v>
-      </x:c>
-      <x:c r="K39" s="15" t="n">
+      </x:c>
+      <x:c r="K39" s="15" t="str">
         <x:f>IF(B39="","",IFERROR(VLOOKUP(B39,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="34" customHeight="1">
-      <x:c r="A40" s="12" t="str">
-        <x:v>draft_attic_table_01</x:v>
-      </x:c>
-      <x:c r="B40" s="12" t="str">
-        <x:v>attic_table_01</x:v>
-      </x:c>
-      <x:c r="C40" s="12" t="str"/>
-      <x:c r="D40" s="12" t="str">
-        <x:v>detail</x:v>
-      </x:c>
-      <x:c r="E40" s="13" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F40" s="12" t="str">
-        <x:v>false</x:v>
-      </x:c>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="32" customHeight="1">
+      <x:c r="A40" s="12"/>
+      <x:c r="B40" s="12"/>
+      <x:c r="C40" s="12"/>
+      <x:c r="D40" s="12"/>
+      <x:c r="E40" s="13"/>
+      <x:c r="F40" s="12"/>
       <x:c r="G40" s="15" t="str">
         <x:f>IF(B40="","",IFERROR(VLOOKUP(B40,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>attic</x:v>
       </x:c>
       <x:c r="H40" s="15" t="str">
         <x:f>IF(G40="","",IFERROR(VLOOKUP(G40,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Attic</x:v>
       </x:c>
       <x:c r="I40" s="15" t="str">
         <x:f>IF(B40="","",IFERROR(VLOOKUP(B40,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Research table</x:v>
       </x:c>
       <x:c r="J40" s="15" t="str">
         <x:f>IF(B40="","",IFERROR(VLOOKUP(B40,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>collection</x:v>
-      </x:c>
-      <x:c r="K40" s="15" t="n">
+      </x:c>
+      <x:c r="K40" s="15" t="str">
         <x:f>IF(B40="","",IFERROR(VLOOKUP(B40,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41" ht="34" customHeight="1">
-      <x:c r="A41" s="12" t="str">
-        <x:v>draft_natural_history_panel_02</x:v>
-      </x:c>
-      <x:c r="B41" s="12" t="str">
-        <x:v>natural_history_panel_02</x:v>
-      </x:c>
-      <x:c r="C41" s="12" t="str"/>
-      <x:c r="D41" s="12" t="str">
-        <x:v>detail</x:v>
-      </x:c>
-      <x:c r="E41" s="13" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F41" s="12" t="str">
-        <x:v>false</x:v>
-      </x:c>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="32" customHeight="1">
+      <x:c r="A41" s="12"/>
+      <x:c r="B41" s="12"/>
+      <x:c r="C41" s="12"/>
+      <x:c r="D41" s="12"/>
+      <x:c r="E41" s="13"/>
+      <x:c r="F41" s="12"/>
       <x:c r="G41" s="15" t="str">
         <x:f>IF(B41="","",IFERROR(VLOOKUP(B41,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>natural_history</x:v>
       </x:c>
       <x:c r="H41" s="15" t="str">
         <x:f>IF(G41="","",IFERROR(VLOOKUP(G41,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Natural History Museum</x:v>
       </x:c>
       <x:c r="I41" s="15" t="str">
         <x:f>IF(B41="","",IFERROR(VLOOKUP(B41,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Central recessed panel</x:v>
       </x:c>
       <x:c r="J41" s="15" t="str">
         <x:f>IF(B41="","",IFERROR(VLOOKUP(B41,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>collection</x:v>
-      </x:c>
-      <x:c r="K41" s="15" t="n">
+      </x:c>
+      <x:c r="K41" s="15" t="str">
         <x:f>IF(B41="","",IFERROR(VLOOKUP(B41,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42" ht="34" customHeight="1">
-      <x:c r="A42" s="12" t="str">
-        <x:v>draft_conservators_office_shelves_01</x:v>
-      </x:c>
-      <x:c r="B42" s="12" t="str">
-        <x:v>conservators_office_shelves_01</x:v>
-      </x:c>
-      <x:c r="C42" s="12" t="str"/>
-      <x:c r="D42" s="12" t="str">
-        <x:v>detail</x:v>
-      </x:c>
-      <x:c r="E42" s="13" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F42" s="12" t="str">
-        <x:v>false</x:v>
-      </x:c>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="32" customHeight="1">
+      <x:c r="A42" s="12"/>
+      <x:c r="B42" s="12"/>
+      <x:c r="C42" s="12"/>
+      <x:c r="D42" s="12"/>
+      <x:c r="E42" s="13"/>
+      <x:c r="F42" s="12"/>
       <x:c r="G42" s="15" t="str">
         <x:f>IF(B42="","",IFERROR(VLOOKUP(B42,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>conservators_office</x:v>
       </x:c>
       <x:c r="H42" s="15" t="str">
         <x:f>IF(G42="","",IFERROR(VLOOKUP(G42,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Conservator's Office</x:v>
       </x:c>
       <x:c r="I42" s="15" t="str">
         <x:f>IF(B42="","",IFERROR(VLOOKUP(B42,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Left shelving</x:v>
       </x:c>
       <x:c r="J42" s="15" t="str">
         <x:f>IF(B42="","",IFERROR(VLOOKUP(B42,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>collection</x:v>
-      </x:c>
-      <x:c r="K42" s="15" t="n">
+      </x:c>
+      <x:c r="K42" s="15" t="str">
         <x:f>IF(B42="","",IFERROR(VLOOKUP(B42,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43" ht="34" customHeight="1">
-      <x:c r="A43" s="12" t="str">
-        <x:v>draft_conservators_office_shelves_02</x:v>
-      </x:c>
-      <x:c r="B43" s="12" t="str">
-        <x:v>conservators_office_shelves_02</x:v>
-      </x:c>
-      <x:c r="C43" s="12" t="str"/>
-      <x:c r="D43" s="12" t="str">
-        <x:v>detail</x:v>
-      </x:c>
-      <x:c r="E43" s="13" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F43" s="12" t="str">
-        <x:v>false</x:v>
-      </x:c>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="32" customHeight="1">
+      <x:c r="A43" s="12"/>
+      <x:c r="B43" s="12"/>
+      <x:c r="C43" s="12"/>
+      <x:c r="D43" s="12"/>
+      <x:c r="E43" s="13"/>
+      <x:c r="F43" s="12"/>
       <x:c r="G43" s="15" t="str">
         <x:f>IF(B43="","",IFERROR(VLOOKUP(B43,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>conservators_office</x:v>
       </x:c>
       <x:c r="H43" s="15" t="str">
         <x:f>IF(G43="","",IFERROR(VLOOKUP(G43,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Conservator's Office</x:v>
       </x:c>
       <x:c r="I43" s="15" t="str">
         <x:f>IF(B43="","",IFERROR(VLOOKUP(B43,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Rear shelving</x:v>
       </x:c>
       <x:c r="J43" s="15" t="str">
         <x:f>IF(B43="","",IFERROR(VLOOKUP(B43,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>collection</x:v>
-      </x:c>
-      <x:c r="K43" s="15" t="n">
+      </x:c>
+      <x:c r="K43" s="15" t="str">
         <x:f>IF(B43="","",IFERROR(VLOOKUP(B43,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44" ht="34" customHeight="1">
-      <x:c r="A44" s="12" t="str">
-        <x:v>draft_conservators_office_shelves_03</x:v>
-      </x:c>
-      <x:c r="B44" s="12" t="str">
-        <x:v>conservators_office_shelves_03</x:v>
-      </x:c>
-      <x:c r="C44" s="12" t="str"/>
-      <x:c r="D44" s="12" t="str">
-        <x:v>detail</x:v>
-      </x:c>
-      <x:c r="E44" s="13" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F44" s="12" t="str">
-        <x:v>false</x:v>
-      </x:c>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="32" customHeight="1">
+      <x:c r="A44" s="12"/>
+      <x:c r="B44" s="12"/>
+      <x:c r="C44" s="12"/>
+      <x:c r="D44" s="12"/>
+      <x:c r="E44" s="13"/>
+      <x:c r="F44" s="12"/>
       <x:c r="G44" s="15" t="str">
         <x:f>IF(B44="","",IFERROR(VLOOKUP(B44,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>conservators_office</x:v>
       </x:c>
       <x:c r="H44" s="15" t="str">
         <x:f>IF(G44="","",IFERROR(VLOOKUP(G44,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Conservator's Office</x:v>
       </x:c>
       <x:c r="I44" s="15" t="str">
         <x:f>IF(B44="","",IFERROR(VLOOKUP(B44,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Right shelving</x:v>
       </x:c>
       <x:c r="J44" s="15" t="str">
         <x:f>IF(B44="","",IFERROR(VLOOKUP(B44,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>collection</x:v>
-      </x:c>
-      <x:c r="K44" s="15" t="n">
+      </x:c>
+      <x:c r="K44" s="15" t="str">
         <x:f>IF(B44="","",IFERROR(VLOOKUP(B44,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" ht="34" customHeight="1">
-      <x:c r="A45" s="12" t="str">
-        <x:v>draft_lab_bench_01</x:v>
-      </x:c>
-      <x:c r="B45" s="12" t="str">
-        <x:v>lab_bench_01</x:v>
-      </x:c>
-      <x:c r="C45" s="12" t="str"/>
-      <x:c r="D45" s="12" t="str">
-        <x:v>detail</x:v>
-      </x:c>
-      <x:c r="E45" s="13" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F45" s="12" t="str">
-        <x:v>false</x:v>
-      </x:c>
-      <x:c r="G45" s="15" t="str">
-        <x:f>IF(B45="","",IFERROR(VLOOKUP(B45,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>lab</x:v>
-      </x:c>
-      <x:c r="H45" s="15" t="str">
-        <x:f>IF(G45="","",IFERROR(VLOOKUP(G45,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Lab</x:v>
-      </x:c>
-      <x:c r="I45" s="15" t="str">
-        <x:f>IF(B45="","",IFERROR(VLOOKUP(B45,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Analysis bench</x:v>
-      </x:c>
-      <x:c r="J45" s="15" t="str">
-        <x:f>IF(B45="","",IFERROR(VLOOKUP(B45,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>collection</x:v>
-      </x:c>
-      <x:c r="K45" s="15" t="n">
-        <x:f>IF(B45="","",IFERROR(VLOOKUP(B45,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" ht="34" customHeight="1">
-      <x:c r="A46" s="12" t="str">
-        <x:v>draft_lab_equipment_01</x:v>
-      </x:c>
-      <x:c r="B46" s="12" t="str">
-        <x:v>lab_equipment_01</x:v>
-      </x:c>
-      <x:c r="C46" s="12" t="str"/>
-      <x:c r="D46" s="12" t="str">
-        <x:v>detail</x:v>
-      </x:c>
-      <x:c r="E46" s="13" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F46" s="12" t="str">
-        <x:v>false</x:v>
-      </x:c>
-      <x:c r="G46" s="15" t="str">
-        <x:f>IF(B46="","",IFERROR(VLOOKUP(B46,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>lab</x:v>
-      </x:c>
-      <x:c r="H46" s="15" t="str">
-        <x:f>IF(G46="","",IFERROR(VLOOKUP(G46,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Lab</x:v>
-      </x:c>
-      <x:c r="I46" s="15" t="str">
-        <x:f>IF(B46="","",IFERROR(VLOOKUP(B46,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Equipment</x:v>
-      </x:c>
-      <x:c r="J46" s="15" t="str">
-        <x:f>IF(B46="","",IFERROR(VLOOKUP(B46,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>collection</x:v>
-      </x:c>
-      <x:c r="K46" s="15" t="n">
-        <x:f>IF(B46="","",IFERROR(VLOOKUP(B46,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47" ht="34" customHeight="1">
-      <x:c r="A47" s="12" t="str">
-        <x:v>draft_lab_cabinet_01</x:v>
-      </x:c>
-      <x:c r="B47" s="12" t="str">
-        <x:v>lab_cabinet_01</x:v>
-      </x:c>
-      <x:c r="C47" s="12" t="str"/>
-      <x:c r="D47" s="12" t="str">
-        <x:v>detail</x:v>
-      </x:c>
-      <x:c r="E47" s="13" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F47" s="12" t="str">
-        <x:v>false</x:v>
-      </x:c>
-      <x:c r="G47" s="15" t="str">
-        <x:f>IF(B47="","",IFERROR(VLOOKUP(B47,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>lab</x:v>
-      </x:c>
-      <x:c r="H47" s="15" t="str">
-        <x:f>IF(G47="","",IFERROR(VLOOKUP(G47,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Lab</x:v>
-      </x:c>
-      <x:c r="I47" s="15" t="str">
-        <x:f>IF(B47="","",IFERROR(VLOOKUP(B47,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Left cabinet</x:v>
-      </x:c>
-      <x:c r="J47" s="15" t="str">
-        <x:f>IF(B47="","",IFERROR(VLOOKUP(B47,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>collection</x:v>
-      </x:c>
-      <x:c r="K47" s="15" t="n">
-        <x:f>IF(B47="","",IFERROR(VLOOKUP(B47,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48" ht="34" customHeight="1">
-      <x:c r="A48" s="12" t="str">
-        <x:v>draft_lab_cabinet_02</x:v>
-      </x:c>
-      <x:c r="B48" s="12" t="str">
-        <x:v>lab_cabinet_02</x:v>
-      </x:c>
-      <x:c r="C48" s="12" t="str"/>
-      <x:c r="D48" s="12" t="str">
-        <x:v>detail</x:v>
-      </x:c>
-      <x:c r="E48" s="13" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F48" s="12" t="str">
-        <x:v>false</x:v>
-      </x:c>
-      <x:c r="G48" s="15" t="str">
-        <x:f>IF(B48="","",IFERROR(VLOOKUP(B48,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>lab</x:v>
-      </x:c>
-      <x:c r="H48" s="15" t="str">
-        <x:f>IF(G48="","",IFERROR(VLOOKUP(G48,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Lab</x:v>
-      </x:c>
-      <x:c r="I48" s="15" t="str">
-        <x:f>IF(B48="","",IFERROR(VLOOKUP(B48,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Right cabinet</x:v>
-      </x:c>
-      <x:c r="J48" s="15" t="str">
-        <x:f>IF(B48="","",IFERROR(VLOOKUP(B48,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>collection</x:v>
-      </x:c>
-      <x:c r="K48" s="15" t="n">
-        <x:f>IF(B48="","",IFERROR(VLOOKUP(B48,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49" ht="32" customHeight="1">
-      <x:c r="A49" s="12"/>
-      <x:c r="B49" s="12"/>
-      <x:c r="C49" s="12"/>
-      <x:c r="D49" s="12"/>
-      <x:c r="E49" s="13"/>
-      <x:c r="F49" s="12"/>
-      <x:c r="G49" s="15" t="str">
-        <x:f>IF(B49="","",IFERROR(VLOOKUP(B49,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="H49" s="15" t="str">
-        <x:f>IF(G49="","",IFERROR(VLOOKUP(G49,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-      </x:c>
-      <x:c r="I49" s="15" t="str">
-        <x:f>IF(B49="","",IFERROR(VLOOKUP(B49,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="J49" s="15" t="str">
-        <x:f>IF(B49="","",IFERROR(VLOOKUP(B49,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K49" s="15" t="str">
-        <x:f>IF(B49="","",IFERROR(VLOOKUP(B49,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="50" ht="32" customHeight="1">
-      <x:c r="A50" s="12"/>
-      <x:c r="B50" s="12"/>
-      <x:c r="C50" s="12"/>
-      <x:c r="D50" s="12"/>
-      <x:c r="E50" s="13"/>
-      <x:c r="F50" s="12"/>
-      <x:c r="G50" s="15" t="str">
-        <x:f>IF(B50="","",IFERROR(VLOOKUP(B50,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="H50" s="15" t="str">
-        <x:f>IF(G50="","",IFERROR(VLOOKUP(G50,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-      </x:c>
-      <x:c r="I50" s="15" t="str">
-        <x:f>IF(B50="","",IFERROR(VLOOKUP(B50,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="J50" s="15" t="str">
-        <x:f>IF(B50="","",IFERROR(VLOOKUP(B50,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K50" s="15" t="str">
-        <x:f>IF(B50="","",IFERROR(VLOOKUP(B50,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="51" ht="32" customHeight="1">
-      <x:c r="A51" s="12"/>
-      <x:c r="B51" s="12"/>
-      <x:c r="C51" s="12"/>
-      <x:c r="D51" s="12"/>
-      <x:c r="E51" s="13"/>
-      <x:c r="F51" s="12"/>
-      <x:c r="G51" s="15" t="str">
-        <x:f>IF(B51="","",IFERROR(VLOOKUP(B51,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="H51" s="15" t="str">
-        <x:f>IF(G51="","",IFERROR(VLOOKUP(G51,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-      </x:c>
-      <x:c r="I51" s="15" t="str">
-        <x:f>IF(B51="","",IFERROR(VLOOKUP(B51,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="J51" s="15" t="str">
-        <x:f>IF(B51="","",IFERROR(VLOOKUP(B51,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K51" s="15" t="str">
-        <x:f>IF(B51="","",IFERROR(VLOOKUP(B51,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="52" ht="32" customHeight="1">
-      <x:c r="A52" s="12"/>
-      <x:c r="B52" s="12"/>
-      <x:c r="C52" s="12"/>
-      <x:c r="D52" s="12"/>
-      <x:c r="E52" s="13"/>
-      <x:c r="F52" s="12"/>
-      <x:c r="G52" s="15" t="str">
-        <x:f>IF(B52="","",IFERROR(VLOOKUP(B52,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="H52" s="15" t="str">
-        <x:f>IF(G52="","",IFERROR(VLOOKUP(G52,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-      </x:c>
-      <x:c r="I52" s="15" t="str">
-        <x:f>IF(B52="","",IFERROR(VLOOKUP(B52,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="J52" s="15" t="str">
-        <x:f>IF(B52="","",IFERROR(VLOOKUP(B52,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K52" s="15" t="str">
-        <x:f>IF(B52="","",IFERROR(VLOOKUP(B52,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="53" ht="32" customHeight="1">
-      <x:c r="A53" s="12"/>
-      <x:c r="B53" s="12"/>
-      <x:c r="C53" s="12"/>
-      <x:c r="D53" s="12"/>
-      <x:c r="E53" s="13"/>
-      <x:c r="F53" s="12"/>
-      <x:c r="G53" s="15" t="str">
-        <x:f>IF(B53="","",IFERROR(VLOOKUP(B53,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="H53" s="15" t="str">
-        <x:f>IF(G53="","",IFERROR(VLOOKUP(G53,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-      </x:c>
-      <x:c r="I53" s="15" t="str">
-        <x:f>IF(B53="","",IFERROR(VLOOKUP(B53,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="J53" s="15" t="str">
-        <x:f>IF(B53="","",IFERROR(VLOOKUP(B53,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K53" s="15" t="str">
-        <x:f>IF(B53="","",IFERROR(VLOOKUP(B53,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="54" ht="32" customHeight="1">
-      <x:c r="A54" s="12"/>
-      <x:c r="B54" s="12"/>
-      <x:c r="C54" s="12"/>
-      <x:c r="D54" s="12"/>
-      <x:c r="E54" s="13"/>
-      <x:c r="F54" s="12"/>
-      <x:c r="G54" s="15" t="str">
-        <x:f>IF(B54="","",IFERROR(VLOOKUP(B54,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="H54" s="15" t="str">
-        <x:f>IF(G54="","",IFERROR(VLOOKUP(G54,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-      </x:c>
-      <x:c r="I54" s="15" t="str">
-        <x:f>IF(B54="","",IFERROR(VLOOKUP(B54,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="J54" s="15" t="str">
-        <x:f>IF(B54="","",IFERROR(VLOOKUP(B54,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K54" s="15" t="str">
-        <x:f>IF(B54="","",IFERROR(VLOOKUP(B54,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="55" ht="32" customHeight="1">
-      <x:c r="A55" s="12"/>
-      <x:c r="B55" s="12"/>
-      <x:c r="C55" s="12"/>
-      <x:c r="D55" s="12"/>
-      <x:c r="E55" s="13"/>
-      <x:c r="F55" s="12"/>
-      <x:c r="G55" s="15" t="str">
-        <x:f>IF(B55="","",IFERROR(VLOOKUP(B55,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="H55" s="15" t="str">
-        <x:f>IF(G55="","",IFERROR(VLOOKUP(G55,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-      </x:c>
-      <x:c r="I55" s="15" t="str">
-        <x:f>IF(B55="","",IFERROR(VLOOKUP(B55,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="J55" s="15" t="str">
-        <x:f>IF(B55="","",IFERROR(VLOOKUP(B55,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K55" s="15" t="str">
-        <x:f>IF(B55="","",IFERROR(VLOOKUP(B55,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="56" ht="32" customHeight="1">
-      <x:c r="A56" s="12"/>
-      <x:c r="B56" s="12"/>
-      <x:c r="C56" s="12"/>
-      <x:c r="D56" s="12"/>
-      <x:c r="E56" s="13"/>
-      <x:c r="F56" s="12"/>
-      <x:c r="G56" s="15" t="str">
-        <x:f>IF(B56="","",IFERROR(VLOOKUP(B56,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="H56" s="15" t="str">
-        <x:f>IF(G56="","",IFERROR(VLOOKUP(G56,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-      </x:c>
-      <x:c r="I56" s="15" t="str">
-        <x:f>IF(B56="","",IFERROR(VLOOKUP(B56,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="J56" s="15" t="str">
-        <x:f>IF(B56="","",IFERROR(VLOOKUP(B56,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K56" s="15" t="str">
-        <x:f>IF(B56="","",IFERROR(VLOOKUP(B56,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="57" ht="32" customHeight="1">
-      <x:c r="A57" s="12"/>
-      <x:c r="B57" s="12"/>
-      <x:c r="C57" s="12"/>
-      <x:c r="D57" s="12"/>
-      <x:c r="E57" s="13"/>
-      <x:c r="F57" s="12"/>
-      <x:c r="G57" s="15" t="str">
-        <x:f>IF(B57="","",IFERROR(VLOOKUP(B57,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="H57" s="15" t="str">
-        <x:f>IF(G57="","",IFERROR(VLOOKUP(G57,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-      </x:c>
-      <x:c r="I57" s="15" t="str">
-        <x:f>IF(B57="","",IFERROR(VLOOKUP(B57,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="J57" s="15" t="str">
-        <x:f>IF(B57="","",IFERROR(VLOOKUP(B57,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K57" s="15" t="str">
-        <x:f>IF(B57="","",IFERROR(VLOOKUP(B57,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="58" ht="32" customHeight="1">
-      <x:c r="A58" s="12"/>
-      <x:c r="B58" s="12"/>
-      <x:c r="C58" s="12"/>
-      <x:c r="D58" s="12"/>
-      <x:c r="E58" s="13"/>
-      <x:c r="F58" s="12"/>
-      <x:c r="G58" s="15" t="str">
-        <x:f>IF(B58="","",IFERROR(VLOOKUP(B58,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="H58" s="15" t="str">
-        <x:f>IF(G58="","",IFERROR(VLOOKUP(G58,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-      </x:c>
-      <x:c r="I58" s="15" t="str">
-        <x:f>IF(B58="","",IFERROR(VLOOKUP(B58,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="J58" s="15" t="str">
-        <x:f>IF(B58="","",IFERROR(VLOOKUP(B58,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K58" s="15" t="str">
-        <x:f>IF(B58="","",IFERROR(VLOOKUP(B58,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="59" ht="32" customHeight="1">
-      <x:c r="A59" s="12"/>
-      <x:c r="B59" s="12"/>
-      <x:c r="C59" s="12"/>
-      <x:c r="D59" s="12"/>
-      <x:c r="E59" s="13"/>
-      <x:c r="F59" s="12"/>
-      <x:c r="G59" s="15" t="str">
-        <x:f>IF(B59="","",IFERROR(VLOOKUP(B59,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="H59" s="15" t="str">
-        <x:f>IF(G59="","",IFERROR(VLOOKUP(G59,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-      </x:c>
-      <x:c r="I59" s="15" t="str">
-        <x:f>IF(B59="","",IFERROR(VLOOKUP(B59,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="J59" s="15" t="str">
-        <x:f>IF(B59="","",IFERROR(VLOOKUP(B59,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K59" s="15" t="str">
-        <x:f>IF(B59="","",IFERROR(VLOOKUP(B59,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="60" ht="32" customHeight="1">
-      <x:c r="A60" s="12"/>
-      <x:c r="B60" s="12"/>
-      <x:c r="C60" s="12"/>
-      <x:c r="D60" s="12"/>
-      <x:c r="E60" s="13"/>
-      <x:c r="F60" s="12"/>
-      <x:c r="G60" s="15" t="str">
-        <x:f>IF(B60="","",IFERROR(VLOOKUP(B60,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="H60" s="15" t="str">
-        <x:f>IF(G60="","",IFERROR(VLOOKUP(G60,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-      </x:c>
-      <x:c r="I60" s="15" t="str">
-        <x:f>IF(B60="","",IFERROR(VLOOKUP(B60,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="J60" s="15" t="str">
-        <x:f>IF(B60="","",IFERROR(VLOOKUP(B60,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K60" s="15" t="str">
-        <x:f>IF(B60="","",IFERROR(VLOOKUP(B60,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="61" ht="32" customHeight="1">
-      <x:c r="A61" s="12"/>
-      <x:c r="B61" s="12"/>
-      <x:c r="C61" s="12"/>
-      <x:c r="D61" s="12"/>
-      <x:c r="E61" s="13"/>
-      <x:c r="F61" s="12"/>
-      <x:c r="G61" s="15" t="str">
-        <x:f>IF(B61="","",IFERROR(VLOOKUP(B61,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="H61" s="15" t="str">
-        <x:f>IF(G61="","",IFERROR(VLOOKUP(G61,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-      </x:c>
-      <x:c r="I61" s="15" t="str">
-        <x:f>IF(B61="","",IFERROR(VLOOKUP(B61,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="J61" s="15" t="str">
-        <x:f>IF(B61="","",IFERROR(VLOOKUP(B61,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K61" s="15" t="str">
-        <x:f>IF(B61="","",IFERROR(VLOOKUP(B61,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="62" ht="32" customHeight="1">
-      <x:c r="A62" s="12"/>
-      <x:c r="B62" s="12"/>
-      <x:c r="C62" s="12"/>
-      <x:c r="D62" s="12"/>
-      <x:c r="E62" s="13"/>
-      <x:c r="F62" s="12"/>
-      <x:c r="G62" s="15" t="str">
-        <x:f>IF(B62="","",IFERROR(VLOOKUP(B62,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="H62" s="15" t="str">
-        <x:f>IF(G62="","",IFERROR(VLOOKUP(G62,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-      </x:c>
-      <x:c r="I62" s="15" t="str">
-        <x:f>IF(B62="","",IFERROR(VLOOKUP(B62,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="J62" s="15" t="str">
-        <x:f>IF(B62="","",IFERROR(VLOOKUP(B62,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K62" s="15" t="str">
-        <x:f>IF(B62="","",IFERROR(VLOOKUP(B62,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="63" ht="32" customHeight="1">
-      <x:c r="A63" s="12"/>
-      <x:c r="B63" s="12"/>
-      <x:c r="C63" s="12"/>
-      <x:c r="D63" s="12"/>
-      <x:c r="E63" s="13"/>
-      <x:c r="F63" s="12"/>
-      <x:c r="G63" s="15" t="str">
-        <x:f>IF(B63="","",IFERROR(VLOOKUP(B63,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="H63" s="15" t="str">
-        <x:f>IF(G63="","",IFERROR(VLOOKUP(G63,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-      </x:c>
-      <x:c r="I63" s="15" t="str">
-        <x:f>IF(B63="","",IFERROR(VLOOKUP(B63,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="J63" s="15" t="str">
-        <x:f>IF(B63="","",IFERROR(VLOOKUP(B63,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K63" s="15" t="str">
-        <x:f>IF(B63="","",IFERROR(VLOOKUP(B63,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="C2:C63">
+  <x:conditionalFormatting sqref="C2:C44">
     <x:cfRule type="expression" dxfId="0" priority="1">
       <x:formula>AND($A2&lt;&gt;"",$C2="")</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="B2:B63">
+  <x:conditionalFormatting sqref="B2:B44">
     <x:cfRule type="expression" dxfId="1" priority="2">
       <x:formula>AND($A2&lt;&gt;"",$B2&lt;&gt;"",COUNTIF(Slots!$A$2:$A$501,$B2)=0)</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="F2:F63">
+  <x:conditionalFormatting sqref="F2:F44">
     <x:cfRule type="expression" dxfId="2" priority="3">
       <x:formula>AND($A2&lt;&gt;"",$F2="true",COUNTIFS($B$2:$B$501,$B2,$E$2:$E$501,$E2,$F$2:$F$501,"true")&gt;1)</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="E2:E63">
+  <x:conditionalFormatting sqref="E2:E44">
     <x:cfRule type="expression" dxfId="3" priority="4">
       <x:formula>AND($A2&lt;&gt;"",$F2="true",$E2&lt;&gt;"",COUNTIFS($B$2:$B$501,$B2,$E$2:$E$501,$E2,$F$2:$F$501,"true")&gt;1)</x:formula>
     </x:cfRule>
@@ -2790,7 +2070,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f049993c1ff409f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb8f9943b3944d57"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3287,14 +2567,24 @@
       <x:c r="F26" s="12" t="str"/>
       <x:c r="G26" s="12" t="str"/>
     </x:row>
-    <x:row r="27" ht="32" customHeight="1">
-      <x:c r="A27" s="12"/>
-      <x:c r="B27" s="12"/>
-      <x:c r="C27" s="12"/>
-      <x:c r="D27" s="12"/>
-      <x:c r="E27" s="16"/>
-      <x:c r="F27" s="12"/>
-      <x:c r="G27" s="12"/>
+    <x:row r="27" ht="34" customHeight="1">
+      <x:c r="A27" s="12" t="str">
+        <x:v>geib-flute</x:v>
+      </x:c>
+      <x:c r="B27" s="12" t="str">
+        <x:v>Geib Flute</x:v>
+      </x:c>
+      <x:c r="C27" s="12" t="str">
+        <x:v>test</x:v>
+      </x:c>
+      <x:c r="D27" s="12" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E27" s="16" t="str"/>
+      <x:c r="F27" s="12" t="str">
+        <x:v>/assets/img/editorial/geib-flute-3ec90b3a3ce8.jpeg</x:v>
+      </x:c>
+      <x:c r="G27" s="12" t="str"/>
     </x:row>
     <x:row r="28" ht="32" customHeight="1">
       <x:c r="A28" s="12"/>
@@ -3422,6 +2712,15 @@
       <x:c r="F41" s="12"/>
       <x:c r="G41" s="12"/>
     </x:row>
+    <x:row r="42" ht="32" customHeight="1">
+      <x:c r="A42" s="12"/>
+      <x:c r="B42" s="12"/>
+      <x:c r="C42" s="12"/>
+      <x:c r="D42" s="12"/>
+      <x:c r="E42" s="16"/>
+      <x:c r="F42" s="12"/>
+      <x:c r="G42" s="12"/>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="D2:D501">
@@ -3430,7 +2729,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09e92d2bf3554497"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6895ef182dd4d11"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4084,7 +3383,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83d4c2c883cb4067"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b3c8770a7f04d8d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4324,7 +3623,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf04caeb299d84ab1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80e09748f4a44bdd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4604,7 +3903,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R700f09465b8748f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra703ac2c40a1469b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6154,7 +5453,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0384a261f5b3489f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc331f24ec500493a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6694,7 +5993,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38a2304ed9024c31"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84ce73e7a8fd4c13"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6891,7 +6190,7 @@
         <x:v>_data/placements.csv</x:v>
       </x:c>
       <x:c r="B23" s="24" t="str">
-        <x:v>087a2f718b5ee1c6783cafeb30f16a5ad934822d66ecf6c0484d19156f86b918</x:v>
+        <x:v>a07011a65d6dec2fc9ed28b5e10d4aa2fc3b613a593d5296654ccbe7e062d813</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="58" customHeight="1">
@@ -6899,7 +6198,7 @@
         <x:v>_data/room_content.csv</x:v>
       </x:c>
       <x:c r="B24" s="24" t="str">
-        <x:v>c859709397870b691cca329d6d1ec56fb9dc756d035b2636081111dc46ecebf6</x:v>
+        <x:v>fed299761ab52e9c4c50988789cf740082a9035d97745f7e2a879f57c08a6763</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="58" customHeight="1">
@@ -6907,7 +6206,7 @@
         <x:v>_data/timeline_events.csv</x:v>
       </x:c>
       <x:c r="B25" s="24" t="str">
-        <x:v>6d440f2d8e35129dc48ee25acadc58e8491ea7bfea2e6b250ab9c792731c031e</x:v>
+        <x:v>1e783da63ae487794669258fcdc30342bf647796258d2fdd28d134c54f88f722</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="58" customHeight="1">
@@ -6915,7 +6214,7 @@
         <x:v>_data/room_timelines.csv</x:v>
       </x:c>
       <x:c r="B26" s="24" t="str">
-        <x:v>5b177dd4ed184a477cf576a2a6b5d86871b8f2332f353c70e0177ebaff2a68c0</x:v>
+        <x:v>24dc2020209d20195d39ff7fd7497d560db9f86e846752d8d3ccbd90c428722c</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="58" customHeight="1">
@@ -6923,7 +6222,7 @@
         <x:v>_data/rooms.csv</x:v>
       </x:c>
       <x:c r="B27" s="24" t="str">
-        <x:v>9de7372fc7eff45ffcb4fb71f0686068f46e8401632faa59971ffb9e42c15fb5</x:v>
+        <x:v>8614c904f8ec00274a1b8c7198e5910f350e761c0cdf5203cb48afce61557b35</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="58" customHeight="1">
@@ -6931,7 +6230,7 @@
         <x:v>_data/exhibit_slots.csv</x:v>
       </x:c>
       <x:c r="B28" s="24" t="str">
-        <x:v>d3e4333d6d7ec2dd97f99009148754df2099538d822c07f0c6d7f0bb2e0270ac</x:v>
+        <x:v>61f0da63b21935f1116ed34da3e824716b98af51a209f83c7bd993fbc99aae02</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="58" customHeight="1">
@@ -6939,7 +6238,7 @@
         <x:v>_data/demo-metadata.csv</x:v>
       </x:c>
       <x:c r="B29" s="24" t="str">
-        <x:v>4b52545ce188c6aadc29a35bfe23c0c935ab202baaa080c7a0dee9fa4257b543</x:v>
+        <x:v>7bd0bf689e14b3c0bf3dcaba7cc8f289f4be361750c6cda612fc8c45c8c5829b</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Enable visual editorial mounts for shared media
Use the existing anchor capability model: presentation_mode remains
interaction behavior, while inline_content controls in-room media
rendering. Mark only the existing reserved Gallery rear display and
Natural History recessed panel as visual editorial mounts; retain
interaction-only behavior for illustrated fixtures, tools, and authored
scenery.

Move the published Geib Flute placement to the enabled Natural History
recessed-panel mount. Regenerate the editorial workbook so its data and
stale-source hashes match the authoritative CSVs. Harden the media
resolver to treat only true or 'true' inline_content values as visual
capabilities, and cover this plus Geib unpublishing in focused tests.

Document the semantics and full 45-slot capability classification.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/archivory-editorial/ArchIvory Editorial Workbook.xlsx
+++ b/outputs/archivory-editorial/ArchIvory Editorial Workbook.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Placements" sheetId="1" r:id="Rf9fb81c59d2d442d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content" sheetId="2" r:id="Rbe706e17fb9a417d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="3" r:id="R15f8978f1cfe421b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timelines" sheetId="4" r:id="Rabbebed5e7af4dd6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rooms" sheetId="5" r:id="Re21abc23a4584d29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slots" sheetId="6" r:id="R0dd33f77310d47ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection" sheetId="7" r:id="Rde3aeb45d1ed4b63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="Rfbb2d1e9fb5940e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Placements" sheetId="1" r:id="R62910e8b1e654193"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content" sheetId="2" r:id="R6d706709117c4efa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="3" r:id="R01e5051be94b407c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timelines" sheetId="4" r:id="R94869fca09e74b1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rooms" sheetId="5" r:id="Rd30042ed73c7471a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slots" sheetId="6" r:id="Rcefcced59951437a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection" sheetId="7" r:id="Rd196e7bcbe854e56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="R3e85da649fc9454b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -196,7 +196,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PlacementsTable" displayName="PlacementsTable" ref="A1:K44" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PlacementsTable" displayName="PlacementsTable" ref="A1:K63" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="placement_id"/>
     <x:tableColumn id="2" name="slot_id"/>
@@ -1653,7 +1653,7 @@
         <x:v>geib-flute</x:v>
       </x:c>
       <x:c r="B29" s="12" t="str">
-        <x:v>gallery_wall_01</x:v>
+        <x:v>natural_history_panel_02</x:v>
       </x:c>
       <x:c r="C29" s="12" t="str">
         <x:v>geib-flute</x:v>
@@ -1669,15 +1669,15 @@
       </x:c>
       <x:c r="G29" s="15" t="str">
         <x:f>IF(B29="","",IFERROR(VLOOKUP(B29,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>gallery</x:v>
+        <x:v>natural_history</x:v>
       </x:c>
       <x:c r="H29" s="15" t="str">
         <x:f>IF(G29="","",IFERROR(VLOOKUP(G29,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Gallery</x:v>
+        <x:v>Natural History Museum</x:v>
       </x:c>
       <x:c r="I29" s="15" t="str">
         <x:f>IF(B29="","",IFERROR(VLOOKUP(B29,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Near left-wall relief</x:v>
+        <x:v>Central recessed panel</x:v>
       </x:c>
       <x:c r="J29" s="15" t="str">
         <x:f>IF(B29="","",IFERROR(VLOOKUP(B29,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
@@ -1688,368 +1688,1090 @@
         <x:v>8</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="32" customHeight="1">
-      <x:c r="A30" s="12"/>
-      <x:c r="B30" s="12"/>
-      <x:c r="C30" s="12"/>
-      <x:c r="D30" s="12"/>
-      <x:c r="E30" s="13"/>
-      <x:c r="F30" s="12"/>
+    <x:row r="30" ht="34" customHeight="1">
+      <x:c r="A30" s="12" t="str">
+        <x:v>draft_historical_society_intro</x:v>
+      </x:c>
+      <x:c r="B30" s="12" t="str">
+        <x:v>historical_society_intro</x:v>
+      </x:c>
+      <x:c r="C30" s="12" t="str"/>
+      <x:c r="D30" s="12" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E30" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F30" s="12" t="str">
+        <x:v>false</x:v>
+      </x:c>
       <x:c r="G30" s="15" t="str">
         <x:f>IF(B30="","",IFERROR(VLOOKUP(B30,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+        <x:v>historical_society</x:v>
       </x:c>
       <x:c r="H30" s="15" t="str">
         <x:f>IF(G30="","",IFERROR(VLOOKUP(G30,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Historical Society</x:v>
       </x:c>
       <x:c r="I30" s="15" t="str">
         <x:f>IF(B30="","",IFERROR(VLOOKUP(B30,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+        <x:v>Historical Society introduction</x:v>
       </x:c>
       <x:c r="J30" s="15" t="str">
         <x:f>IF(B30="","",IFERROR(VLOOKUP(B30,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K30" s="15" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="K30" s="15" t="n">
         <x:f>IF(B30="","",IFERROR(VLOOKUP(B30,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="32" customHeight="1">
-      <x:c r="A31" s="12"/>
-      <x:c r="B31" s="12"/>
-      <x:c r="C31" s="12"/>
-      <x:c r="D31" s="12"/>
-      <x:c r="E31" s="13"/>
-      <x:c r="F31" s="12"/>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="34" customHeight="1">
+      <x:c r="A31" s="12" t="str">
+        <x:v>draft_attic_intro</x:v>
+      </x:c>
+      <x:c r="B31" s="12" t="str">
+        <x:v>attic_intro</x:v>
+      </x:c>
+      <x:c r="C31" s="12" t="str"/>
+      <x:c r="D31" s="12" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E31" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F31" s="12" t="str">
+        <x:v>false</x:v>
+      </x:c>
       <x:c r="G31" s="15" t="str">
         <x:f>IF(B31="","",IFERROR(VLOOKUP(B31,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+        <x:v>attic</x:v>
       </x:c>
       <x:c r="H31" s="15" t="str">
         <x:f>IF(G31="","",IFERROR(VLOOKUP(G31,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Attic</x:v>
       </x:c>
       <x:c r="I31" s="15" t="str">
         <x:f>IF(B31="","",IFERROR(VLOOKUP(B31,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+        <x:v>Attic introduction</x:v>
       </x:c>
       <x:c r="J31" s="15" t="str">
         <x:f>IF(B31="","",IFERROR(VLOOKUP(B31,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K31" s="15" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="K31" s="15" t="n">
         <x:f>IF(B31="","",IFERROR(VLOOKUP(B31,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="32" customHeight="1">
-      <x:c r="A32" s="12"/>
-      <x:c r="B32" s="12"/>
-      <x:c r="C32" s="12"/>
-      <x:c r="D32" s="12"/>
-      <x:c r="E32" s="13"/>
-      <x:c r="F32" s="12"/>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="34" customHeight="1">
+      <x:c r="A32" s="12" t="str">
+        <x:v>draft_natural_history_intro</x:v>
+      </x:c>
+      <x:c r="B32" s="12" t="str">
+        <x:v>natural_history_intro</x:v>
+      </x:c>
+      <x:c r="C32" s="12" t="str"/>
+      <x:c r="D32" s="12" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E32" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F32" s="12" t="str">
+        <x:v>false</x:v>
+      </x:c>
       <x:c r="G32" s="15" t="str">
         <x:f>IF(B32="","",IFERROR(VLOOKUP(B32,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+        <x:v>natural_history</x:v>
       </x:c>
       <x:c r="H32" s="15" t="str">
         <x:f>IF(G32="","",IFERROR(VLOOKUP(G32,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Natural History Museum</x:v>
       </x:c>
       <x:c r="I32" s="15" t="str">
         <x:f>IF(B32="","",IFERROR(VLOOKUP(B32,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+        <x:v>Natural History Museum introduction</x:v>
       </x:c>
       <x:c r="J32" s="15" t="str">
         <x:f>IF(B32="","",IFERROR(VLOOKUP(B32,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K32" s="15" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="K32" s="15" t="n">
         <x:f>IF(B32="","",IFERROR(VLOOKUP(B32,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="32" customHeight="1">
-      <x:c r="A33" s="12"/>
-      <x:c r="B33" s="12"/>
-      <x:c r="C33" s="12"/>
-      <x:c r="D33" s="12"/>
-      <x:c r="E33" s="13"/>
-      <x:c r="F33" s="12"/>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="34" customHeight="1">
+      <x:c r="A33" s="12" t="str">
+        <x:v>draft_conservators_office_intro</x:v>
+      </x:c>
+      <x:c r="B33" s="12" t="str">
+        <x:v>conservators_office_intro</x:v>
+      </x:c>
+      <x:c r="C33" s="12" t="str"/>
+      <x:c r="D33" s="12" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E33" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F33" s="12" t="str">
+        <x:v>false</x:v>
+      </x:c>
       <x:c r="G33" s="15" t="str">
         <x:f>IF(B33="","",IFERROR(VLOOKUP(B33,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+        <x:v>conservators_office</x:v>
       </x:c>
       <x:c r="H33" s="15" t="str">
         <x:f>IF(G33="","",IFERROR(VLOOKUP(G33,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Conservator's Office</x:v>
       </x:c>
       <x:c r="I33" s="15" t="str">
         <x:f>IF(B33="","",IFERROR(VLOOKUP(B33,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+        <x:v>Conservator's Office introduction</x:v>
       </x:c>
       <x:c r="J33" s="15" t="str">
         <x:f>IF(B33="","",IFERROR(VLOOKUP(B33,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K33" s="15" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="K33" s="15" t="n">
         <x:f>IF(B33="","",IFERROR(VLOOKUP(B33,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="32" customHeight="1">
-      <x:c r="A34" s="12"/>
-      <x:c r="B34" s="12"/>
-      <x:c r="C34" s="12"/>
-      <x:c r="D34" s="12"/>
-      <x:c r="E34" s="13"/>
-      <x:c r="F34" s="12"/>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="34" customHeight="1">
+      <x:c r="A34" s="12" t="str">
+        <x:v>draft_lab_intro</x:v>
+      </x:c>
+      <x:c r="B34" s="12" t="str">
+        <x:v>lab_intro</x:v>
+      </x:c>
+      <x:c r="C34" s="12" t="str"/>
+      <x:c r="D34" s="12" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E34" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F34" s="12" t="str">
+        <x:v>false</x:v>
+      </x:c>
       <x:c r="G34" s="15" t="str">
         <x:f>IF(B34="","",IFERROR(VLOOKUP(B34,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+        <x:v>lab</x:v>
       </x:c>
       <x:c r="H34" s="15" t="str">
         <x:f>IF(G34="","",IFERROR(VLOOKUP(G34,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Lab</x:v>
       </x:c>
       <x:c r="I34" s="15" t="str">
         <x:f>IF(B34="","",IFERROR(VLOOKUP(B34,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+        <x:v>Lab introduction</x:v>
       </x:c>
       <x:c r="J34" s="15" t="str">
         <x:f>IF(B34="","",IFERROR(VLOOKUP(B34,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K34" s="15" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="K34" s="15" t="n">
         <x:f>IF(B34="","",IFERROR(VLOOKUP(B34,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="32" customHeight="1">
-      <x:c r="A35" s="12"/>
-      <x:c r="B35" s="12"/>
-      <x:c r="C35" s="12"/>
-      <x:c r="D35" s="12"/>
-      <x:c r="E35" s="13"/>
-      <x:c r="F35" s="12"/>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="34" customHeight="1">
+      <x:c r="A35" s="12" t="str">
+        <x:v>draft_gallery_case_02</x:v>
+      </x:c>
+      <x:c r="B35" s="12" t="str">
+        <x:v>gallery_case_02</x:v>
+      </x:c>
+      <x:c r="C35" s="12" t="str"/>
+      <x:c r="D35" s="12" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E35" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F35" s="12" t="str">
+        <x:v>false</x:v>
+      </x:c>
       <x:c r="G35" s="15" t="str">
         <x:f>IF(B35="","",IFERROR(VLOOKUP(B35,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+        <x:v>gallery</x:v>
       </x:c>
       <x:c r="H35" s="15" t="str">
         <x:f>IF(G35="","",IFERROR(VLOOKUP(G35,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Gallery</x:v>
       </x:c>
       <x:c r="I35" s="15" t="str">
         <x:f>IF(B35="","",IFERROR(VLOOKUP(B35,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+        <x:v>Rear round display</x:v>
       </x:c>
       <x:c r="J35" s="15" t="str">
         <x:f>IF(B35="","",IFERROR(VLOOKUP(B35,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K35" s="15" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K35" s="15" t="n">
         <x:f>IF(B35="","",IFERROR(VLOOKUP(B35,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="32" customHeight="1">
-      <x:c r="A36" s="12"/>
-      <x:c r="B36" s="12"/>
-      <x:c r="C36" s="12"/>
-      <x:c r="D36" s="12"/>
-      <x:c r="E36" s="13"/>
-      <x:c r="F36" s="12"/>
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="34" customHeight="1">
+      <x:c r="A36" s="12" t="str">
+        <x:v>draft_historical_society_case_01</x:v>
+      </x:c>
+      <x:c r="B36" s="12" t="str">
+        <x:v>historical_society_case_01</x:v>
+      </x:c>
+      <x:c r="C36" s="12" t="str"/>
+      <x:c r="D36" s="12" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E36" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F36" s="12" t="str">
+        <x:v>false</x:v>
+      </x:c>
       <x:c r="G36" s="15" t="str">
         <x:f>IF(B36="","",IFERROR(VLOOKUP(B36,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+        <x:v>historical_society</x:v>
       </x:c>
       <x:c r="H36" s="15" t="str">
         <x:f>IF(G36="","",IFERROR(VLOOKUP(G36,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Historical Society</x:v>
       </x:c>
       <x:c r="I36" s="15" t="str">
         <x:f>IF(B36="","",IFERROR(VLOOKUP(B36,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+        <x:v>Window-side case</x:v>
       </x:c>
       <x:c r="J36" s="15" t="str">
         <x:f>IF(B36="","",IFERROR(VLOOKUP(B36,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K36" s="15" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K36" s="15" t="n">
         <x:f>IF(B36="","",IFERROR(VLOOKUP(B36,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="32" customHeight="1">
-      <x:c r="A37" s="12"/>
-      <x:c r="B37" s="12"/>
-      <x:c r="C37" s="12"/>
-      <x:c r="D37" s="12"/>
-      <x:c r="E37" s="13"/>
-      <x:c r="F37" s="12"/>
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="34" customHeight="1">
+      <x:c r="A37" s="12" t="str">
+        <x:v>draft_historical_society_case_02</x:v>
+      </x:c>
+      <x:c r="B37" s="12" t="str">
+        <x:v>historical_society_case_02</x:v>
+      </x:c>
+      <x:c r="C37" s="12" t="str"/>
+      <x:c r="D37" s="12" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E37" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F37" s="12" t="str">
+        <x:v>false</x:v>
+      </x:c>
       <x:c r="G37" s="15" t="str">
         <x:f>IF(B37="","",IFERROR(VLOOKUP(B37,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+        <x:v>historical_society</x:v>
       </x:c>
       <x:c r="H37" s="15" t="str">
         <x:f>IF(G37="","",IFERROR(VLOOKUP(G37,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Historical Society</x:v>
       </x:c>
       <x:c r="I37" s="15" t="str">
         <x:f>IF(B37="","",IFERROR(VLOOKUP(B37,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+        <x:v>Foreground-right case</x:v>
       </x:c>
       <x:c r="J37" s="15" t="str">
         <x:f>IF(B37="","",IFERROR(VLOOKUP(B37,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K37" s="15" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K37" s="15" t="n">
         <x:f>IF(B37="","",IFERROR(VLOOKUP(B37,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="32" customHeight="1">
-      <x:c r="A38" s="12"/>
-      <x:c r="B38" s="12"/>
-      <x:c r="C38" s="12"/>
-      <x:c r="D38" s="12"/>
-      <x:c r="E38" s="13"/>
-      <x:c r="F38" s="12"/>
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="34" customHeight="1">
+      <x:c r="A38" s="12" t="str">
+        <x:v>draft_attic_trunk_01</x:v>
+      </x:c>
+      <x:c r="B38" s="12" t="str">
+        <x:v>attic_trunk_01</x:v>
+      </x:c>
+      <x:c r="C38" s="12" t="str"/>
+      <x:c r="D38" s="12" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E38" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F38" s="12" t="str">
+        <x:v>false</x:v>
+      </x:c>
       <x:c r="G38" s="15" t="str">
         <x:f>IF(B38="","",IFERROR(VLOOKUP(B38,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+        <x:v>attic</x:v>
       </x:c>
       <x:c r="H38" s="15" t="str">
         <x:f>IF(G38="","",IFERROR(VLOOKUP(G38,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Attic</x:v>
       </x:c>
       <x:c r="I38" s="15" t="str">
         <x:f>IF(B38="","",IFERROR(VLOOKUP(B38,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+        <x:v>Left open trunk</x:v>
       </x:c>
       <x:c r="J38" s="15" t="str">
         <x:f>IF(B38="","",IFERROR(VLOOKUP(B38,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K38" s="15" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K38" s="15" t="n">
         <x:f>IF(B38="","",IFERROR(VLOOKUP(B38,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="32" customHeight="1">
-      <x:c r="A39" s="12"/>
-      <x:c r="B39" s="12"/>
-      <x:c r="C39" s="12"/>
-      <x:c r="D39" s="12"/>
-      <x:c r="E39" s="13"/>
-      <x:c r="F39" s="12"/>
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="34" customHeight="1">
+      <x:c r="A39" s="12" t="str">
+        <x:v>draft_attic_trunk_02</x:v>
+      </x:c>
+      <x:c r="B39" s="12" t="str">
+        <x:v>attic_trunk_02</x:v>
+      </x:c>
+      <x:c r="C39" s="12" t="str"/>
+      <x:c r="D39" s="12" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E39" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F39" s="12" t="str">
+        <x:v>false</x:v>
+      </x:c>
       <x:c r="G39" s="15" t="str">
         <x:f>IF(B39="","",IFERROR(VLOOKUP(B39,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+        <x:v>attic</x:v>
       </x:c>
       <x:c r="H39" s="15" t="str">
         <x:f>IF(G39="","",IFERROR(VLOOKUP(G39,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Attic</x:v>
       </x:c>
       <x:c r="I39" s="15" t="str">
         <x:f>IF(B39="","",IFERROR(VLOOKUP(B39,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+        <x:v>Right open trunk</x:v>
       </x:c>
       <x:c r="J39" s="15" t="str">
         <x:f>IF(B39="","",IFERROR(VLOOKUP(B39,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K39" s="15" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K39" s="15" t="n">
         <x:f>IF(B39="","",IFERROR(VLOOKUP(B39,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="32" customHeight="1">
-      <x:c r="A40" s="12"/>
-      <x:c r="B40" s="12"/>
-      <x:c r="C40" s="12"/>
-      <x:c r="D40" s="12"/>
-      <x:c r="E40" s="13"/>
-      <x:c r="F40" s="12"/>
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="34" customHeight="1">
+      <x:c r="A40" s="12" t="str">
+        <x:v>draft_attic_shelves_01</x:v>
+      </x:c>
+      <x:c r="B40" s="12" t="str">
+        <x:v>attic_shelves_01</x:v>
+      </x:c>
+      <x:c r="C40" s="12" t="str"/>
+      <x:c r="D40" s="12" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E40" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F40" s="12" t="str">
+        <x:v>false</x:v>
+      </x:c>
       <x:c r="G40" s="15" t="str">
         <x:f>IF(B40="","",IFERROR(VLOOKUP(B40,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+        <x:v>attic</x:v>
       </x:c>
       <x:c r="H40" s="15" t="str">
         <x:f>IF(G40="","",IFERROR(VLOOKUP(G40,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Attic</x:v>
       </x:c>
       <x:c r="I40" s="15" t="str">
         <x:f>IF(B40="","",IFERROR(VLOOKUP(B40,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+        <x:v>Shelving</x:v>
       </x:c>
       <x:c r="J40" s="15" t="str">
         <x:f>IF(B40="","",IFERROR(VLOOKUP(B40,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K40" s="15" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K40" s="15" t="n">
         <x:f>IF(B40="","",IFERROR(VLOOKUP(B40,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="41" ht="32" customHeight="1">
-      <x:c r="A41" s="12"/>
-      <x:c r="B41" s="12"/>
-      <x:c r="C41" s="12"/>
-      <x:c r="D41" s="12"/>
-      <x:c r="E41" s="13"/>
-      <x:c r="F41" s="12"/>
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="34" customHeight="1">
+      <x:c r="A41" s="12" t="str">
+        <x:v>draft_attic_table_01</x:v>
+      </x:c>
+      <x:c r="B41" s="12" t="str">
+        <x:v>attic_table_01</x:v>
+      </x:c>
+      <x:c r="C41" s="12" t="str"/>
+      <x:c r="D41" s="12" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E41" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F41" s="12" t="str">
+        <x:v>false</x:v>
+      </x:c>
       <x:c r="G41" s="15" t="str">
         <x:f>IF(B41="","",IFERROR(VLOOKUP(B41,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+        <x:v>attic</x:v>
       </x:c>
       <x:c r="H41" s="15" t="str">
         <x:f>IF(G41="","",IFERROR(VLOOKUP(G41,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Attic</x:v>
       </x:c>
       <x:c r="I41" s="15" t="str">
         <x:f>IF(B41="","",IFERROR(VLOOKUP(B41,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+        <x:v>Research table</x:v>
       </x:c>
       <x:c r="J41" s="15" t="str">
         <x:f>IF(B41="","",IFERROR(VLOOKUP(B41,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K41" s="15" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K41" s="15" t="n">
         <x:f>IF(B41="","",IFERROR(VLOOKUP(B41,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="42" ht="32" customHeight="1">
-      <x:c r="A42" s="12"/>
-      <x:c r="B42" s="12"/>
-      <x:c r="C42" s="12"/>
-      <x:c r="D42" s="12"/>
-      <x:c r="E42" s="13"/>
-      <x:c r="F42" s="12"/>
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="34" customHeight="1">
+      <x:c r="A42" s="12" t="str">
+        <x:v>draft_conservators_office_shelves_01</x:v>
+      </x:c>
+      <x:c r="B42" s="12" t="str">
+        <x:v>conservators_office_shelves_01</x:v>
+      </x:c>
+      <x:c r="C42" s="12" t="str"/>
+      <x:c r="D42" s="12" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E42" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F42" s="12" t="str">
+        <x:v>false</x:v>
+      </x:c>
       <x:c r="G42" s="15" t="str">
         <x:f>IF(B42="","",IFERROR(VLOOKUP(B42,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+        <x:v>conservators_office</x:v>
       </x:c>
       <x:c r="H42" s="15" t="str">
         <x:f>IF(G42="","",IFERROR(VLOOKUP(G42,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Conservator's Office</x:v>
       </x:c>
       <x:c r="I42" s="15" t="str">
         <x:f>IF(B42="","",IFERROR(VLOOKUP(B42,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+        <x:v>Left shelving</x:v>
       </x:c>
       <x:c r="J42" s="15" t="str">
         <x:f>IF(B42="","",IFERROR(VLOOKUP(B42,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K42" s="15" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K42" s="15" t="n">
         <x:f>IF(B42="","",IFERROR(VLOOKUP(B42,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="43" ht="32" customHeight="1">
-      <x:c r="A43" s="12"/>
-      <x:c r="B43" s="12"/>
-      <x:c r="C43" s="12"/>
-      <x:c r="D43" s="12"/>
-      <x:c r="E43" s="13"/>
-      <x:c r="F43" s="12"/>
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="34" customHeight="1">
+      <x:c r="A43" s="12" t="str">
+        <x:v>draft_conservators_office_shelves_02</x:v>
+      </x:c>
+      <x:c r="B43" s="12" t="str">
+        <x:v>conservators_office_shelves_02</x:v>
+      </x:c>
+      <x:c r="C43" s="12" t="str"/>
+      <x:c r="D43" s="12" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E43" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F43" s="12" t="str">
+        <x:v>false</x:v>
+      </x:c>
       <x:c r="G43" s="15" t="str">
         <x:f>IF(B43="","",IFERROR(VLOOKUP(B43,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+        <x:v>conservators_office</x:v>
       </x:c>
       <x:c r="H43" s="15" t="str">
         <x:f>IF(G43="","",IFERROR(VLOOKUP(G43,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Conservator's Office</x:v>
       </x:c>
       <x:c r="I43" s="15" t="str">
         <x:f>IF(B43="","",IFERROR(VLOOKUP(B43,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+        <x:v>Rear shelving</x:v>
       </x:c>
       <x:c r="J43" s="15" t="str">
         <x:f>IF(B43="","",IFERROR(VLOOKUP(B43,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K43" s="15" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K43" s="15" t="n">
         <x:f>IF(B43="","",IFERROR(VLOOKUP(B43,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="44" ht="32" customHeight="1">
-      <x:c r="A44" s="12"/>
-      <x:c r="B44" s="12"/>
-      <x:c r="C44" s="12"/>
-      <x:c r="D44" s="12"/>
-      <x:c r="E44" s="13"/>
-      <x:c r="F44" s="12"/>
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="34" customHeight="1">
+      <x:c r="A44" s="12" t="str">
+        <x:v>draft_conservators_office_shelves_03</x:v>
+      </x:c>
+      <x:c r="B44" s="12" t="str">
+        <x:v>conservators_office_shelves_03</x:v>
+      </x:c>
+      <x:c r="C44" s="12" t="str"/>
+      <x:c r="D44" s="12" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E44" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F44" s="12" t="str">
+        <x:v>false</x:v>
+      </x:c>
       <x:c r="G44" s="15" t="str">
         <x:f>IF(B44="","",IFERROR(VLOOKUP(B44,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+        <x:v>conservators_office</x:v>
       </x:c>
       <x:c r="H44" s="15" t="str">
         <x:f>IF(G44="","",IFERROR(VLOOKUP(G44,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Conservator's Office</x:v>
       </x:c>
       <x:c r="I44" s="15" t="str">
         <x:f>IF(B44="","",IFERROR(VLOOKUP(B44,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+        <x:v>Right shelving</x:v>
       </x:c>
       <x:c r="J44" s="15" t="str">
         <x:f>IF(B44="","",IFERROR(VLOOKUP(B44,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K44" s="15" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K44" s="15" t="n">
         <x:f>IF(B44="","",IFERROR(VLOOKUP(B44,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="34" customHeight="1">
+      <x:c r="A45" s="12" t="str">
+        <x:v>draft_lab_bench_01</x:v>
+      </x:c>
+      <x:c r="B45" s="12" t="str">
+        <x:v>lab_bench_01</x:v>
+      </x:c>
+      <x:c r="C45" s="12" t="str"/>
+      <x:c r="D45" s="12" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E45" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F45" s="12" t="str">
+        <x:v>false</x:v>
+      </x:c>
+      <x:c r="G45" s="15" t="str">
+        <x:f>IF(B45="","",IFERROR(VLOOKUP(B45,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+        <x:v>lab</x:v>
+      </x:c>
+      <x:c r="H45" s="15" t="str">
+        <x:f>IF(G45="","",IFERROR(VLOOKUP(G45,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Lab</x:v>
+      </x:c>
+      <x:c r="I45" s="15" t="str">
+        <x:f>IF(B45="","",IFERROR(VLOOKUP(B45,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+        <x:v>Analysis bench</x:v>
+      </x:c>
+      <x:c r="J45" s="15" t="str">
+        <x:f>IF(B45="","",IFERROR(VLOOKUP(B45,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K45" s="15" t="n">
+        <x:f>IF(B45="","",IFERROR(VLOOKUP(B45,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="34" customHeight="1">
+      <x:c r="A46" s="12" t="str">
+        <x:v>draft_lab_equipment_01</x:v>
+      </x:c>
+      <x:c r="B46" s="12" t="str">
+        <x:v>lab_equipment_01</x:v>
+      </x:c>
+      <x:c r="C46" s="12" t="str"/>
+      <x:c r="D46" s="12" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E46" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F46" s="12" t="str">
+        <x:v>false</x:v>
+      </x:c>
+      <x:c r="G46" s="15" t="str">
+        <x:f>IF(B46="","",IFERROR(VLOOKUP(B46,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+        <x:v>lab</x:v>
+      </x:c>
+      <x:c r="H46" s="15" t="str">
+        <x:f>IF(G46="","",IFERROR(VLOOKUP(G46,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Lab</x:v>
+      </x:c>
+      <x:c r="I46" s="15" t="str">
+        <x:f>IF(B46="","",IFERROR(VLOOKUP(B46,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="J46" s="15" t="str">
+        <x:f>IF(B46="","",IFERROR(VLOOKUP(B46,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K46" s="15" t="n">
+        <x:f>IF(B46="","",IFERROR(VLOOKUP(B46,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="34" customHeight="1">
+      <x:c r="A47" s="12" t="str">
+        <x:v>draft_lab_cabinet_01</x:v>
+      </x:c>
+      <x:c r="B47" s="12" t="str">
+        <x:v>lab_cabinet_01</x:v>
+      </x:c>
+      <x:c r="C47" s="12" t="str"/>
+      <x:c r="D47" s="12" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E47" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F47" s="12" t="str">
+        <x:v>false</x:v>
+      </x:c>
+      <x:c r="G47" s="15" t="str">
+        <x:f>IF(B47="","",IFERROR(VLOOKUP(B47,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+        <x:v>lab</x:v>
+      </x:c>
+      <x:c r="H47" s="15" t="str">
+        <x:f>IF(G47="","",IFERROR(VLOOKUP(G47,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Lab</x:v>
+      </x:c>
+      <x:c r="I47" s="15" t="str">
+        <x:f>IF(B47="","",IFERROR(VLOOKUP(B47,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+        <x:v>Left cabinet</x:v>
+      </x:c>
+      <x:c r="J47" s="15" t="str">
+        <x:f>IF(B47="","",IFERROR(VLOOKUP(B47,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K47" s="15" t="n">
+        <x:f>IF(B47="","",IFERROR(VLOOKUP(B47,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="34" customHeight="1">
+      <x:c r="A48" s="12" t="str">
+        <x:v>draft_lab_cabinet_02</x:v>
+      </x:c>
+      <x:c r="B48" s="12" t="str">
+        <x:v>lab_cabinet_02</x:v>
+      </x:c>
+      <x:c r="C48" s="12" t="str"/>
+      <x:c r="D48" s="12" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E48" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F48" s="12" t="str">
+        <x:v>false</x:v>
+      </x:c>
+      <x:c r="G48" s="15" t="str">
+        <x:f>IF(B48="","",IFERROR(VLOOKUP(B48,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+        <x:v>lab</x:v>
+      </x:c>
+      <x:c r="H48" s="15" t="str">
+        <x:f>IF(G48="","",IFERROR(VLOOKUP(G48,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Lab</x:v>
+      </x:c>
+      <x:c r="I48" s="15" t="str">
+        <x:f>IF(B48="","",IFERROR(VLOOKUP(B48,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+        <x:v>Right cabinet</x:v>
+      </x:c>
+      <x:c r="J48" s="15" t="str">
+        <x:f>IF(B48="","",IFERROR(VLOOKUP(B48,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K48" s="15" t="n">
+        <x:f>IF(B48="","",IFERROR(VLOOKUP(B48,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="32" customHeight="1">
+      <x:c r="A49" s="12"/>
+      <x:c r="B49" s="12"/>
+      <x:c r="C49" s="12"/>
+      <x:c r="D49" s="12"/>
+      <x:c r="E49" s="13"/>
+      <x:c r="F49" s="12"/>
+      <x:c r="G49" s="15" t="str">
+        <x:f>IF(B49="","",IFERROR(VLOOKUP(B49,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="H49" s="15" t="str">
+        <x:f>IF(G49="","",IFERROR(VLOOKUP(G49,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I49" s="15" t="str">
+        <x:f>IF(B49="","",IFERROR(VLOOKUP(B49,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="J49" s="15" t="str">
+        <x:f>IF(B49="","",IFERROR(VLOOKUP(B49,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K49" s="15" t="str">
+        <x:f>IF(B49="","",IFERROR(VLOOKUP(B49,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="32" customHeight="1">
+      <x:c r="A50" s="12"/>
+      <x:c r="B50" s="12"/>
+      <x:c r="C50" s="12"/>
+      <x:c r="D50" s="12"/>
+      <x:c r="E50" s="13"/>
+      <x:c r="F50" s="12"/>
+      <x:c r="G50" s="15" t="str">
+        <x:f>IF(B50="","",IFERROR(VLOOKUP(B50,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="H50" s="15" t="str">
+        <x:f>IF(G50="","",IFERROR(VLOOKUP(G50,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I50" s="15" t="str">
+        <x:f>IF(B50="","",IFERROR(VLOOKUP(B50,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="J50" s="15" t="str">
+        <x:f>IF(B50="","",IFERROR(VLOOKUP(B50,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K50" s="15" t="str">
+        <x:f>IF(B50="","",IFERROR(VLOOKUP(B50,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="32" customHeight="1">
+      <x:c r="A51" s="12"/>
+      <x:c r="B51" s="12"/>
+      <x:c r="C51" s="12"/>
+      <x:c r="D51" s="12"/>
+      <x:c r="E51" s="13"/>
+      <x:c r="F51" s="12"/>
+      <x:c r="G51" s="15" t="str">
+        <x:f>IF(B51="","",IFERROR(VLOOKUP(B51,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="H51" s="15" t="str">
+        <x:f>IF(G51="","",IFERROR(VLOOKUP(G51,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I51" s="15" t="str">
+        <x:f>IF(B51="","",IFERROR(VLOOKUP(B51,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="J51" s="15" t="str">
+        <x:f>IF(B51="","",IFERROR(VLOOKUP(B51,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K51" s="15" t="str">
+        <x:f>IF(B51="","",IFERROR(VLOOKUP(B51,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="32" customHeight="1">
+      <x:c r="A52" s="12"/>
+      <x:c r="B52" s="12"/>
+      <x:c r="C52" s="12"/>
+      <x:c r="D52" s="12"/>
+      <x:c r="E52" s="13"/>
+      <x:c r="F52" s="12"/>
+      <x:c r="G52" s="15" t="str">
+        <x:f>IF(B52="","",IFERROR(VLOOKUP(B52,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="H52" s="15" t="str">
+        <x:f>IF(G52="","",IFERROR(VLOOKUP(G52,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I52" s="15" t="str">
+        <x:f>IF(B52="","",IFERROR(VLOOKUP(B52,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="J52" s="15" t="str">
+        <x:f>IF(B52="","",IFERROR(VLOOKUP(B52,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K52" s="15" t="str">
+        <x:f>IF(B52="","",IFERROR(VLOOKUP(B52,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="32" customHeight="1">
+      <x:c r="A53" s="12"/>
+      <x:c r="B53" s="12"/>
+      <x:c r="C53" s="12"/>
+      <x:c r="D53" s="12"/>
+      <x:c r="E53" s="13"/>
+      <x:c r="F53" s="12"/>
+      <x:c r="G53" s="15" t="str">
+        <x:f>IF(B53="","",IFERROR(VLOOKUP(B53,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="H53" s="15" t="str">
+        <x:f>IF(G53="","",IFERROR(VLOOKUP(G53,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I53" s="15" t="str">
+        <x:f>IF(B53="","",IFERROR(VLOOKUP(B53,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="J53" s="15" t="str">
+        <x:f>IF(B53="","",IFERROR(VLOOKUP(B53,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K53" s="15" t="str">
+        <x:f>IF(B53="","",IFERROR(VLOOKUP(B53,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="32" customHeight="1">
+      <x:c r="A54" s="12"/>
+      <x:c r="B54" s="12"/>
+      <x:c r="C54" s="12"/>
+      <x:c r="D54" s="12"/>
+      <x:c r="E54" s="13"/>
+      <x:c r="F54" s="12"/>
+      <x:c r="G54" s="15" t="str">
+        <x:f>IF(B54="","",IFERROR(VLOOKUP(B54,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="H54" s="15" t="str">
+        <x:f>IF(G54="","",IFERROR(VLOOKUP(G54,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I54" s="15" t="str">
+        <x:f>IF(B54="","",IFERROR(VLOOKUP(B54,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="J54" s="15" t="str">
+        <x:f>IF(B54="","",IFERROR(VLOOKUP(B54,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K54" s="15" t="str">
+        <x:f>IF(B54="","",IFERROR(VLOOKUP(B54,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="32" customHeight="1">
+      <x:c r="A55" s="12"/>
+      <x:c r="B55" s="12"/>
+      <x:c r="C55" s="12"/>
+      <x:c r="D55" s="12"/>
+      <x:c r="E55" s="13"/>
+      <x:c r="F55" s="12"/>
+      <x:c r="G55" s="15" t="str">
+        <x:f>IF(B55="","",IFERROR(VLOOKUP(B55,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="H55" s="15" t="str">
+        <x:f>IF(G55="","",IFERROR(VLOOKUP(G55,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I55" s="15" t="str">
+        <x:f>IF(B55="","",IFERROR(VLOOKUP(B55,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="J55" s="15" t="str">
+        <x:f>IF(B55="","",IFERROR(VLOOKUP(B55,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K55" s="15" t="str">
+        <x:f>IF(B55="","",IFERROR(VLOOKUP(B55,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="32" customHeight="1">
+      <x:c r="A56" s="12"/>
+      <x:c r="B56" s="12"/>
+      <x:c r="C56" s="12"/>
+      <x:c r="D56" s="12"/>
+      <x:c r="E56" s="13"/>
+      <x:c r="F56" s="12"/>
+      <x:c r="G56" s="15" t="str">
+        <x:f>IF(B56="","",IFERROR(VLOOKUP(B56,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="H56" s="15" t="str">
+        <x:f>IF(G56="","",IFERROR(VLOOKUP(G56,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I56" s="15" t="str">
+        <x:f>IF(B56="","",IFERROR(VLOOKUP(B56,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="J56" s="15" t="str">
+        <x:f>IF(B56="","",IFERROR(VLOOKUP(B56,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K56" s="15" t="str">
+        <x:f>IF(B56="","",IFERROR(VLOOKUP(B56,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="32" customHeight="1">
+      <x:c r="A57" s="12"/>
+      <x:c r="B57" s="12"/>
+      <x:c r="C57" s="12"/>
+      <x:c r="D57" s="12"/>
+      <x:c r="E57" s="13"/>
+      <x:c r="F57" s="12"/>
+      <x:c r="G57" s="15" t="str">
+        <x:f>IF(B57="","",IFERROR(VLOOKUP(B57,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="H57" s="15" t="str">
+        <x:f>IF(G57="","",IFERROR(VLOOKUP(G57,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I57" s="15" t="str">
+        <x:f>IF(B57="","",IFERROR(VLOOKUP(B57,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="J57" s="15" t="str">
+        <x:f>IF(B57="","",IFERROR(VLOOKUP(B57,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K57" s="15" t="str">
+        <x:f>IF(B57="","",IFERROR(VLOOKUP(B57,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="32" customHeight="1">
+      <x:c r="A58" s="12"/>
+      <x:c r="B58" s="12"/>
+      <x:c r="C58" s="12"/>
+      <x:c r="D58" s="12"/>
+      <x:c r="E58" s="13"/>
+      <x:c r="F58" s="12"/>
+      <x:c r="G58" s="15" t="str">
+        <x:f>IF(B58="","",IFERROR(VLOOKUP(B58,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="H58" s="15" t="str">
+        <x:f>IF(G58="","",IFERROR(VLOOKUP(G58,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I58" s="15" t="str">
+        <x:f>IF(B58="","",IFERROR(VLOOKUP(B58,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="J58" s="15" t="str">
+        <x:f>IF(B58="","",IFERROR(VLOOKUP(B58,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K58" s="15" t="str">
+        <x:f>IF(B58="","",IFERROR(VLOOKUP(B58,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="32" customHeight="1">
+      <x:c r="A59" s="12"/>
+      <x:c r="B59" s="12"/>
+      <x:c r="C59" s="12"/>
+      <x:c r="D59" s="12"/>
+      <x:c r="E59" s="13"/>
+      <x:c r="F59" s="12"/>
+      <x:c r="G59" s="15" t="str">
+        <x:f>IF(B59="","",IFERROR(VLOOKUP(B59,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="H59" s="15" t="str">
+        <x:f>IF(G59="","",IFERROR(VLOOKUP(G59,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I59" s="15" t="str">
+        <x:f>IF(B59="","",IFERROR(VLOOKUP(B59,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="J59" s="15" t="str">
+        <x:f>IF(B59="","",IFERROR(VLOOKUP(B59,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K59" s="15" t="str">
+        <x:f>IF(B59="","",IFERROR(VLOOKUP(B59,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="32" customHeight="1">
+      <x:c r="A60" s="12"/>
+      <x:c r="B60" s="12"/>
+      <x:c r="C60" s="12"/>
+      <x:c r="D60" s="12"/>
+      <x:c r="E60" s="13"/>
+      <x:c r="F60" s="12"/>
+      <x:c r="G60" s="15" t="str">
+        <x:f>IF(B60="","",IFERROR(VLOOKUP(B60,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="H60" s="15" t="str">
+        <x:f>IF(G60="","",IFERROR(VLOOKUP(G60,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I60" s="15" t="str">
+        <x:f>IF(B60="","",IFERROR(VLOOKUP(B60,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="J60" s="15" t="str">
+        <x:f>IF(B60="","",IFERROR(VLOOKUP(B60,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K60" s="15" t="str">
+        <x:f>IF(B60="","",IFERROR(VLOOKUP(B60,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="32" customHeight="1">
+      <x:c r="A61" s="12"/>
+      <x:c r="B61" s="12"/>
+      <x:c r="C61" s="12"/>
+      <x:c r="D61" s="12"/>
+      <x:c r="E61" s="13"/>
+      <x:c r="F61" s="12"/>
+      <x:c r="G61" s="15" t="str">
+        <x:f>IF(B61="","",IFERROR(VLOOKUP(B61,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="H61" s="15" t="str">
+        <x:f>IF(G61="","",IFERROR(VLOOKUP(G61,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I61" s="15" t="str">
+        <x:f>IF(B61="","",IFERROR(VLOOKUP(B61,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="J61" s="15" t="str">
+        <x:f>IF(B61="","",IFERROR(VLOOKUP(B61,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K61" s="15" t="str">
+        <x:f>IF(B61="","",IFERROR(VLOOKUP(B61,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="32" customHeight="1">
+      <x:c r="A62" s="12"/>
+      <x:c r="B62" s="12"/>
+      <x:c r="C62" s="12"/>
+      <x:c r="D62" s="12"/>
+      <x:c r="E62" s="13"/>
+      <x:c r="F62" s="12"/>
+      <x:c r="G62" s="15" t="str">
+        <x:f>IF(B62="","",IFERROR(VLOOKUP(B62,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="H62" s="15" t="str">
+        <x:f>IF(G62="","",IFERROR(VLOOKUP(G62,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I62" s="15" t="str">
+        <x:f>IF(B62="","",IFERROR(VLOOKUP(B62,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="J62" s="15" t="str">
+        <x:f>IF(B62="","",IFERROR(VLOOKUP(B62,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K62" s="15" t="str">
+        <x:f>IF(B62="","",IFERROR(VLOOKUP(B62,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="32" customHeight="1">
+      <x:c r="A63" s="12"/>
+      <x:c r="B63" s="12"/>
+      <x:c r="C63" s="12"/>
+      <x:c r="D63" s="12"/>
+      <x:c r="E63" s="13"/>
+      <x:c r="F63" s="12"/>
+      <x:c r="G63" s="15" t="str">
+        <x:f>IF(B63="","",IFERROR(VLOOKUP(B63,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="H63" s="15" t="str">
+        <x:f>IF(G63="","",IFERROR(VLOOKUP(G63,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I63" s="15" t="str">
+        <x:f>IF(B63="","",IFERROR(VLOOKUP(B63,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="J63" s="15" t="str">
+        <x:f>IF(B63="","",IFERROR(VLOOKUP(B63,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K63" s="15" t="str">
+        <x:f>IF(B63="","",IFERROR(VLOOKUP(B63,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="C2:C44">
+  <x:conditionalFormatting sqref="C2:C63">
     <x:cfRule type="expression" dxfId="0" priority="1">
       <x:formula>AND($A2&lt;&gt;"",$C2="")</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="B2:B44">
+  <x:conditionalFormatting sqref="B2:B63">
     <x:cfRule type="expression" dxfId="1" priority="2">
       <x:formula>AND($A2&lt;&gt;"",$B2&lt;&gt;"",COUNTIF(Slots!$A$2:$A$501,$B2)=0)</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="F2:F44">
+  <x:conditionalFormatting sqref="F2:F63">
     <x:cfRule type="expression" dxfId="2" priority="3">
       <x:formula>AND($A2&lt;&gt;"",$F2="true",COUNTIFS($B$2:$B$501,$B2,$E$2:$E$501,$E2,$F$2:$F$501,"true")&gt;1)</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="E2:E44">
+  <x:conditionalFormatting sqref="E2:E63">
     <x:cfRule type="expression" dxfId="3" priority="4">
       <x:formula>AND($A2&lt;&gt;"",$F2="true",$E2&lt;&gt;"",COUNTIFS($B$2:$B$501,$B2,$E$2:$E$501,$E2,$F$2:$F$501,"true")&gt;1)</x:formula>
     </x:cfRule>
@@ -2070,7 +2792,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb8f9943b3944d57"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf05d92a80e6421e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2729,7 +3451,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6895ef182dd4d11"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62be95dcee1540c0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3383,7 +4105,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b3c8770a7f04d8d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0ffb5d20cfe4ab7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3623,7 +4345,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80e09748f4a44bdd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7eeedd787854ecf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3903,7 +4625,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra703ac2c40a1469b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e486a4ba3db490d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5453,7 +6175,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc331f24ec500493a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7c4edf946dd41d0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5993,7 +6715,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84ce73e7a8fd4c13"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb3a29f3290d42a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6190,7 +6912,7 @@
         <x:v>_data/placements.csv</x:v>
       </x:c>
       <x:c r="B23" s="24" t="str">
-        <x:v>a07011a65d6dec2fc9ed28b5e10d4aa2fc3b613a593d5296654ccbe7e062d813</x:v>
+        <x:v>fbca8d56f9e71f2c0692f7e800b0bc75ba10af0e9498432551789a039715cc6f</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="58" customHeight="1">
@@ -6238,7 +6960,7 @@
         <x:v>_data/demo-metadata.csv</x:v>
       </x:c>
       <x:c r="B29" s="24" t="str">
-        <x:v>7bd0bf689e14b3c0bf3dcaba7cc8f289f4be361750c6cda612fc8c45c8c5829b</x:v>
+        <x:v>2e46b740c50d02d3a29a3f0da94d21ad77f4c8a800d9106c3fc64b631c107af1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Polish ArchIvory room interactions for team demo
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/archivory-editorial/ArchIvory Editorial Workbook.xlsx
+++ b/outputs/archivory-editorial/ArchIvory Editorial Workbook.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Placements" sheetId="1" r:id="R62910e8b1e654193"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content" sheetId="2" r:id="R6d706709117c4efa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="3" r:id="R01e5051be94b407c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timelines" sheetId="4" r:id="R94869fca09e74b1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rooms" sheetId="5" r:id="Rd30042ed73c7471a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slots" sheetId="6" r:id="Rcefcced59951437a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection" sheetId="7" r:id="Rd196e7bcbe854e56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="R3e85da649fc9454b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Placements" sheetId="1" r:id="R1fccf5d178ae46f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content" sheetId="2" r:id="R422173620e7d4ad2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="3" r:id="R1cc35f938afe451a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timelines" sheetId="4" r:id="Rfa29d11885134574"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rooms" sheetId="5" r:id="R60f5f1cbece142c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slots" sheetId="6" r:id="Rd14f991a94ae4277"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection" sheetId="7" r:id="R22658ec397394493"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="Rae415e6155134866"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -196,7 +196,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PlacementsTable" displayName="PlacementsTable" ref="A1:K63" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PlacementsTable" displayName="PlacementsTable" ref="A1:K65" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="placement_id"/>
     <x:tableColumn id="2" name="slot_id"/>
@@ -274,7 +274,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="SlotsTable" displayName="SlotsTable" ref="A1:J61" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="SlotsTable" displayName="SlotsTable" ref="A1:J63" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="slot_id"/>
     <x:tableColumn id="2" name="room_id"/>
@@ -1376,10 +1376,10 @@
         <x:v>natural_history_timeline_01</x:v>
       </x:c>
       <x:c r="C22" s="12" t="str">
-        <x:v>proboscidean-timeline</x:v>
+        <x:v>deep_time_evidence</x:v>
       </x:c>
       <x:c r="D22" s="12" t="str">
-        <x:v>tool</x:v>
+        <x:v>timeline</x:v>
       </x:c>
       <x:c r="E22" s="13" t="n">
         <x:v>1</x:v>
@@ -1397,11 +1397,11 @@
       </x:c>
       <x:c r="I22" s="15" t="str">
         <x:f>IF(B22="","",IFERROR(VLOOKUP(B22,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Deep-time explorer</x:v>
+        <x:v>Ivory Through Time poster</x:v>
       </x:c>
       <x:c r="J22" s="15" t="str">
         <x:f>IF(B22="","",IFERROR(VLOOKUP(B22,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>tool</x:v>
+        <x:v>timeline</x:v>
       </x:c>
       <x:c r="K22" s="15" t="n">
         <x:f>IF(B22="","",IFERROR(VLOOKUP(B22,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
@@ -1450,16 +1450,16 @@
     </x:row>
     <x:row r="24" ht="34" customHeight="1">
       <x:c r="A24" s="12" t="str">
-        <x:v>natural_history_timeline_02_1</x:v>
+        <x:v>natural_history_inquiry_01_1</x:v>
       </x:c>
       <x:c r="B24" s="12" t="str">
-        <x:v>natural_history_timeline_02</x:v>
+        <x:v>natural_history_inquiry_01</x:v>
       </x:c>
       <x:c r="C24" s="12" t="str">
-        <x:v>deep_time_evidence</x:v>
+        <x:v>natural-history-tusk</x:v>
       </x:c>
       <x:c r="D24" s="12" t="str">
-        <x:v>timeline</x:v>
+        <x:v>tool</x:v>
       </x:c>
       <x:c r="E24" s="13" t="n">
         <x:v>1</x:v>
@@ -1477,11 +1477,11 @@
       </x:c>
       <x:c r="I24" s="15" t="str">
         <x:f>IF(B24="","",IFERROR(VLOOKUP(B24,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Arrange the evidence</x:v>
+        <x:v>Ivory inquiry</x:v>
       </x:c>
       <x:c r="J24" s="15" t="str">
         <x:f>IF(B24="","",IFERROR(VLOOKUP(B24,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>timeline</x:v>
+        <x:v>tool</x:v>
       </x:c>
       <x:c r="K24" s="15" t="n">
         <x:f>IF(B24="","",IFERROR(VLOOKUP(B24,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
@@ -1490,13 +1490,13 @@
     </x:row>
     <x:row r="25" ht="34" customHeight="1">
       <x:c r="A25" s="12" t="str">
-        <x:v>natural_history_inquiry_01_1</x:v>
+        <x:v>conservators_office_terminal_01_1</x:v>
       </x:c>
       <x:c r="B25" s="12" t="str">
-        <x:v>natural_history_inquiry_01</x:v>
+        <x:v>conservators_office_terminal_01</x:v>
       </x:c>
       <x:c r="C25" s="12" t="str">
-        <x:v>natural-history-tusk</x:v>
+        <x:v>conservator-terminal</x:v>
       </x:c>
       <x:c r="D25" s="12" t="str">
         <x:v>tool</x:v>
@@ -1509,15 +1509,15 @@
       </x:c>
       <x:c r="G25" s="15" t="str">
         <x:f>IF(B25="","",IFERROR(VLOOKUP(B25,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>natural_history</x:v>
+        <x:v>conservators_office</x:v>
       </x:c>
       <x:c r="H25" s="15" t="str">
         <x:f>IF(G25="","",IFERROR(VLOOKUP(G25,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Natural History Museum</x:v>
+        <x:v>Conservator's Office</x:v>
       </x:c>
       <x:c r="I25" s="15" t="str">
         <x:f>IF(B25="","",IFERROR(VLOOKUP(B25,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Ivory inquiry</x:v>
+        <x:v>Desk terminal</x:v>
       </x:c>
       <x:c r="J25" s="15" t="str">
         <x:f>IF(B25="","",IFERROR(VLOOKUP(B25,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
@@ -1530,16 +1530,16 @@
     </x:row>
     <x:row r="26" ht="34" customHeight="1">
       <x:c r="A26" s="12" t="str">
-        <x:v>conservators_office_terminal_01_1</x:v>
+        <x:v>conservators_office_panel_01_1</x:v>
       </x:c>
       <x:c r="B26" s="12" t="str">
-        <x:v>conservators_office_terminal_01</x:v>
+        <x:v>conservators_office_panel_01</x:v>
       </x:c>
       <x:c r="C26" s="12" t="str">
-        <x:v>conservator-terminal</x:v>
+        <x:v>conservators_office_intro</x:v>
       </x:c>
       <x:c r="D26" s="12" t="str">
-        <x:v>tool</x:v>
+        <x:v>detail</x:v>
       </x:c>
       <x:c r="E26" s="13" t="n">
         <x:v>1</x:v>
@@ -1557,11 +1557,11 @@
       </x:c>
       <x:c r="I26" s="15" t="str">
         <x:f>IF(B26="","",IFERROR(VLOOKUP(B26,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Desk terminal</x:v>
+        <x:v>Elephant wall panel</x:v>
       </x:c>
       <x:c r="J26" s="15" t="str">
         <x:f>IF(B26="","",IFERROR(VLOOKUP(B26,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>tool</x:v>
+        <x:v>detail</x:v>
       </x:c>
       <x:c r="K26" s="15" t="n">
         <x:f>IF(B26="","",IFERROR(VLOOKUP(B26,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
@@ -1570,16 +1570,16 @@
     </x:row>
     <x:row r="27" ht="34" customHeight="1">
       <x:c r="A27" s="12" t="str">
-        <x:v>conservators_office_panel_01_1</x:v>
+        <x:v>lab_attic_context_01_1</x:v>
       </x:c>
       <x:c r="B27" s="12" t="str">
-        <x:v>conservators_office_panel_01</x:v>
+        <x:v>lab_attic_context_01</x:v>
       </x:c>
       <x:c r="C27" s="12" t="str">
-        <x:v>conservators_office_intro</x:v>
+        <x:v>lab-attic-sequence</x:v>
       </x:c>
       <x:c r="D27" s="12" t="str">
-        <x:v>detail</x:v>
+        <x:v>tool</x:v>
       </x:c>
       <x:c r="E27" s="13" t="n">
         <x:v>1</x:v>
@@ -1589,19 +1589,19 @@
       </x:c>
       <x:c r="G27" s="15" t="str">
         <x:f>IF(B27="","",IFERROR(VLOOKUP(B27,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>conservators_office</x:v>
+        <x:v>lab</x:v>
       </x:c>
       <x:c r="H27" s="15" t="str">
         <x:f>IF(G27="","",IFERROR(VLOOKUP(G27,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Conservator's Office</x:v>
+        <x:v>Lab</x:v>
       </x:c>
       <x:c r="I27" s="15" t="str">
         <x:f>IF(B27="","",IFERROR(VLOOKUP(B27,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Elephant wall panel</x:v>
+        <x:v>Attic access context</x:v>
       </x:c>
       <x:c r="J27" s="15" t="str">
         <x:f>IF(B27="","",IFERROR(VLOOKUP(B27,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>detail</x:v>
+        <x:v>tool</x:v>
       </x:c>
       <x:c r="K27" s="15" t="n">
         <x:f>IF(B27="","",IFERROR(VLOOKUP(B27,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
@@ -1610,16 +1610,16 @@
     </x:row>
     <x:row r="28" ht="34" customHeight="1">
       <x:c r="A28" s="12" t="str">
-        <x:v>lab_attic_context_01_1</x:v>
+        <x:v>geib-flute</x:v>
       </x:c>
       <x:c r="B28" s="12" t="str">
-        <x:v>lab_attic_context_01</x:v>
+        <x:v>natural_history_panel_02</x:v>
       </x:c>
       <x:c r="C28" s="12" t="str">
-        <x:v>lab-attic-sequence</x:v>
+        <x:v>geib-flute</x:v>
       </x:c>
       <x:c r="D28" s="12" t="str">
-        <x:v>tool</x:v>
+        <x:v>detail</x:v>
       </x:c>
       <x:c r="E28" s="13" t="n">
         <x:v>1</x:v>
@@ -1629,35 +1629,33 @@
       </x:c>
       <x:c r="G28" s="15" t="str">
         <x:f>IF(B28="","",IFERROR(VLOOKUP(B28,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>lab</x:v>
+        <x:v>natural_history</x:v>
       </x:c>
       <x:c r="H28" s="15" t="str">
         <x:f>IF(G28="","",IFERROR(VLOOKUP(G28,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Lab</x:v>
+        <x:v>Natural History Museum</x:v>
       </x:c>
       <x:c r="I28" s="15" t="str">
         <x:f>IF(B28="","",IFERROR(VLOOKUP(B28,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Attic access context</x:v>
+        <x:v>Central recessed panel</x:v>
       </x:c>
       <x:c r="J28" s="15" t="str">
         <x:f>IF(B28="","",IFERROR(VLOOKUP(B28,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>tool</x:v>
+        <x:v>collection</x:v>
       </x:c>
       <x:c r="K28" s="15" t="n">
         <x:f>IF(B28="","",IFERROR(VLOOKUP(B28,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>1</x:v>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="34" customHeight="1">
       <x:c r="A29" s="12" t="str">
-        <x:v>geib-flute</x:v>
+        <x:v>draft_historical_society_intro</x:v>
       </x:c>
       <x:c r="B29" s="12" t="str">
-        <x:v>natural_history_panel_02</x:v>
-      </x:c>
-      <x:c r="C29" s="12" t="str">
-        <x:v>geib-flute</x:v>
-      </x:c>
+        <x:v>historical_society_intro</x:v>
+      </x:c>
+      <x:c r="C29" s="12" t="str"/>
       <x:c r="D29" s="12" t="str">
         <x:v>detail</x:v>
       </x:c>
@@ -1665,35 +1663,35 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F29" s="12" t="str">
-        <x:v>true</x:v>
+        <x:v>false</x:v>
       </x:c>
       <x:c r="G29" s="15" t="str">
         <x:f>IF(B29="","",IFERROR(VLOOKUP(B29,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>natural_history</x:v>
+        <x:v>historical_society</x:v>
       </x:c>
       <x:c r="H29" s="15" t="str">
         <x:f>IF(G29="","",IFERROR(VLOOKUP(G29,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Natural History Museum</x:v>
+        <x:v>Historical Society</x:v>
       </x:c>
       <x:c r="I29" s="15" t="str">
         <x:f>IF(B29="","",IFERROR(VLOOKUP(B29,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Central recessed panel</x:v>
+        <x:v>Historical Society introduction</x:v>
       </x:c>
       <x:c r="J29" s="15" t="str">
         <x:f>IF(B29="","",IFERROR(VLOOKUP(B29,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>collection</x:v>
+        <x:v>detail</x:v>
       </x:c>
       <x:c r="K29" s="15" t="n">
         <x:f>IF(B29="","",IFERROR(VLOOKUP(B29,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="34" customHeight="1">
       <x:c r="A30" s="12" t="str">
-        <x:v>draft_historical_society_intro</x:v>
+        <x:v>draft_attic_intro</x:v>
       </x:c>
       <x:c r="B30" s="12" t="str">
-        <x:v>historical_society_intro</x:v>
+        <x:v>attic_intro</x:v>
       </x:c>
       <x:c r="C30" s="12" t="str"/>
       <x:c r="D30" s="12" t="str">
@@ -1707,15 +1705,15 @@
       </x:c>
       <x:c r="G30" s="15" t="str">
         <x:f>IF(B30="","",IFERROR(VLOOKUP(B30,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>historical_society</x:v>
+        <x:v>attic</x:v>
       </x:c>
       <x:c r="H30" s="15" t="str">
         <x:f>IF(G30="","",IFERROR(VLOOKUP(G30,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Historical Society</x:v>
+        <x:v>Attic</x:v>
       </x:c>
       <x:c r="I30" s="15" t="str">
         <x:f>IF(B30="","",IFERROR(VLOOKUP(B30,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Historical Society introduction</x:v>
+        <x:v>Attic introduction</x:v>
       </x:c>
       <x:c r="J30" s="15" t="str">
         <x:f>IF(B30="","",IFERROR(VLOOKUP(B30,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
@@ -1728,10 +1726,10 @@
     </x:row>
     <x:row r="31" ht="34" customHeight="1">
       <x:c r="A31" s="12" t="str">
-        <x:v>draft_attic_intro</x:v>
+        <x:v>draft_natural_history_intro</x:v>
       </x:c>
       <x:c r="B31" s="12" t="str">
-        <x:v>attic_intro</x:v>
+        <x:v>natural_history_intro</x:v>
       </x:c>
       <x:c r="C31" s="12" t="str"/>
       <x:c r="D31" s="12" t="str">
@@ -1745,15 +1743,15 @@
       </x:c>
       <x:c r="G31" s="15" t="str">
         <x:f>IF(B31="","",IFERROR(VLOOKUP(B31,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>attic</x:v>
+        <x:v>natural_history</x:v>
       </x:c>
       <x:c r="H31" s="15" t="str">
         <x:f>IF(G31="","",IFERROR(VLOOKUP(G31,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Attic</x:v>
+        <x:v>Natural History Museum</x:v>
       </x:c>
       <x:c r="I31" s="15" t="str">
         <x:f>IF(B31="","",IFERROR(VLOOKUP(B31,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Attic introduction</x:v>
+        <x:v>Natural History Museum introduction</x:v>
       </x:c>
       <x:c r="J31" s="15" t="str">
         <x:f>IF(B31="","",IFERROR(VLOOKUP(B31,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
@@ -1766,10 +1764,10 @@
     </x:row>
     <x:row r="32" ht="34" customHeight="1">
       <x:c r="A32" s="12" t="str">
-        <x:v>draft_natural_history_intro</x:v>
+        <x:v>draft_conservators_office_intro</x:v>
       </x:c>
       <x:c r="B32" s="12" t="str">
-        <x:v>natural_history_intro</x:v>
+        <x:v>conservators_office_intro</x:v>
       </x:c>
       <x:c r="C32" s="12" t="str"/>
       <x:c r="D32" s="12" t="str">
@@ -1783,15 +1781,15 @@
       </x:c>
       <x:c r="G32" s="15" t="str">
         <x:f>IF(B32="","",IFERROR(VLOOKUP(B32,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>natural_history</x:v>
+        <x:v>conservators_office</x:v>
       </x:c>
       <x:c r="H32" s="15" t="str">
         <x:f>IF(G32="","",IFERROR(VLOOKUP(G32,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Natural History Museum</x:v>
+        <x:v>Conservator's Office</x:v>
       </x:c>
       <x:c r="I32" s="15" t="str">
         <x:f>IF(B32="","",IFERROR(VLOOKUP(B32,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Natural History Museum introduction</x:v>
+        <x:v>Conservator's Office introduction</x:v>
       </x:c>
       <x:c r="J32" s="15" t="str">
         <x:f>IF(B32="","",IFERROR(VLOOKUP(B32,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
@@ -1804,10 +1802,10 @@
     </x:row>
     <x:row r="33" ht="34" customHeight="1">
       <x:c r="A33" s="12" t="str">
-        <x:v>draft_conservators_office_intro</x:v>
+        <x:v>draft_lab_intro</x:v>
       </x:c>
       <x:c r="B33" s="12" t="str">
-        <x:v>conservators_office_intro</x:v>
+        <x:v>lab_intro</x:v>
       </x:c>
       <x:c r="C33" s="12" t="str"/>
       <x:c r="D33" s="12" t="str">
@@ -1821,15 +1819,15 @@
       </x:c>
       <x:c r="G33" s="15" t="str">
         <x:f>IF(B33="","",IFERROR(VLOOKUP(B33,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>conservators_office</x:v>
+        <x:v>lab</x:v>
       </x:c>
       <x:c r="H33" s="15" t="str">
         <x:f>IF(G33="","",IFERROR(VLOOKUP(G33,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Conservator's Office</x:v>
+        <x:v>Lab</x:v>
       </x:c>
       <x:c r="I33" s="15" t="str">
         <x:f>IF(B33="","",IFERROR(VLOOKUP(B33,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Conservator's Office introduction</x:v>
+        <x:v>Lab introduction</x:v>
       </x:c>
       <x:c r="J33" s="15" t="str">
         <x:f>IF(B33="","",IFERROR(VLOOKUP(B33,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
@@ -1842,10 +1840,10 @@
     </x:row>
     <x:row r="34" ht="34" customHeight="1">
       <x:c r="A34" s="12" t="str">
-        <x:v>draft_lab_intro</x:v>
+        <x:v>draft_gallery_case_02</x:v>
       </x:c>
       <x:c r="B34" s="12" t="str">
-        <x:v>lab_intro</x:v>
+        <x:v>gallery_case_02</x:v>
       </x:c>
       <x:c r="C34" s="12" t="str"/>
       <x:c r="D34" s="12" t="str">
@@ -1859,31 +1857,31 @@
       </x:c>
       <x:c r="G34" s="15" t="str">
         <x:f>IF(B34="","",IFERROR(VLOOKUP(B34,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>lab</x:v>
+        <x:v>gallery</x:v>
       </x:c>
       <x:c r="H34" s="15" t="str">
         <x:f>IF(G34="","",IFERROR(VLOOKUP(G34,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Lab</x:v>
+        <x:v>Gallery</x:v>
       </x:c>
       <x:c r="I34" s="15" t="str">
         <x:f>IF(B34="","",IFERROR(VLOOKUP(B34,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Lab introduction</x:v>
+        <x:v>Rear round display</x:v>
       </x:c>
       <x:c r="J34" s="15" t="str">
         <x:f>IF(B34="","",IFERROR(VLOOKUP(B34,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-        <x:v>detail</x:v>
+        <x:v>collection</x:v>
       </x:c>
       <x:c r="K34" s="15" t="n">
         <x:f>IF(B34="","",IFERROR(VLOOKUP(B34,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>1</x:v>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="34" customHeight="1">
       <x:c r="A35" s="12" t="str">
-        <x:v>draft_gallery_case_02</x:v>
+        <x:v>draft_historical_society_case_01</x:v>
       </x:c>
       <x:c r="B35" s="12" t="str">
-        <x:v>gallery_case_02</x:v>
+        <x:v>historical_society_case_01</x:v>
       </x:c>
       <x:c r="C35" s="12" t="str"/>
       <x:c r="D35" s="12" t="str">
@@ -1897,15 +1895,15 @@
       </x:c>
       <x:c r="G35" s="15" t="str">
         <x:f>IF(B35="","",IFERROR(VLOOKUP(B35,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>gallery</x:v>
+        <x:v>historical_society</x:v>
       </x:c>
       <x:c r="H35" s="15" t="str">
         <x:f>IF(G35="","",IFERROR(VLOOKUP(G35,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Gallery</x:v>
+        <x:v>Historical Society</x:v>
       </x:c>
       <x:c r="I35" s="15" t="str">
         <x:f>IF(B35="","",IFERROR(VLOOKUP(B35,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Rear round display</x:v>
+        <x:v>Window-side case</x:v>
       </x:c>
       <x:c r="J35" s="15" t="str">
         <x:f>IF(B35="","",IFERROR(VLOOKUP(B35,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
@@ -1918,10 +1916,10 @@
     </x:row>
     <x:row r="36" ht="34" customHeight="1">
       <x:c r="A36" s="12" t="str">
-        <x:v>draft_historical_society_case_01</x:v>
+        <x:v>draft_historical_society_case_02</x:v>
       </x:c>
       <x:c r="B36" s="12" t="str">
-        <x:v>historical_society_case_01</x:v>
+        <x:v>historical_society_case_02</x:v>
       </x:c>
       <x:c r="C36" s="12" t="str"/>
       <x:c r="D36" s="12" t="str">
@@ -1943,7 +1941,7 @@
       </x:c>
       <x:c r="I36" s="15" t="str">
         <x:f>IF(B36="","",IFERROR(VLOOKUP(B36,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Window-side case</x:v>
+        <x:v>Foreground-right case</x:v>
       </x:c>
       <x:c r="J36" s="15" t="str">
         <x:f>IF(B36="","",IFERROR(VLOOKUP(B36,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
@@ -1956,10 +1954,10 @@
     </x:row>
     <x:row r="37" ht="34" customHeight="1">
       <x:c r="A37" s="12" t="str">
-        <x:v>draft_historical_society_case_02</x:v>
+        <x:v>draft_attic_trunk_01</x:v>
       </x:c>
       <x:c r="B37" s="12" t="str">
-        <x:v>historical_society_case_02</x:v>
+        <x:v>attic_trunk_01</x:v>
       </x:c>
       <x:c r="C37" s="12" t="str"/>
       <x:c r="D37" s="12" t="str">
@@ -1973,15 +1971,15 @@
       </x:c>
       <x:c r="G37" s="15" t="str">
         <x:f>IF(B37="","",IFERROR(VLOOKUP(B37,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>historical_society</x:v>
+        <x:v>attic</x:v>
       </x:c>
       <x:c r="H37" s="15" t="str">
         <x:f>IF(G37="","",IFERROR(VLOOKUP(G37,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Historical Society</x:v>
+        <x:v>Attic</x:v>
       </x:c>
       <x:c r="I37" s="15" t="str">
         <x:f>IF(B37="","",IFERROR(VLOOKUP(B37,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Foreground-right case</x:v>
+        <x:v>Left open trunk</x:v>
       </x:c>
       <x:c r="J37" s="15" t="str">
         <x:f>IF(B37="","",IFERROR(VLOOKUP(B37,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
@@ -1994,10 +1992,10 @@
     </x:row>
     <x:row r="38" ht="34" customHeight="1">
       <x:c r="A38" s="12" t="str">
-        <x:v>draft_attic_trunk_01</x:v>
+        <x:v>draft_attic_trunk_02</x:v>
       </x:c>
       <x:c r="B38" s="12" t="str">
-        <x:v>attic_trunk_01</x:v>
+        <x:v>attic_trunk_02</x:v>
       </x:c>
       <x:c r="C38" s="12" t="str"/>
       <x:c r="D38" s="12" t="str">
@@ -2019,7 +2017,7 @@
       </x:c>
       <x:c r="I38" s="15" t="str">
         <x:f>IF(B38="","",IFERROR(VLOOKUP(B38,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Left open trunk</x:v>
+        <x:v>Right open trunk</x:v>
       </x:c>
       <x:c r="J38" s="15" t="str">
         <x:f>IF(B38="","",IFERROR(VLOOKUP(B38,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
@@ -2032,10 +2030,10 @@
     </x:row>
     <x:row r="39" ht="34" customHeight="1">
       <x:c r="A39" s="12" t="str">
-        <x:v>draft_attic_trunk_02</x:v>
+        <x:v>draft_attic_shelves_01</x:v>
       </x:c>
       <x:c r="B39" s="12" t="str">
-        <x:v>attic_trunk_02</x:v>
+        <x:v>attic_shelves_01</x:v>
       </x:c>
       <x:c r="C39" s="12" t="str"/>
       <x:c r="D39" s="12" t="str">
@@ -2057,7 +2055,7 @@
       </x:c>
       <x:c r="I39" s="15" t="str">
         <x:f>IF(B39="","",IFERROR(VLOOKUP(B39,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Right open trunk</x:v>
+        <x:v>Shelving</x:v>
       </x:c>
       <x:c r="J39" s="15" t="str">
         <x:f>IF(B39="","",IFERROR(VLOOKUP(B39,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
@@ -2070,10 +2068,10 @@
     </x:row>
     <x:row r="40" ht="34" customHeight="1">
       <x:c r="A40" s="12" t="str">
-        <x:v>draft_attic_shelves_01</x:v>
+        <x:v>draft_attic_table_01</x:v>
       </x:c>
       <x:c r="B40" s="12" t="str">
-        <x:v>attic_shelves_01</x:v>
+        <x:v>attic_table_01</x:v>
       </x:c>
       <x:c r="C40" s="12" t="str"/>
       <x:c r="D40" s="12" t="str">
@@ -2095,7 +2093,7 @@
       </x:c>
       <x:c r="I40" s="15" t="str">
         <x:f>IF(B40="","",IFERROR(VLOOKUP(B40,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Shelving</x:v>
+        <x:v>Research table</x:v>
       </x:c>
       <x:c r="J40" s="15" t="str">
         <x:f>IF(B40="","",IFERROR(VLOOKUP(B40,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
@@ -2108,10 +2106,10 @@
     </x:row>
     <x:row r="41" ht="34" customHeight="1">
       <x:c r="A41" s="12" t="str">
-        <x:v>draft_attic_table_01</x:v>
+        <x:v>draft_natural_history_timeline_02</x:v>
       </x:c>
       <x:c r="B41" s="12" t="str">
-        <x:v>attic_table_01</x:v>
+        <x:v>natural_history_timeline_02</x:v>
       </x:c>
       <x:c r="C41" s="12" t="str"/>
       <x:c r="D41" s="12" t="str">
@@ -2125,15 +2123,15 @@
       </x:c>
       <x:c r="G41" s="15" t="str">
         <x:f>IF(B41="","",IFERROR(VLOOKUP(B41,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>attic</x:v>
+        <x:v>natural_history</x:v>
       </x:c>
       <x:c r="H41" s="15" t="str">
         <x:f>IF(G41="","",IFERROR(VLOOKUP(G41,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Attic</x:v>
+        <x:v>Natural History Museum</x:v>
       </x:c>
       <x:c r="I41" s="15" t="str">
         <x:f>IF(B41="","",IFERROR(VLOOKUP(B41,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Research table</x:v>
+        <x:v>Background wall curator mount</x:v>
       </x:c>
       <x:c r="J41" s="15" t="str">
         <x:f>IF(B41="","",IFERROR(VLOOKUP(B41,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
@@ -2146,10 +2144,10 @@
     </x:row>
     <x:row r="42" ht="34" customHeight="1">
       <x:c r="A42" s="12" t="str">
-        <x:v>draft_conservators_office_shelves_01</x:v>
+        <x:v>draft_natural_history_table_01</x:v>
       </x:c>
       <x:c r="B42" s="12" t="str">
-        <x:v>conservators_office_shelves_01</x:v>
+        <x:v>natural_history_table_01</x:v>
       </x:c>
       <x:c r="C42" s="12" t="str"/>
       <x:c r="D42" s="12" t="str">
@@ -2163,15 +2161,15 @@
       </x:c>
       <x:c r="G42" s="15" t="str">
         <x:f>IF(B42="","",IFERROR(VLOOKUP(B42,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>conservators_office</x:v>
+        <x:v>natural_history</x:v>
       </x:c>
       <x:c r="H42" s="15" t="str">
         <x:f>IF(G42="","",IFERROR(VLOOKUP(G42,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Conservator's Office</x:v>
+        <x:v>Natural History Museum</x:v>
       </x:c>
       <x:c r="I42" s="15" t="str">
         <x:f>IF(B42="","",IFERROR(VLOOKUP(B42,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Left shelving</x:v>
+        <x:v>Foreground table left</x:v>
       </x:c>
       <x:c r="J42" s="15" t="str">
         <x:f>IF(B42="","",IFERROR(VLOOKUP(B42,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
@@ -2179,15 +2177,15 @@
       </x:c>
       <x:c r="K42" s="15" t="n">
         <x:f>IF(B42="","",IFERROR(VLOOKUP(B42,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="34" customHeight="1">
       <x:c r="A43" s="12" t="str">
-        <x:v>draft_conservators_office_shelves_02</x:v>
+        <x:v>draft_natural_history_table_02</x:v>
       </x:c>
       <x:c r="B43" s="12" t="str">
-        <x:v>conservators_office_shelves_02</x:v>
+        <x:v>natural_history_table_02</x:v>
       </x:c>
       <x:c r="C43" s="12" t="str"/>
       <x:c r="D43" s="12" t="str">
@@ -2201,15 +2199,15 @@
       </x:c>
       <x:c r="G43" s="15" t="str">
         <x:f>IF(B43="","",IFERROR(VLOOKUP(B43,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>conservators_office</x:v>
+        <x:v>natural_history</x:v>
       </x:c>
       <x:c r="H43" s="15" t="str">
         <x:f>IF(G43="","",IFERROR(VLOOKUP(G43,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Conservator's Office</x:v>
+        <x:v>Natural History Museum</x:v>
       </x:c>
       <x:c r="I43" s="15" t="str">
         <x:f>IF(B43="","",IFERROR(VLOOKUP(B43,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Rear shelving</x:v>
+        <x:v>Foreground table right</x:v>
       </x:c>
       <x:c r="J43" s="15" t="str">
         <x:f>IF(B43="","",IFERROR(VLOOKUP(B43,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
@@ -2217,15 +2215,15 @@
       </x:c>
       <x:c r="K43" s="15" t="n">
         <x:f>IF(B43="","",IFERROR(VLOOKUP(B43,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="34" customHeight="1">
       <x:c r="A44" s="12" t="str">
-        <x:v>draft_conservators_office_shelves_03</x:v>
+        <x:v>draft_conservators_office_shelves_01</x:v>
       </x:c>
       <x:c r="B44" s="12" t="str">
-        <x:v>conservators_office_shelves_03</x:v>
+        <x:v>conservators_office_shelves_01</x:v>
       </x:c>
       <x:c r="C44" s="12" t="str"/>
       <x:c r="D44" s="12" t="str">
@@ -2247,7 +2245,7 @@
       </x:c>
       <x:c r="I44" s="15" t="str">
         <x:f>IF(B44="","",IFERROR(VLOOKUP(B44,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Right shelving</x:v>
+        <x:v>Left shelving</x:v>
       </x:c>
       <x:c r="J44" s="15" t="str">
         <x:f>IF(B44="","",IFERROR(VLOOKUP(B44,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
@@ -2260,10 +2258,10 @@
     </x:row>
     <x:row r="45" ht="34" customHeight="1">
       <x:c r="A45" s="12" t="str">
-        <x:v>draft_lab_bench_01</x:v>
+        <x:v>draft_conservators_office_shelves_02</x:v>
       </x:c>
       <x:c r="B45" s="12" t="str">
-        <x:v>lab_bench_01</x:v>
+        <x:v>conservators_office_shelves_02</x:v>
       </x:c>
       <x:c r="C45" s="12" t="str"/>
       <x:c r="D45" s="12" t="str">
@@ -2277,15 +2275,15 @@
       </x:c>
       <x:c r="G45" s="15" t="str">
         <x:f>IF(B45="","",IFERROR(VLOOKUP(B45,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>lab</x:v>
+        <x:v>conservators_office</x:v>
       </x:c>
       <x:c r="H45" s="15" t="str">
         <x:f>IF(G45="","",IFERROR(VLOOKUP(G45,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Lab</x:v>
+        <x:v>Conservator's Office</x:v>
       </x:c>
       <x:c r="I45" s="15" t="str">
         <x:f>IF(B45="","",IFERROR(VLOOKUP(B45,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Analysis bench</x:v>
+        <x:v>Rear shelving</x:v>
       </x:c>
       <x:c r="J45" s="15" t="str">
         <x:f>IF(B45="","",IFERROR(VLOOKUP(B45,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
@@ -2298,10 +2296,10 @@
     </x:row>
     <x:row r="46" ht="34" customHeight="1">
       <x:c r="A46" s="12" t="str">
-        <x:v>draft_lab_equipment_01</x:v>
+        <x:v>draft_conservators_office_shelves_03</x:v>
       </x:c>
       <x:c r="B46" s="12" t="str">
-        <x:v>lab_equipment_01</x:v>
+        <x:v>conservators_office_shelves_03</x:v>
       </x:c>
       <x:c r="C46" s="12" t="str"/>
       <x:c r="D46" s="12" t="str">
@@ -2315,15 +2313,15 @@
       </x:c>
       <x:c r="G46" s="15" t="str">
         <x:f>IF(B46="","",IFERROR(VLOOKUP(B46,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
-        <x:v>lab</x:v>
+        <x:v>conservators_office</x:v>
       </x:c>
       <x:c r="H46" s="15" t="str">
         <x:f>IF(G46="","",IFERROR(VLOOKUP(G46,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
-        <x:v>Lab</x:v>
+        <x:v>Conservator's Office</x:v>
       </x:c>
       <x:c r="I46" s="15" t="str">
         <x:f>IF(B46="","",IFERROR(VLOOKUP(B46,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Equipment</x:v>
+        <x:v>Right shelving</x:v>
       </x:c>
       <x:c r="J46" s="15" t="str">
         <x:f>IF(B46="","",IFERROR(VLOOKUP(B46,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
@@ -2336,10 +2334,10 @@
     </x:row>
     <x:row r="47" ht="34" customHeight="1">
       <x:c r="A47" s="12" t="str">
-        <x:v>draft_lab_cabinet_01</x:v>
+        <x:v>draft_lab_bench_01</x:v>
       </x:c>
       <x:c r="B47" s="12" t="str">
-        <x:v>lab_cabinet_01</x:v>
+        <x:v>lab_bench_01</x:v>
       </x:c>
       <x:c r="C47" s="12" t="str"/>
       <x:c r="D47" s="12" t="str">
@@ -2361,7 +2359,7 @@
       </x:c>
       <x:c r="I47" s="15" t="str">
         <x:f>IF(B47="","",IFERROR(VLOOKUP(B47,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Left cabinet</x:v>
+        <x:v>Analysis bench</x:v>
       </x:c>
       <x:c r="J47" s="15" t="str">
         <x:f>IF(B47="","",IFERROR(VLOOKUP(B47,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
@@ -2374,10 +2372,10 @@
     </x:row>
     <x:row r="48" ht="34" customHeight="1">
       <x:c r="A48" s="12" t="str">
-        <x:v>draft_lab_cabinet_02</x:v>
+        <x:v>draft_lab_equipment_01</x:v>
       </x:c>
       <x:c r="B48" s="12" t="str">
-        <x:v>lab_cabinet_02</x:v>
+        <x:v>lab_equipment_01</x:v>
       </x:c>
       <x:c r="C48" s="12" t="str"/>
       <x:c r="D48" s="12" t="str">
@@ -2399,7 +2397,7 @@
       </x:c>
       <x:c r="I48" s="15" t="str">
         <x:f>IF(B48="","",IFERROR(VLOOKUP(B48,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
-        <x:v>Right cabinet</x:v>
+        <x:v>Equipment</x:v>
       </x:c>
       <x:c r="J48" s="15" t="str">
         <x:f>IF(B48="","",IFERROR(VLOOKUP(B48,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
@@ -2410,50 +2408,80 @@
         <x:v>8</x:v>
       </x:c>
     </x:row>
-    <x:row r="49" ht="32" customHeight="1">
-      <x:c r="A49" s="12"/>
-      <x:c r="B49" s="12"/>
-      <x:c r="C49" s="12"/>
-      <x:c r="D49" s="12"/>
-      <x:c r="E49" s="13"/>
-      <x:c r="F49" s="12"/>
+    <x:row r="49" ht="34" customHeight="1">
+      <x:c r="A49" s="12" t="str">
+        <x:v>draft_lab_cabinet_01</x:v>
+      </x:c>
+      <x:c r="B49" s="12" t="str">
+        <x:v>lab_cabinet_01</x:v>
+      </x:c>
+      <x:c r="C49" s="12" t="str"/>
+      <x:c r="D49" s="12" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E49" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F49" s="12" t="str">
+        <x:v>false</x:v>
+      </x:c>
       <x:c r="G49" s="15" t="str">
         <x:f>IF(B49="","",IFERROR(VLOOKUP(B49,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+        <x:v>lab</x:v>
       </x:c>
       <x:c r="H49" s="15" t="str">
         <x:f>IF(G49="","",IFERROR(VLOOKUP(G49,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Lab</x:v>
       </x:c>
       <x:c r="I49" s="15" t="str">
         <x:f>IF(B49="","",IFERROR(VLOOKUP(B49,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+        <x:v>Left cabinet</x:v>
       </x:c>
       <x:c r="J49" s="15" t="str">
         <x:f>IF(B49="","",IFERROR(VLOOKUP(B49,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K49" s="15" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K49" s="15" t="n">
         <x:f>IF(B49="","",IFERROR(VLOOKUP(B49,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="50" ht="32" customHeight="1">
-      <x:c r="A50" s="12"/>
-      <x:c r="B50" s="12"/>
-      <x:c r="C50" s="12"/>
-      <x:c r="D50" s="12"/>
-      <x:c r="E50" s="13"/>
-      <x:c r="F50" s="12"/>
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="34" customHeight="1">
+      <x:c r="A50" s="12" t="str">
+        <x:v>draft_lab_cabinet_02</x:v>
+      </x:c>
+      <x:c r="B50" s="12" t="str">
+        <x:v>lab_cabinet_02</x:v>
+      </x:c>
+      <x:c r="C50" s="12" t="str"/>
+      <x:c r="D50" s="12" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E50" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F50" s="12" t="str">
+        <x:v>false</x:v>
+      </x:c>
       <x:c r="G50" s="15" t="str">
         <x:f>IF(B50="","",IFERROR(VLOOKUP(B50,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+        <x:v>lab</x:v>
       </x:c>
       <x:c r="H50" s="15" t="str">
         <x:f>IF(G50="","",IFERROR(VLOOKUP(G50,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Lab</x:v>
       </x:c>
       <x:c r="I50" s="15" t="str">
         <x:f>IF(B50="","",IFERROR(VLOOKUP(B50,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+        <x:v>Right cabinet</x:v>
       </x:c>
       <x:c r="J50" s="15" t="str">
         <x:f>IF(B50="","",IFERROR(VLOOKUP(B50,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K50" s="15" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="K50" s="15" t="n">
         <x:f>IF(B50="","",IFERROR(VLOOKUP(B50,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="32" customHeight="1">
@@ -2755,23 +2783,69 @@
         <x:f>IF(B63="","",IFERROR(VLOOKUP(B63,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
       </x:c>
     </x:row>
+    <x:row r="64" ht="32" customHeight="1">
+      <x:c r="A64" s="12"/>
+      <x:c r="B64" s="12"/>
+      <x:c r="C64" s="12"/>
+      <x:c r="D64" s="12"/>
+      <x:c r="E64" s="13"/>
+      <x:c r="F64" s="12"/>
+      <x:c r="G64" s="15" t="str">
+        <x:f>IF(B64="","",IFERROR(VLOOKUP(B64,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="H64" s="15" t="str">
+        <x:f>IF(G64="","",IFERROR(VLOOKUP(G64,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I64" s="15" t="str">
+        <x:f>IF(B64="","",IFERROR(VLOOKUP(B64,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="J64" s="15" t="str">
+        <x:f>IF(B64="","",IFERROR(VLOOKUP(B64,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K64" s="15" t="str">
+        <x:f>IF(B64="","",IFERROR(VLOOKUP(B64,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="32" customHeight="1">
+      <x:c r="A65" s="12"/>
+      <x:c r="B65" s="12"/>
+      <x:c r="C65" s="12"/>
+      <x:c r="D65" s="12"/>
+      <x:c r="E65" s="13"/>
+      <x:c r="F65" s="12"/>
+      <x:c r="G65" s="15" t="str">
+        <x:f>IF(B65="","",IFERROR(VLOOKUP(B65,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="H65" s="15" t="str">
+        <x:f>IF(G65="","",IFERROR(VLOOKUP(G65,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I65" s="15" t="str">
+        <x:f>IF(B65="","",IFERROR(VLOOKUP(B65,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="J65" s="15" t="str">
+        <x:f>IF(B65="","",IFERROR(VLOOKUP(B65,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K65" s="15" t="str">
+        <x:f>IF(B65="","",IFERROR(VLOOKUP(B65,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="C2:C63">
+  <x:conditionalFormatting sqref="C2:C65">
     <x:cfRule type="expression" dxfId="0" priority="1">
       <x:formula>AND($A2&lt;&gt;"",$C2="")</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="B2:B63">
+  <x:conditionalFormatting sqref="B2:B65">
     <x:cfRule type="expression" dxfId="1" priority="2">
       <x:formula>AND($A2&lt;&gt;"",$B2&lt;&gt;"",COUNTIF(Slots!$A$2:$A$501,$B2)=0)</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="F2:F63">
+  <x:conditionalFormatting sqref="F2:F65">
     <x:cfRule type="expression" dxfId="2" priority="3">
       <x:formula>AND($A2&lt;&gt;"",$F2="true",COUNTIFS($B$2:$B$501,$B2,$E$2:$E$501,$E2,$F$2:$F$501,"true")&gt;1)</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="E2:E63">
+  <x:conditionalFormatting sqref="E2:E65">
     <x:cfRule type="expression" dxfId="3" priority="4">
       <x:formula>AND($A2&lt;&gt;"",$F2="true",$E2&lt;&gt;"",COUNTIFS($B$2:$B$501,$B2,$E$2:$E$501,$E2,$F$2:$F$501,"true")&gt;1)</x:formula>
     </x:cfRule>
@@ -2792,7 +2866,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf05d92a80e6421e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23a0015b40224927"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2969,7 +3043,7 @@
         <x:v>tool</x:v>
       </x:c>
       <x:c r="E9" s="16" t="str">
-        <x:v>trigger:.welcome-mantle</x:v>
+        <x:v>trigger:.vestibule-welcome-trigger</x:v>
       </x:c>
       <x:c r="F9" s="12" t="str"/>
       <x:c r="G9" s="12" t="str"/>
@@ -3451,7 +3525,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62be95dcee1540c0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ccf8dbe9e9c427c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4105,7 +4179,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0ffb5d20cfe4ab7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b375df68ac14d4a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4345,7 +4419,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7eeedd787854ecf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb080e66598cf433b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4625,7 +4699,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e486a4ba3db490d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc701a1079022438c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5584,7 +5658,7 @@
       <x:c r="I32" s="17" t="str"/>
       <x:c r="J32" s="17" t="str"/>
     </x:row>
-    <x:row r="33" ht="34" customHeight="1">
+    <x:row r="33" ht="44" customHeight="1">
       <x:c r="A33" s="17" t="str">
         <x:v>natural_history_timeline_01</x:v>
       </x:c>
@@ -5592,13 +5666,13 @@
         <x:v>natural_history</x:v>
       </x:c>
       <x:c r="C33" s="17" t="str">
+        <x:v>poster</x:v>
+      </x:c>
+      <x:c r="D33" s="17" t="str">
+        <x:v>Ivory Through Time poster</x:v>
+      </x:c>
+      <x:c r="E33" s="17" t="str">
         <x:v>timeline</x:v>
-      </x:c>
-      <x:c r="D33" s="17" t="str">
-        <x:v>Deep-time explorer</x:v>
-      </x:c>
-      <x:c r="E33" s="17" t="str">
-        <x:v>tool</x:v>
       </x:c>
       <x:c r="F33" s="18" t="n">
         <x:v>1</x:v>
@@ -5609,7 +5683,9 @@
       <x:c r="H33" s="17" t="str">
         <x:v>true</x:v>
       </x:c>
-      <x:c r="I33" s="17" t="str"/>
+      <x:c r="I33" s="17" t="str">
+        <x:v>Arrange the Evidence is the only visitor-facing Natural History timeline activity.</x:v>
+      </x:c>
       <x:c r="J33" s="17" t="str"/>
     </x:row>
     <x:row r="34" ht="34" customHeight="1">
@@ -5640,7 +5716,7 @@
       <x:c r="I34" s="17" t="str"/>
       <x:c r="J34" s="17" t="str"/>
     </x:row>
-    <x:row r="35" ht="34" customHeight="1">
+    <x:row r="35" ht="44" customHeight="1">
       <x:c r="A35" s="17" t="str">
         <x:v>natural_history_timeline_02</x:v>
       </x:c>
@@ -5648,16 +5724,16 @@
         <x:v>natural_history</x:v>
       </x:c>
       <x:c r="C35" s="17" t="str">
-        <x:v>timeline</x:v>
+        <x:v>background_wall</x:v>
       </x:c>
       <x:c r="D35" s="17" t="str">
-        <x:v>Arrange the evidence</x:v>
+        <x:v>Background wall curator mount</x:v>
       </x:c>
       <x:c r="E35" s="17" t="str">
-        <x:v>timeline</x:v>
+        <x:v>collection</x:v>
       </x:c>
       <x:c r="F35" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G35" s="16" t="str">
         <x:v>natural_history_timeline_02_anchor</x:v>
@@ -5665,7 +5741,9 @@
       <x:c r="H35" s="17" t="str">
         <x:v>true</x:v>
       </x:c>
-      <x:c r="I35" s="17" t="str"/>
+      <x:c r="I35" s="17" t="str">
+        <x:v>Available for curator-assigned research and media; no activity is attached.</x:v>
+      </x:c>
       <x:c r="J35" s="17" t="str"/>
     </x:row>
     <x:row r="36" ht="34" customHeight="1">
@@ -5698,81 +5776,85 @@
     </x:row>
     <x:row r="37" ht="34" customHeight="1">
       <x:c r="A37" s="17" t="str">
-        <x:v>conservators_office_terminal_01</x:v>
+        <x:v>natural_history_table_01</x:v>
       </x:c>
       <x:c r="B37" s="17" t="str">
-        <x:v>conservators_office</x:v>
+        <x:v>natural_history</x:v>
       </x:c>
       <x:c r="C37" s="17" t="str">
-        <x:v>terminal</x:v>
+        <x:v>foreground_table</x:v>
       </x:c>
       <x:c r="D37" s="17" t="str">
-        <x:v>Desk terminal</x:v>
+        <x:v>Foreground table left</x:v>
       </x:c>
       <x:c r="E37" s="17" t="str">
-        <x:v>tool</x:v>
+        <x:v>collection</x:v>
       </x:c>
       <x:c r="F37" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G37" s="16" t="str">
-        <x:v>conservators_office_terminal_01_anchor</x:v>
+        <x:v>natural_history_table_01_anchor</x:v>
       </x:c>
       <x:c r="H37" s="17" t="str">
         <x:v>true</x:v>
       </x:c>
-      <x:c r="I37" s="17" t="str"/>
+      <x:c r="I37" s="17" t="str">
+        <x:v>Curator-editable foreground tabletop mount.</x:v>
+      </x:c>
       <x:c r="J37" s="17" t="str"/>
     </x:row>
     <x:row r="38" ht="34" customHeight="1">
       <x:c r="A38" s="17" t="str">
-        <x:v>conservators_office_shelves_01</x:v>
+        <x:v>natural_history_table_02</x:v>
       </x:c>
       <x:c r="B38" s="17" t="str">
-        <x:v>conservators_office</x:v>
+        <x:v>natural_history</x:v>
       </x:c>
       <x:c r="C38" s="17" t="str">
-        <x:v>shelves</x:v>
+        <x:v>foreground_table</x:v>
       </x:c>
       <x:c r="D38" s="17" t="str">
-        <x:v>Left shelving</x:v>
+        <x:v>Foreground table right</x:v>
       </x:c>
       <x:c r="E38" s="17" t="str">
         <x:v>collection</x:v>
       </x:c>
       <x:c r="F38" s="18" t="n">
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G38" s="16" t="str">
-        <x:v>conservators_office_shelves_01_anchor</x:v>
+        <x:v>natural_history_table_02_anchor</x:v>
       </x:c>
       <x:c r="H38" s="17" t="str">
         <x:v>true</x:v>
       </x:c>
-      <x:c r="I38" s="17" t="str"/>
+      <x:c r="I38" s="17" t="str">
+        <x:v>Curator-editable foreground tabletop mount.</x:v>
+      </x:c>
       <x:c r="J38" s="17" t="str"/>
     </x:row>
     <x:row r="39" ht="34" customHeight="1">
       <x:c r="A39" s="17" t="str">
-        <x:v>conservators_office_shelves_02</x:v>
+        <x:v>conservators_office_terminal_01</x:v>
       </x:c>
       <x:c r="B39" s="17" t="str">
         <x:v>conservators_office</x:v>
       </x:c>
       <x:c r="C39" s="17" t="str">
-        <x:v>shelves</x:v>
+        <x:v>terminal</x:v>
       </x:c>
       <x:c r="D39" s="17" t="str">
-        <x:v>Rear shelving</x:v>
+        <x:v>Desk terminal</x:v>
       </x:c>
       <x:c r="E39" s="17" t="str">
-        <x:v>collection</x:v>
+        <x:v>tool</x:v>
       </x:c>
       <x:c r="F39" s="18" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G39" s="16" t="str">
-        <x:v>conservators_office_shelves_02_anchor</x:v>
+        <x:v>conservators_office_terminal_01_anchor</x:v>
       </x:c>
       <x:c r="H39" s="17" t="str">
         <x:v>true</x:v>
@@ -5782,7 +5864,7 @@
     </x:row>
     <x:row r="40" ht="34" customHeight="1">
       <x:c r="A40" s="17" t="str">
-        <x:v>conservators_office_shelves_03</x:v>
+        <x:v>conservators_office_shelves_01</x:v>
       </x:c>
       <x:c r="B40" s="17" t="str">
         <x:v>conservators_office</x:v>
@@ -5791,7 +5873,7 @@
         <x:v>shelves</x:v>
       </x:c>
       <x:c r="D40" s="17" t="str">
-        <x:v>Right shelving</x:v>
+        <x:v>Left shelving</x:v>
       </x:c>
       <x:c r="E40" s="17" t="str">
         <x:v>collection</x:v>
@@ -5800,7 +5882,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G40" s="16" t="str">
-        <x:v>conservators_office_shelves_03_anchor</x:v>
+        <x:v>conservators_office_shelves_01_anchor</x:v>
       </x:c>
       <x:c r="H40" s="17" t="str">
         <x:v>true</x:v>
@@ -5810,25 +5892,25 @@
     </x:row>
     <x:row r="41" ht="34" customHeight="1">
       <x:c r="A41" s="17" t="str">
-        <x:v>conservators_office_panel_01</x:v>
+        <x:v>conservators_office_shelves_02</x:v>
       </x:c>
       <x:c r="B41" s="17" t="str">
         <x:v>conservators_office</x:v>
       </x:c>
       <x:c r="C41" s="17" t="str">
-        <x:v>panel</x:v>
+        <x:v>shelves</x:v>
       </x:c>
       <x:c r="D41" s="17" t="str">
-        <x:v>Elephant wall panel</x:v>
+        <x:v>Rear shelving</x:v>
       </x:c>
       <x:c r="E41" s="17" t="str">
-        <x:v>detail</x:v>
+        <x:v>collection</x:v>
       </x:c>
       <x:c r="F41" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G41" s="16" t="str">
-        <x:v>conservators_office_panel_01_anchor</x:v>
+        <x:v>conservators_office_shelves_02_anchor</x:v>
       </x:c>
       <x:c r="H41" s="17" t="str">
         <x:v>true</x:v>
@@ -5836,18 +5918,18 @@
       <x:c r="I41" s="17" t="str"/>
       <x:c r="J41" s="17" t="str"/>
     </x:row>
-    <x:row r="42" ht="44" customHeight="1">
+    <x:row r="42" ht="34" customHeight="1">
       <x:c r="A42" s="17" t="str">
-        <x:v>lab_bench_01</x:v>
+        <x:v>conservators_office_shelves_03</x:v>
       </x:c>
       <x:c r="B42" s="17" t="str">
-        <x:v>lab</x:v>
+        <x:v>conservators_office</x:v>
       </x:c>
       <x:c r="C42" s="17" t="str">
-        <x:v>bench</x:v>
+        <x:v>shelves</x:v>
       </x:c>
       <x:c r="D42" s="17" t="str">
-        <x:v>Analysis bench</x:v>
+        <x:v>Right shelving</x:v>
       </x:c>
       <x:c r="E42" s="17" t="str">
         <x:v>collection</x:v>
@@ -5856,58 +5938,54 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G42" s="16" t="str">
-        <x:v>lab_bench_01_anchor</x:v>
+        <x:v>conservators_office_shelves_03_anchor</x:v>
       </x:c>
       <x:c r="H42" s="17" t="str">
         <x:v>true</x:v>
       </x:c>
-      <x:c r="I42" s="17" t="str">
-        <x:v>Baseline CSS furnishing; no illustrated replacement authorized as a redesign.</x:v>
-      </x:c>
+      <x:c r="I42" s="17" t="str"/>
       <x:c r="J42" s="17" t="str"/>
     </x:row>
-    <x:row r="43" ht="44" customHeight="1">
+    <x:row r="43" ht="34" customHeight="1">
       <x:c r="A43" s="17" t="str">
-        <x:v>lab_equipment_01</x:v>
+        <x:v>conservators_office_panel_01</x:v>
       </x:c>
       <x:c r="B43" s="17" t="str">
-        <x:v>lab</x:v>
+        <x:v>conservators_office</x:v>
       </x:c>
       <x:c r="C43" s="17" t="str">
-        <x:v>equipment</x:v>
+        <x:v>panel</x:v>
       </x:c>
       <x:c r="D43" s="17" t="str">
-        <x:v>Equipment</x:v>
+        <x:v>Elephant wall panel</x:v>
       </x:c>
       <x:c r="E43" s="17" t="str">
-        <x:v>collection</x:v>
+        <x:v>detail</x:v>
       </x:c>
       <x:c r="F43" s="18" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G43" s="16" t="str">
-        <x:v>lab_equipment_01_anchor</x:v>
+        <x:v>conservators_office_panel_01_anchor</x:v>
       </x:c>
       <x:c r="H43" s="17" t="str">
         <x:v>true</x:v>
       </x:c>
-      <x:c r="I43" s="17" t="str">
-        <x:v>Baseline CSS furnishing; no illustrated replacement authorized as a redesign.</x:v>
-      </x:c>
+      <x:c r="I43" s="17" t="str"/>
       <x:c r="J43" s="17" t="str"/>
     </x:row>
     <x:row r="44" ht="44" customHeight="1">
       <x:c r="A44" s="17" t="str">
-        <x:v>lab_cabinet_01</x:v>
+        <x:v>lab_bench_01</x:v>
       </x:c>
       <x:c r="B44" s="17" t="str">
         <x:v>lab</x:v>
       </x:c>
       <x:c r="C44" s="17" t="str">
-        <x:v>cabinet</x:v>
+        <x:v>bench</x:v>
       </x:c>
       <x:c r="D44" s="17" t="str">
-        <x:v>Left cabinet</x:v>
+        <x:v>Analysis bench</x:v>
       </x:c>
       <x:c r="E44" s="17" t="str">
         <x:v>collection</x:v>
@@ -5916,7 +5994,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G44" s="16" t="str">
-        <x:v>lab_cabinet_01_anchor</x:v>
+        <x:v>lab_bench_01_anchor</x:v>
       </x:c>
       <x:c r="H44" s="17" t="str">
         <x:v>true</x:v>
@@ -5928,16 +6006,16 @@
     </x:row>
     <x:row r="45" ht="44" customHeight="1">
       <x:c r="A45" s="17" t="str">
-        <x:v>lab_cabinet_02</x:v>
+        <x:v>lab_equipment_01</x:v>
       </x:c>
       <x:c r="B45" s="17" t="str">
         <x:v>lab</x:v>
       </x:c>
       <x:c r="C45" s="17" t="str">
-        <x:v>cabinet</x:v>
+        <x:v>equipment</x:v>
       </x:c>
       <x:c r="D45" s="17" t="str">
-        <x:v>Right cabinet</x:v>
+        <x:v>Equipment</x:v>
       </x:c>
       <x:c r="E45" s="17" t="str">
         <x:v>collection</x:v>
@@ -5946,7 +6024,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G45" s="16" t="str">
-        <x:v>lab_cabinet_02_anchor</x:v>
+        <x:v>lab_equipment_01_anchor</x:v>
       </x:c>
       <x:c r="H45" s="17" t="str">
         <x:v>true</x:v>
@@ -5956,57 +6034,93 @@
       </x:c>
       <x:c r="J45" s="17" t="str"/>
     </x:row>
-    <x:row r="46" ht="34" customHeight="1">
+    <x:row r="46" ht="44" customHeight="1">
       <x:c r="A46" s="17" t="str">
-        <x:v>lab_attic_context_01</x:v>
+        <x:v>lab_cabinet_01</x:v>
       </x:c>
       <x:c r="B46" s="17" t="str">
         <x:v>lab</x:v>
       </x:c>
       <x:c r="C46" s="17" t="str">
+        <x:v>cabinet</x:v>
+      </x:c>
+      <x:c r="D46" s="17" t="str">
+        <x:v>Left cabinet</x:v>
+      </x:c>
+      <x:c r="E46" s="17" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="F46" s="18" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G46" s="16" t="str">
+        <x:v>lab_cabinet_01_anchor</x:v>
+      </x:c>
+      <x:c r="H46" s="17" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="I46" s="17" t="str">
+        <x:v>Baseline CSS furnishing; no illustrated replacement authorized as a redesign.</x:v>
+      </x:c>
+      <x:c r="J46" s="17" t="str"/>
+    </x:row>
+    <x:row r="47" ht="44" customHeight="1">
+      <x:c r="A47" s="17" t="str">
+        <x:v>lab_cabinet_02</x:v>
+      </x:c>
+      <x:c r="B47" s="17" t="str">
+        <x:v>lab</x:v>
+      </x:c>
+      <x:c r="C47" s="17" t="str">
+        <x:v>cabinet</x:v>
+      </x:c>
+      <x:c r="D47" s="17" t="str">
+        <x:v>Right cabinet</x:v>
+      </x:c>
+      <x:c r="E47" s="17" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="F47" s="18" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G47" s="16" t="str">
+        <x:v>lab_cabinet_02_anchor</x:v>
+      </x:c>
+      <x:c r="H47" s="17" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="I47" s="17" t="str">
+        <x:v>Baseline CSS furnishing; no illustrated replacement authorized as a redesign.</x:v>
+      </x:c>
+      <x:c r="J47" s="17" t="str"/>
+    </x:row>
+    <x:row r="48" ht="34" customHeight="1">
+      <x:c r="A48" s="17" t="str">
+        <x:v>lab_attic_context_01</x:v>
+      </x:c>
+      <x:c r="B48" s="17" t="str">
+        <x:v>lab</x:v>
+      </x:c>
+      <x:c r="C48" s="17" t="str">
         <x:v>attic</x:v>
       </x:c>
-      <x:c r="D46" s="17" t="str">
+      <x:c r="D48" s="17" t="str">
         <x:v>Attic access context</x:v>
       </x:c>
-      <x:c r="E46" s="17" t="str">
+      <x:c r="E48" s="17" t="str">
         <x:v>tool</x:v>
       </x:c>
-      <x:c r="F46" s="18" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G46" s="16" t="str">
+      <x:c r="F48" s="18" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G48" s="16" t="str">
         <x:v>lab_attic_context_01_anchor</x:v>
       </x:c>
-      <x:c r="H46" s="17" t="str">
-        <x:v>true</x:v>
-      </x:c>
-      <x:c r="I46" s="17" t="str"/>
-      <x:c r="J46" s="17" t="str"/>
-    </x:row>
-    <x:row r="47" ht="32" customHeight="1">
-      <x:c r="A47" s="17"/>
-      <x:c r="B47" s="17"/>
-      <x:c r="C47" s="17"/>
-      <x:c r="D47" s="17"/>
-      <x:c r="E47" s="17"/>
-      <x:c r="F47" s="18"/>
-      <x:c r="G47" s="16"/>
-      <x:c r="H47" s="17"/>
-      <x:c r="I47" s="17"/>
-      <x:c r="J47" s="17"/>
-    </x:row>
-    <x:row r="48" ht="32" customHeight="1">
-      <x:c r="A48" s="17"/>
-      <x:c r="B48" s="17"/>
-      <x:c r="C48" s="17"/>
-      <x:c r="D48" s="17"/>
-      <x:c r="E48" s="17"/>
-      <x:c r="F48" s="18"/>
-      <x:c r="G48" s="16"/>
-      <x:c r="H48" s="17"/>
-      <x:c r="I48" s="17"/>
-      <x:c r="J48" s="17"/>
+      <x:c r="H48" s="17" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="I48" s="17" t="str"/>
+      <x:c r="J48" s="17" t="str"/>
     </x:row>
     <x:row r="49" ht="32" customHeight="1">
       <x:c r="A49" s="17"/>
@@ -6164,6 +6278,30 @@
       <x:c r="I61" s="17"/>
       <x:c r="J61" s="17"/>
     </x:row>
+    <x:row r="62" ht="32" customHeight="1">
+      <x:c r="A62" s="17"/>
+      <x:c r="B62" s="17"/>
+      <x:c r="C62" s="17"/>
+      <x:c r="D62" s="17"/>
+      <x:c r="E62" s="17"/>
+      <x:c r="F62" s="18"/>
+      <x:c r="G62" s="16"/>
+      <x:c r="H62" s="17"/>
+      <x:c r="I62" s="17"/>
+      <x:c r="J62" s="17"/>
+    </x:row>
+    <x:row r="63" ht="32" customHeight="1">
+      <x:c r="A63" s="17"/>
+      <x:c r="B63" s="17"/>
+      <x:c r="C63" s="17"/>
+      <x:c r="D63" s="17"/>
+      <x:c r="E63" s="17"/>
+      <x:c r="F63" s="18"/>
+      <x:c r="G63" s="16"/>
+      <x:c r="H63" s="17"/>
+      <x:c r="I63" s="17"/>
+      <x:c r="J63" s="17"/>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="H2:H501">
@@ -6175,7 +6313,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7c4edf946dd41d0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R663e447f57e34a87"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6715,7 +6853,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb3a29f3290d42a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b3b285d709e46e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6912,7 +7050,7 @@
         <x:v>_data/placements.csv</x:v>
       </x:c>
       <x:c r="B23" s="24" t="str">
-        <x:v>fbca8d56f9e71f2c0692f7e800b0bc75ba10af0e9498432551789a039715cc6f</x:v>
+        <x:v>a3ecc1379c5724e2ab4022bbada405f4d6d2a1894c4b53de24c43b6d7563f5e4</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="58" customHeight="1">
@@ -6920,7 +7058,7 @@
         <x:v>_data/room_content.csv</x:v>
       </x:c>
       <x:c r="B24" s="24" t="str">
-        <x:v>fed299761ab52e9c4c50988789cf740082a9035d97745f7e2a879f57c08a6763</x:v>
+        <x:v>f5964f9accabcc3a9a94d6ab5737bed1542febb3a818df7d153798bcea3fde48</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="58" customHeight="1">
@@ -6952,7 +7090,7 @@
         <x:v>_data/exhibit_slots.csv</x:v>
       </x:c>
       <x:c r="B28" s="24" t="str">
-        <x:v>61f0da63b21935f1116ed34da3e824716b98af51a209f83c7bd993fbc99aae02</x:v>
+        <x:v>2d093b6723b5aa46864919db8329a560a6c36333435f1cf40e12018bd6aa4e77</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="58" customHeight="1">

</xml_diff>

<commit_message>
Add interpretive timeline engine and guided editorial workflow
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/archivory-editorial/ArchIvory Editorial Workbook.xlsx
+++ b/outputs/archivory-editorial/ArchIvory Editorial Workbook.xlsx
@@ -2,14 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Placements" sheetId="1" r:id="R1fccf5d178ae46f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content" sheetId="2" r:id="R422173620e7d4ad2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="3" r:id="R1cc35f938afe451a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timelines" sheetId="4" r:id="Rfa29d11885134574"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rooms" sheetId="5" r:id="R60f5f1cbece142c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slots" sheetId="6" r:id="Rd14f991a94ae4277"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection" sheetId="7" r:id="R22658ec397394493"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="Rae415e6155134866"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Placements" sheetId="1" r:id="R0cf6673335704b3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content" sheetId="2" r:id="R1ba60e2bb612419a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="3" r:id="Rf83177706bc24d9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timelines" sheetId="4" r:id="Re33f1023b6364a91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rooms" sheetId="5" r:id="Rbd5db61eaa964efc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slots" sheetId="6" r:id="R20d23e67ab7d40d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection" sheetId="7" r:id="R7c1592b892834ca5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="Re4288a1cbadb4731"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edit Items" sheetId="9" r:id="Rb1c922022850484c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline Cards" sheetId="10" r:id="Rc28f0ab5e3bb42d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Room Overview" sheetId="11" r:id="R66b6e898cc664bbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing" sheetId="12" r:id="R12462e242c344dea"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +30,7 @@
     <x:numFmt numFmtId="202" formatCode="General"/>
     <x:numFmt numFmtId="203" formatCode="0.000000"/>
   </x:numFmts>
-  <x:fonts count="4">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -48,8 +52,20 @@
       <x:color rgb="FF28313B"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="13"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -76,6 +92,11 @@
         <x:fgColor rgb="FFF0F1F2"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF806238"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -83,7 +104,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="26">
+  <x:cellXfs count="36">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -158,6 +179,24 @@
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -230,8 +269,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="EventsTable" displayName="EventsTable" ref="A1:I32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="9">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="EventsTable" displayName="EventsTable" ref="A1:L32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="12">
     <x:tableColumn id="1" name="timeline_id"/>
     <x:tableColumn id="2" name="id"/>
     <x:tableColumn id="3" name="sortKey"/>
@@ -241,20 +280,33 @@
     <x:tableColumn id="7" name="image"/>
     <x:tableColumn id="8" name="citation"/>
     <x:tableColumn id="9" name="extendedExplanation"/>
+    <x:tableColumn id="10" name="revealText"/>
+    <x:tableColumn id="11" name="promptText"/>
+    <x:tableColumn id="12" name="published"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TimelinesTable" displayName="TimelinesTable" ref="A1:F20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="6">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TimelinesTable" displayName="TimelinesTable" ref="A1:P20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="16">
     <x:tableColumn id="1" name="timeline_id"/>
     <x:tableColumn id="2" name="room_id"/>
     <x:tableColumn id="3" name="roomName"/>
     <x:tableColumn id="4" name="temporalScale"/>
     <x:tableColumn id="5" name="introduction"/>
     <x:tableColumn id="6" name="successText"/>
+    <x:tableColumn id="7" name="title"/>
+    <x:tableColumn id="8" name="subtitle"/>
+    <x:tableColumn id="9" name="deep_question"/>
+    <x:tableColumn id="10" name="intro_text"/>
+    <x:tableColumn id="11" name="start_date"/>
+    <x:tableColumn id="12" name="end_date"/>
+    <x:tableColumn id="13" name="scale_mode"/>
+    <x:tableColumn id="14" name="scale_config"/>
+    <x:tableColumn id="15" name="published"/>
+    <x:tableColumn id="16" name="completion_reflection"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -2866,8 +2918,2406 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23a0015b40224927"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45d9315a020e4989"/>
   </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="32" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="46" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="38" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="32" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="38" customHeight="1">
+      <x:c r="A1" s="28" t="str">
+        <x:v>Add timeline cards by choosing a timeline, supplying a human-readable historical date, and writing the text that appears after a correct placement. Use Events and Timelines for the normalized records imported by the website.</x:v>
+      </x:c>
+      <x:c r="B1" t="str"/>
+      <x:c r="C1" t="str"/>
+      <x:c r="D1" t="str"/>
+      <x:c r="E1" t="str"/>
+      <x:c r="F1" t="str"/>
+      <x:c r="G1" t="str"/>
+      <x:c r="H1" t="str"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str"/>
+      <x:c r="B2" t="str"/>
+      <x:c r="C2" t="str"/>
+      <x:c r="D2" t="str"/>
+      <x:c r="E2" t="str"/>
+      <x:c r="F2" t="str"/>
+      <x:c r="G2" t="str"/>
+      <x:c r="H2" t="str"/>
+    </x:row>
+    <x:row r="3" ht="32" customHeight="1">
+      <x:c r="A3" s="31" t="str">
+        <x:v>Room</x:v>
+      </x:c>
+      <x:c r="B3" s="31" t="str">
+        <x:v>Timeline</x:v>
+      </x:c>
+      <x:c r="C3" s="31" t="str">
+        <x:v>Item title</x:v>
+      </x:c>
+      <x:c r="D3" s="31" t="str">
+        <x:v>Historical date</x:v>
+      </x:c>
+      <x:c r="E3" s="31" t="str">
+        <x:v>Reveal text</x:v>
+      </x:c>
+      <x:c r="F3" s="31" t="str">
+        <x:v>Interpretive prompt</x:v>
+      </x:c>
+      <x:c r="G3" s="31" t="str">
+        <x:v>Image</x:v>
+      </x:c>
+      <x:c r="H3" s="31" t="str">
+        <x:v>Show to visitors?</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="34" customHeight="1">
+      <x:c r="A4" s="35" t="str">
+        <x:v>historical_society</x:v>
+      </x:c>
+      <x:c r="B4" s="35" t="str">
+        <x:v>Historical Society</x:v>
+      </x:c>
+      <x:c r="C4" s="35" t="str">
+        <x:v>Household inventory</x:v>
+      </x:c>
+      <x:c r="D4" s="35" t="str">
+        <x:v>1880 (fictional)</x:v>
+      </x:c>
+      <x:c r="E4" s="35" t="str"/>
+      <x:c r="F4" s="35" t="str"/>
+      <x:c r="G4" s="35" t="str"/>
+      <x:c r="H4" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="34" customHeight="1">
+      <x:c r="A5" s="35" t="str">
+        <x:v>historical_society</x:v>
+      </x:c>
+      <x:c r="B5" s="35" t="str">
+        <x:v>Historical Society</x:v>
+      </x:c>
+      <x:c r="C5" s="35" t="str">
+        <x:v>Letter about a proposed gift</x:v>
+      </x:c>
+      <x:c r="D5" s="35" t="str">
+        <x:v>1905 (fictional)</x:v>
+      </x:c>
+      <x:c r="E5" s="35" t="str"/>
+      <x:c r="F5" s="35" t="str"/>
+      <x:c r="G5" s="35" t="str"/>
+      <x:c r="H5" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="34" customHeight="1">
+      <x:c r="A6" s="35" t="str">
+        <x:v>historical_society</x:v>
+      </x:c>
+      <x:c r="B6" s="35" t="str">
+        <x:v>Historical Society</x:v>
+      </x:c>
+      <x:c r="C6" s="35" t="str">
+        <x:v>Institutional accession</x:v>
+      </x:c>
+      <x:c r="D6" s="35" t="str">
+        <x:v>1910 (fictional)</x:v>
+      </x:c>
+      <x:c r="E6" s="35" t="str"/>
+      <x:c r="F6" s="35" t="str"/>
+      <x:c r="G6" s="35" t="str"/>
+      <x:c r="H6" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="34" customHeight="1">
+      <x:c r="A7" s="35" t="str">
+        <x:v>historical_society</x:v>
+      </x:c>
+      <x:c r="B7" s="35" t="str">
+        <x:v>Historical Society</x:v>
+      </x:c>
+      <x:c r="C7" s="35" t="str">
+        <x:v>Exhibit relabeling</x:v>
+      </x:c>
+      <x:c r="D7" s="35" t="str">
+        <x:v>1935 (fictional)</x:v>
+      </x:c>
+      <x:c r="E7" s="35" t="str"/>
+      <x:c r="F7" s="35" t="str"/>
+      <x:c r="G7" s="35" t="str"/>
+      <x:c r="H7" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="34" customHeight="1">
+      <x:c r="A8" s="35" t="str">
+        <x:v>conservation_lab</x:v>
+      </x:c>
+      <x:c r="B8" s="35" t="str">
+        <x:v>Conservation Lab</x:v>
+      </x:c>
+      <x:c r="C8" s="35" t="str">
+        <x:v>Early carved sample</x:v>
+      </x:c>
+      <x:c r="D8" s="35" t="str">
+        <x:v>2000 BCE (fictional sample)</x:v>
+      </x:c>
+      <x:c r="E8" s="35" t="str"/>
+      <x:c r="F8" s="35" t="str"/>
+      <x:c r="G8" s="35" t="str"/>
+      <x:c r="H8" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="34" customHeight="1">
+      <x:c r="A9" s="35" t="str">
+        <x:v>conservation_lab</x:v>
+      </x:c>
+      <x:c r="B9" s="35" t="str">
+        <x:v>Conservation Lab</x:v>
+      </x:c>
+      <x:c r="C9" s="35" t="str">
+        <x:v>Relief workshop sample</x:v>
+      </x:c>
+      <x:c r="D9" s="35" t="str">
+        <x:v>500 CE (fictional sample)</x:v>
+      </x:c>
+      <x:c r="E9" s="35" t="str"/>
+      <x:c r="F9" s="35" t="str"/>
+      <x:c r="G9" s="35" t="str"/>
+      <x:c r="H9" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="34" customHeight="1">
+      <x:c r="A10" s="35" t="str">
+        <x:v>conservation_lab</x:v>
+      </x:c>
+      <x:c r="B10" s="35" t="str">
+        <x:v>Conservation Lab</x:v>
+      </x:c>
+      <x:c r="C10" s="35" t="str">
+        <x:v>Joined-panel sample</x:v>
+      </x:c>
+      <x:c r="D10" s="35" t="str">
+        <x:v>1200 CE (fictional sample)</x:v>
+      </x:c>
+      <x:c r="E10" s="35" t="str"/>
+      <x:c r="F10" s="35" t="str"/>
+      <x:c r="G10" s="35" t="str"/>
+      <x:c r="H10" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="34" customHeight="1">
+      <x:c r="A11" s="35" t="str">
+        <x:v>conservation_lab</x:v>
+      </x:c>
+      <x:c r="B11" s="35" t="str">
+        <x:v>Conservation Lab</x:v>
+      </x:c>
+      <x:c r="C11" s="35" t="str">
+        <x:v>Turned-object sample</x:v>
+      </x:c>
+      <x:c r="D11" s="35" t="str">
+        <x:v>1800 CE (fictional sample)</x:v>
+      </x:c>
+      <x:c r="E11" s="35" t="str"/>
+      <x:c r="F11" s="35" t="str"/>
+      <x:c r="G11" s="35" t="str"/>
+      <x:c r="H11" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="34" customHeight="1">
+      <x:c r="A12" s="35" t="str">
+        <x:v>attic</x:v>
+      </x:c>
+      <x:c r="B12" s="35" t="str">
+        <x:v>Attic</x:v>
+      </x:c>
+      <x:c r="C12" s="35" t="str">
+        <x:v>Old inventory</x:v>
+      </x:c>
+      <x:c r="D12" s="35" t="str">
+        <x:v>1900 (fictional)</x:v>
+      </x:c>
+      <x:c r="E12" s="35" t="str"/>
+      <x:c r="F12" s="35" t="str"/>
+      <x:c r="G12" s="35" t="str"/>
+      <x:c r="H12" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="34" customHeight="1">
+      <x:c r="A13" s="35" t="str">
+        <x:v>attic</x:v>
+      </x:c>
+      <x:c r="B13" s="35" t="str">
+        <x:v>Attic</x:v>
+      </x:c>
+      <x:c r="C13" s="35" t="str">
+        <x:v>Undated photograph</x:v>
+      </x:c>
+      <x:c r="D13" s="35" t="str">
+        <x:v>1920s, uncertain (fictional)</x:v>
+      </x:c>
+      <x:c r="E13" s="35" t="str"/>
+      <x:c r="F13" s="35" t="str"/>
+      <x:c r="G13" s="35" t="str"/>
+      <x:c r="H13" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="34" customHeight="1">
+      <x:c r="A14" s="35" t="str">
+        <x:v>attic</x:v>
+      </x:c>
+      <x:c r="B14" s="35" t="str">
+        <x:v>Attic</x:v>
+      </x:c>
+      <x:c r="C14" s="35" t="str">
+        <x:v>Loose envelope</x:v>
+      </x:c>
+      <x:c r="D14" s="35" t="str">
+        <x:v>1920s, uncertain (fictional)</x:v>
+      </x:c>
+      <x:c r="E14" s="35" t="str"/>
+      <x:c r="F14" s="35" t="str"/>
+      <x:c r="G14" s="35" t="str"/>
+      <x:c r="H14" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="34" customHeight="1">
+      <x:c r="A15" s="35" t="str">
+        <x:v>attic</x:v>
+      </x:c>
+      <x:c r="B15" s="35" t="str">
+        <x:v>Attic</x:v>
+      </x:c>
+      <x:c r="C15" s="35" t="str">
+        <x:v>Trunk rediscovered</x:v>
+      </x:c>
+      <x:c r="D15" s="35" t="str">
+        <x:v>1970 (fictional)</x:v>
+      </x:c>
+      <x:c r="E15" s="35" t="str"/>
+      <x:c r="F15" s="35" t="str"/>
+      <x:c r="G15" s="35" t="str"/>
+      <x:c r="H15" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="34" customHeight="1">
+      <x:c r="A16" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B16" s="35" t="str">
+        <x:v>Ivory Through Time</x:v>
+      </x:c>
+      <x:c r="C16" s="35" t="str">
+        <x:v>Early Proboscideans</x:v>
+      </x:c>
+      <x:c r="D16" s="35" t="str">
+        <x:v>ca. 60–34 million years ago</x:v>
+      </x:c>
+      <x:c r="E16" s="35" t="str">
+        <x:v>The earliest part of the axis represents long ecological change before modern elephants or human ivory trade.</x:v>
+      </x:c>
+      <x:c r="F16" s="35" t="str">
+        <x:v>What evidence can show environmental change across this much time?</x:v>
+      </x:c>
+      <x:c r="G16" s="35" t="str"/>
+      <x:c r="H16" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="34" customHeight="1">
+      <x:c r="A17" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B17" s="35" t="str">
+        <x:v>Ivory Through Time</x:v>
+      </x:c>
+      <x:c r="C17" s="35" t="str">
+        <x:v>Miocene Dispersal</x:v>
+      </x:c>
+      <x:c r="D17" s="35" t="str">
+        <x:v>ca. 23–5.3 million years ago</x:v>
+      </x:c>
+      <x:c r="E17" s="35" t="str">
+        <x:v>Dispersal links fossil evidence to changing habitats and migration routes rather than a single fixed homeland.</x:v>
+      </x:c>
+      <x:c r="F17" s="35" t="str">
+        <x:v>How might movement across regions change the materials and stories available to people?</x:v>
+      </x:c>
+      <x:c r="G17" s="35" t="str"/>
+      <x:c r="H17" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="34" customHeight="1">
+      <x:c r="A18" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B18" s="35" t="str">
+        <x:v>Ivory Through Time</x:v>
+      </x:c>
+      <x:c r="C18" s="35" t="str">
+        <x:v>Pleistocene Diversity</x:v>
+      </x:c>
+      <x:c r="D18" s="35" t="str">
+        <x:v>ca. 2.6 million–11,700 years ago</x:v>
+      </x:c>
+      <x:c r="E18" s="35" t="str">
+        <x:v>The compressed late band still covers millions of years of diverse proboscidean lives and environments.</x:v>
+      </x:c>
+      <x:c r="F18" s="35" t="str">
+        <x:v>What is lost when a long period is treated as a single moment?</x:v>
+      </x:c>
+      <x:c r="G18" s="35" t="str"/>
+      <x:c r="H18" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="34" customHeight="1">
+      <x:c r="A19" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B19" s="35" t="str">
+        <x:v>Ivory Through Time</x:v>
+      </x:c>
+      <x:c r="C19" s="35" t="str">
+        <x:v>Late Proboscidean Extinctions</x:v>
+      </x:c>
+      <x:c r="D19" s="35" t="str">
+        <x:v>Late Pleistocene–Holocene</x:v>
+      </x:c>
+      <x:c r="E19" s="35" t="str">
+        <x:v>Late extinctions bring ecological pressures and human action into the same interpretive frame without reducing either to one cause.</x:v>
+      </x:c>
+      <x:c r="F19" s="35" t="str">
+        <x:v>How should uncertainty shape the stories we tell about extinction and extraction?</x:v>
+      </x:c>
+      <x:c r="G19" s="35" t="str"/>
+      <x:c r="H19" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="32" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="46" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="38" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="38" customHeight="1">
+      <x:c r="A1" s="28" t="str">
+        <x:v>Use this room-by-room overview to find available locations. Reserved locations become visible only after supported content is assigned and published.</x:v>
+      </x:c>
+      <x:c r="B1" t="str"/>
+      <x:c r="C1" t="str"/>
+      <x:c r="D1" t="str"/>
+      <x:c r="E1" t="str"/>
+      <x:c r="F1" t="str"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str"/>
+      <x:c r="B2" t="str"/>
+      <x:c r="C2" t="str"/>
+      <x:c r="D2" t="str"/>
+      <x:c r="E2" t="str"/>
+      <x:c r="F2" t="str"/>
+    </x:row>
+    <x:row r="3" ht="32" customHeight="1">
+      <x:c r="A3" s="31" t="str">
+        <x:v>Room</x:v>
+      </x:c>
+      <x:c r="B3" s="31" t="str">
+        <x:v>Location</x:v>
+      </x:c>
+      <x:c r="C3" s="31" t="str">
+        <x:v>What kind of item is this?</x:v>
+      </x:c>
+      <x:c r="D3" s="31" t="str">
+        <x:v>Capacity</x:v>
+      </x:c>
+      <x:c r="E3" s="31" t="str">
+        <x:v>Ready for editing?</x:v>
+      </x:c>
+      <x:c r="F3" s="31" t="str">
+        <x:v>Current visitor content</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="34" customHeight="1">
+      <x:c r="A4" s="35" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="B4" s="35" t="str">
+        <x:v>Gallery introduction</x:v>
+      </x:c>
+      <x:c r="C4" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="D4" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E4" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F4" s="35" t="str">
+        <x:v>Gallery Intro</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="34" customHeight="1">
+      <x:c r="A5" s="35" t="str">
+        <x:v>conservation_lab</x:v>
+      </x:c>
+      <x:c r="B5" s="35" t="str">
+        <x:v>Conservation Lab introduction</x:v>
+      </x:c>
+      <x:c r="C5" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="D5" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E5" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F5" s="35" t="str">
+        <x:v>Conservation Lab Intro</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="34" customHeight="1">
+      <x:c r="A6" s="35" t="str">
+        <x:v>historical_society</x:v>
+      </x:c>
+      <x:c r="B6" s="35" t="str">
+        <x:v>Historical Society introduction</x:v>
+      </x:c>
+      <x:c r="C6" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="D6" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E6" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F6" s="35" t="str">
+        <x:v>Reserved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="34" customHeight="1">
+      <x:c r="A7" s="35" t="str">
+        <x:v>attic</x:v>
+      </x:c>
+      <x:c r="B7" s="35" t="str">
+        <x:v>Attic introduction</x:v>
+      </x:c>
+      <x:c r="C7" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="D7" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E7" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F7" s="35" t="str">
+        <x:v>Reserved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="34" customHeight="1">
+      <x:c r="A8" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B8" s="35" t="str">
+        <x:v>Natural History Museum introduction</x:v>
+      </x:c>
+      <x:c r="C8" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="D8" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E8" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F8" s="35" t="str">
+        <x:v>Reserved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="34" customHeight="1">
+      <x:c r="A9" s="35" t="str">
+        <x:v>conservators_office</x:v>
+      </x:c>
+      <x:c r="B9" s="35" t="str">
+        <x:v>Conservator's Office introduction</x:v>
+      </x:c>
+      <x:c r="C9" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="D9" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E9" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F9" s="35" t="str">
+        <x:v>Reserved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="34" customHeight="1">
+      <x:c r="A10" s="35" t="str">
+        <x:v>lab</x:v>
+      </x:c>
+      <x:c r="B10" s="35" t="str">
+        <x:v>Lab introduction</x:v>
+      </x:c>
+      <x:c r="C10" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="D10" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E10" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F10" s="35" t="str">
+        <x:v>Reserved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="34" customHeight="1">
+      <x:c r="A11" s="35" t="str">
+        <x:v>vestibule</x:v>
+      </x:c>
+      <x:c r="B11" s="35" t="str">
+        <x:v>Welcome and check-in</x:v>
+      </x:c>
+      <x:c r="C11" s="35" t="str">
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="D11" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E11" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F11" s="35" t="str">
+        <x:v>Welcome to ArchIvory</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="34" customHeight="1">
+      <x:c r="A12" s="35" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="B12" s="35" t="str">
+        <x:v>Near left-wall relief</x:v>
+      </x:c>
+      <x:c r="C12" s="35" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="D12" s="35" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E12" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F12" s="35" t="str">
+        <x:v>Susanna and the Elders</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="34" customHeight="1">
+      <x:c r="A13" s="35" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="B13" s="35" t="str">
+        <x:v>Far left-wall relief</x:v>
+      </x:c>
+      <x:c r="C13" s="35" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="D13" s="35" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E13" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F13" s="35" t="str">
+        <x:v>Illustrated relief — identity unverified; Barberini Ivory</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="34" customHeight="1">
+      <x:c r="A14" s="35" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="B14" s="35" t="str">
+        <x:v>Front glass case</x:v>
+      </x:c>
+      <x:c r="C14" s="35" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="D14" s="35" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E14" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F14" s="35" t="str">
+        <x:v>Illustrated folding fan</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="34" customHeight="1">
+      <x:c r="A15" s="35" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="B15" s="35" t="str">
+        <x:v>Rear round display</x:v>
+      </x:c>
+      <x:c r="C15" s="35" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="D15" s="35" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E15" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F15" s="35" t="str">
+        <x:v>Reserved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="34" customHeight="1">
+      <x:c r="A16" s="35" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="B16" s="35" t="str">
+        <x:v>Small rear-wall frame</x:v>
+      </x:c>
+      <x:c r="C16" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="D16" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E16" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F16" s="35" t="str">
+        <x:v>Roman Wall Sconce</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="34" customHeight="1">
+      <x:c r="A17" s="35" t="str">
+        <x:v>conservation_lab</x:v>
+      </x:c>
+      <x:c r="B17" s="35" t="str">
+        <x:v>Central ivories collection</x:v>
+      </x:c>
+      <x:c r="C17" s="35" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="D17" s="35" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E17" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F17" s="35" t="str">
+        <x:v>IU Eskenazi Museum Ivories</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="34" customHeight="1">
+      <x:c r="A18" s="35" t="str">
+        <x:v>conservation_lab</x:v>
+      </x:c>
+      <x:c r="B18" s="35" t="str">
+        <x:v>Ivory Through the Ages</x:v>
+      </x:c>
+      <x:c r="C18" s="35" t="str">
+        <x:v>timeline</x:v>
+      </x:c>
+      <x:c r="D18" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E18" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F18" s="35" t="str">
+        <x:v>ivory_ages</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="34" customHeight="1">
+      <x:c r="A19" s="35" t="str">
+        <x:v>conservation_lab</x:v>
+      </x:c>
+      <x:c r="B19" s="35" t="str">
+        <x:v>Rear analysis workbench</x:v>
+      </x:c>
+      <x:c r="C19" s="35" t="str">
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="D19" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E19" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F19" s="35" t="str">
+        <x:v>Analysis workbench</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="34" customHeight="1">
+      <x:c r="A20" s="35" t="str">
+        <x:v>historical_society</x:v>
+      </x:c>
+      <x:c r="B20" s="35" t="str">
+        <x:v>Local Lives</x:v>
+      </x:c>
+      <x:c r="C20" s="35" t="str">
+        <x:v>timeline</x:v>
+      </x:c>
+      <x:c r="D20" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E20" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F20" s="35" t="str">
+        <x:v>local_lives</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="34" customHeight="1">
+      <x:c r="A21" s="35" t="str">
+        <x:v>historical_society</x:v>
+      </x:c>
+      <x:c r="B21" s="35" t="str">
+        <x:v>Window-side case</x:v>
+      </x:c>
+      <x:c r="C21" s="35" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="D21" s="35" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E21" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F21" s="35" t="str">
+        <x:v>Reserved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="34" customHeight="1">
+      <x:c r="A22" s="35" t="str">
+        <x:v>historical_society</x:v>
+      </x:c>
+      <x:c r="B22" s="35" t="str">
+        <x:v>Foreground-right case</x:v>
+      </x:c>
+      <x:c r="C22" s="35" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="D22" s="35" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E22" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F22" s="35" t="str">
+        <x:v>Reserved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="34" customHeight="1">
+      <x:c r="A23" s="35" t="str">
+        <x:v>historical_society</x:v>
+      </x:c>
+      <x:c r="B23" s="35" t="str">
+        <x:v>Piano</x:v>
+      </x:c>
+      <x:c r="C23" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="D23" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E23" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F23" s="35" t="str">
+        <x:v>Piano</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="34" customHeight="1">
+      <x:c r="A24" s="35" t="str">
+        <x:v>historical_society</x:v>
+      </x:c>
+      <x:c r="B24" s="35" t="str">
+        <x:v>Billiards table</x:v>
+      </x:c>
+      <x:c r="C24" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="D24" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E24" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F24" s="35" t="str">
+        <x:v>Billiards table</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="34" customHeight="1">
+      <x:c r="A25" s="35" t="str">
+        <x:v>attic</x:v>
+      </x:c>
+      <x:c r="B25" s="35" t="str">
+        <x:v>Family Traces</x:v>
+      </x:c>
+      <x:c r="C25" s="35" t="str">
+        <x:v>timeline</x:v>
+      </x:c>
+      <x:c r="D25" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E25" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F25" s="35" t="str">
+        <x:v>family_traces</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="34" customHeight="1">
+      <x:c r="A26" s="35" t="str">
+        <x:v>attic</x:v>
+      </x:c>
+      <x:c r="B26" s="35" t="str">
+        <x:v>Left open trunk</x:v>
+      </x:c>
+      <x:c r="C26" s="35" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="D26" s="35" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E26" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F26" s="35" t="str">
+        <x:v>Reserved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="34" customHeight="1">
+      <x:c r="A27" s="35" t="str">
+        <x:v>attic</x:v>
+      </x:c>
+      <x:c r="B27" s="35" t="str">
+        <x:v>Right open trunk</x:v>
+      </x:c>
+      <x:c r="C27" s="35" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="D27" s="35" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E27" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F27" s="35" t="str">
+        <x:v>Reserved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="34" customHeight="1">
+      <x:c r="A28" s="35" t="str">
+        <x:v>attic</x:v>
+      </x:c>
+      <x:c r="B28" s="35" t="str">
+        <x:v>Shelving</x:v>
+      </x:c>
+      <x:c r="C28" s="35" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="D28" s="35" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E28" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F28" s="35" t="str">
+        <x:v>Reserved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="34" customHeight="1">
+      <x:c r="A29" s="35" t="str">
+        <x:v>attic</x:v>
+      </x:c>
+      <x:c r="B29" s="35" t="str">
+        <x:v>Research table</x:v>
+      </x:c>
+      <x:c r="C29" s="35" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="D29" s="35" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E29" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F29" s="35" t="str">
+        <x:v>Reserved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="34" customHeight="1">
+      <x:c r="A30" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B30" s="35" t="str">
+        <x:v>Tusk specimen</x:v>
+      </x:c>
+      <x:c r="C30" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="D30" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E30" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F30" s="35" t="str">
+        <x:v>Elephant tusk</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="34" customHeight="1">
+      <x:c r="A31" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B31" s="35" t="str">
+        <x:v>Specimen label</x:v>
+      </x:c>
+      <x:c r="C31" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="D31" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E31" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F31" s="35" t="str">
+        <x:v>Elephant tusk</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="34" customHeight="1">
+      <x:c r="A32" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B32" s="35" t="str">
+        <x:v>Elephant interpretation panel</x:v>
+      </x:c>
+      <x:c r="C32" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="D32" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E32" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F32" s="35" t="str">
+        <x:v>Natural History Intro</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="34" customHeight="1">
+      <x:c r="A33" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B33" s="35" t="str">
+        <x:v>Central recessed panel</x:v>
+      </x:c>
+      <x:c r="C33" s="35" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="D33" s="35" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E33" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F33" s="35" t="str">
+        <x:v>Geib Flute</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="34" customHeight="1">
+      <x:c r="A34" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B34" s="35" t="str">
+        <x:v>Wall map</x:v>
+      </x:c>
+      <x:c r="C34" s="35" t="str">
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="D34" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E34" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F34" s="35" t="str">
+        <x:v>World map</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="34" customHeight="1">
+      <x:c r="A35" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B35" s="35" t="str">
+        <x:v>Ivory Through Time poster</x:v>
+      </x:c>
+      <x:c r="C35" s="35" t="str">
+        <x:v>timeline</x:v>
+      </x:c>
+      <x:c r="D35" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E35" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F35" s="35" t="str">
+        <x:v>Ivory Through Time</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="34" customHeight="1">
+      <x:c r="A36" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B36" s="35" t="str">
+        <x:v>Habitation map within explorer</x:v>
+      </x:c>
+      <x:c r="C36" s="35" t="str">
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="D36" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E36" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F36" s="35" t="str">
+        <x:v>Habitation map</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="34" customHeight="1">
+      <x:c r="A37" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B37" s="35" t="str">
+        <x:v>Background wall curator mount</x:v>
+      </x:c>
+      <x:c r="C37" s="35" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="D37" s="35" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E37" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F37" s="35" t="str">
+        <x:v>Reserved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="34" customHeight="1">
+      <x:c r="A38" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B38" s="35" t="str">
+        <x:v>Ivory inquiry</x:v>
+      </x:c>
+      <x:c r="C38" s="35" t="str">
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="D38" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E38" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F38" s="35" t="str">
+        <x:v>Ivory Inquiry Terminal</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="34" customHeight="1">
+      <x:c r="A39" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B39" s="35" t="str">
+        <x:v>Foreground table left</x:v>
+      </x:c>
+      <x:c r="C39" s="35" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="D39" s="35" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E39" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F39" s="35" t="str">
+        <x:v>Reserved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="34" customHeight="1">
+      <x:c r="A40" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B40" s="35" t="str">
+        <x:v>Foreground table right</x:v>
+      </x:c>
+      <x:c r="C40" s="35" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="D40" s="35" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E40" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F40" s="35" t="str">
+        <x:v>Reserved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="34" customHeight="1">
+      <x:c r="A41" s="35" t="str">
+        <x:v>conservators_office</x:v>
+      </x:c>
+      <x:c r="B41" s="35" t="str">
+        <x:v>Desk terminal</x:v>
+      </x:c>
+      <x:c r="C41" s="35" t="str">
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="D41" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E41" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F41" s="35" t="str">
+        <x:v>Curation terminal</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="34" customHeight="1">
+      <x:c r="A42" s="35" t="str">
+        <x:v>conservators_office</x:v>
+      </x:c>
+      <x:c r="B42" s="35" t="str">
+        <x:v>Left shelving</x:v>
+      </x:c>
+      <x:c r="C42" s="35" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="D42" s="35" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E42" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F42" s="35" t="str">
+        <x:v>Reserved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="34" customHeight="1">
+      <x:c r="A43" s="35" t="str">
+        <x:v>conservators_office</x:v>
+      </x:c>
+      <x:c r="B43" s="35" t="str">
+        <x:v>Rear shelving</x:v>
+      </x:c>
+      <x:c r="C43" s="35" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="D43" s="35" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E43" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F43" s="35" t="str">
+        <x:v>Reserved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="34" customHeight="1">
+      <x:c r="A44" s="35" t="str">
+        <x:v>conservators_office</x:v>
+      </x:c>
+      <x:c r="B44" s="35" t="str">
+        <x:v>Right shelving</x:v>
+      </x:c>
+      <x:c r="C44" s="35" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="D44" s="35" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E44" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F44" s="35" t="str">
+        <x:v>Reserved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="34" customHeight="1">
+      <x:c r="A45" s="35" t="str">
+        <x:v>conservators_office</x:v>
+      </x:c>
+      <x:c r="B45" s="35" t="str">
+        <x:v>Elephant wall panel</x:v>
+      </x:c>
+      <x:c r="C45" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="D45" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E45" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F45" s="35" t="str">
+        <x:v>Conservators Office Intro</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="34" customHeight="1">
+      <x:c r="A46" s="35" t="str">
+        <x:v>lab</x:v>
+      </x:c>
+      <x:c r="B46" s="35" t="str">
+        <x:v>Analysis bench</x:v>
+      </x:c>
+      <x:c r="C46" s="35" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="D46" s="35" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E46" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F46" s="35" t="str">
+        <x:v>Reserved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="34" customHeight="1">
+      <x:c r="A47" s="35" t="str">
+        <x:v>lab</x:v>
+      </x:c>
+      <x:c r="B47" s="35" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="C47" s="35" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="D47" s="35" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E47" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F47" s="35" t="str">
+        <x:v>Reserved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="34" customHeight="1">
+      <x:c r="A48" s="35" t="str">
+        <x:v>lab</x:v>
+      </x:c>
+      <x:c r="B48" s="35" t="str">
+        <x:v>Left cabinet</x:v>
+      </x:c>
+      <x:c r="C48" s="35" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="D48" s="35" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E48" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F48" s="35" t="str">
+        <x:v>Reserved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="34" customHeight="1">
+      <x:c r="A49" s="35" t="str">
+        <x:v>lab</x:v>
+      </x:c>
+      <x:c r="B49" s="35" t="str">
+        <x:v>Right cabinet</x:v>
+      </x:c>
+      <x:c r="C49" s="35" t="str">
+        <x:v>collection</x:v>
+      </x:c>
+      <x:c r="D49" s="35" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E49" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F49" s="35" t="str">
+        <x:v>Reserved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="34" customHeight="1">
+      <x:c r="A50" s="35" t="str">
+        <x:v>lab</x:v>
+      </x:c>
+      <x:c r="B50" s="35" t="str">
+        <x:v>Attic access context</x:v>
+      </x:c>
+      <x:c r="C50" s="35" t="str">
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="D50" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E50" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F50" s="35" t="str">
+        <x:v>Attic investigations</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="32" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="46" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="38" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="38" customHeight="1">
+      <x:c r="A1" s="28" t="str">
+        <x:v>Review what visitors can currently see. Change the backend Placements published field to true or false, then run the workbook check before sharing.</x:v>
+      </x:c>
+      <x:c r="B1" t="str"/>
+      <x:c r="C1" t="str"/>
+      <x:c r="D1" t="str"/>
+      <x:c r="E1" t="str"/>
+      <x:c r="F1" t="str"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str"/>
+      <x:c r="B2" t="str"/>
+      <x:c r="C2" t="str"/>
+      <x:c r="D2" t="str"/>
+      <x:c r="E2" t="str"/>
+      <x:c r="F2" t="str"/>
+    </x:row>
+    <x:row r="3" ht="32" customHeight="1">
+      <x:c r="A3" s="31" t="str">
+        <x:v>Room</x:v>
+      </x:c>
+      <x:c r="B3" s="31" t="str">
+        <x:v>Where should it appear?</x:v>
+      </x:c>
+      <x:c r="C3" s="31" t="str">
+        <x:v>Item title</x:v>
+      </x:c>
+      <x:c r="D3" s="31" t="str">
+        <x:v>What kind of item is this?</x:v>
+      </x:c>
+      <x:c r="E3" s="31" t="str">
+        <x:v>Show to visitors?</x:v>
+      </x:c>
+      <x:c r="F3" s="31" t="str">
+        <x:v>Placement ID</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="34" customHeight="1">
+      <x:c r="A4" s="35" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="B4" s="35" t="str">
+        <x:v>Gallery introduction</x:v>
+      </x:c>
+      <x:c r="C4" s="35" t="str">
+        <x:v>Gallery Intro</x:v>
+      </x:c>
+      <x:c r="D4" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E4" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F4" s="35" t="str">
+        <x:v>gallery_intro_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="34" customHeight="1">
+      <x:c r="A5" s="35" t="str">
+        <x:v>conservation_lab</x:v>
+      </x:c>
+      <x:c r="B5" s="35" t="str">
+        <x:v>Conservation Lab introduction</x:v>
+      </x:c>
+      <x:c r="C5" s="35" t="str">
+        <x:v>Conservation Lab Intro</x:v>
+      </x:c>
+      <x:c r="D5" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E5" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F5" s="35" t="str">
+        <x:v>conservation_lab_intro_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="34" customHeight="1">
+      <x:c r="A6" s="35" t="str">
+        <x:v>vestibule</x:v>
+      </x:c>
+      <x:c r="B6" s="35" t="str">
+        <x:v>Welcome and check-in</x:v>
+      </x:c>
+      <x:c r="C6" s="35" t="str">
+        <x:v>Welcome to ArchIvory</x:v>
+      </x:c>
+      <x:c r="D6" s="35" t="str">
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="E6" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F6" s="35" t="str">
+        <x:v>vestibule_welcome_01_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="34" customHeight="1">
+      <x:c r="A7" s="35" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="B7" s="35" t="str">
+        <x:v>Near left-wall relief</x:v>
+      </x:c>
+      <x:c r="C7" s="35" t="str">
+        <x:v>Illustrated relief — identity unverified</x:v>
+      </x:c>
+      <x:c r="D7" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E7" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F7" s="35" t="str">
+        <x:v>gallery_wall_01_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="34" customHeight="1">
+      <x:c r="A8" s="35" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="B8" s="35" t="str">
+        <x:v>Near left-wall relief</x:v>
+      </x:c>
+      <x:c r="C8" s="35" t="str">
+        <x:v>Susanna and the Elders</x:v>
+      </x:c>
+      <x:c r="D8" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E8" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F8" s="35" t="str">
+        <x:v>gallery_wall_01_2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="34" customHeight="1">
+      <x:c r="A9" s="35" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="B9" s="35" t="str">
+        <x:v>Far left-wall relief</x:v>
+      </x:c>
+      <x:c r="C9" s="35" t="str">
+        <x:v>Illustrated relief — identity unverified</x:v>
+      </x:c>
+      <x:c r="D9" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E9" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F9" s="35" t="str">
+        <x:v>gallery_wall_02_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="34" customHeight="1">
+      <x:c r="A10" s="35" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="B10" s="35" t="str">
+        <x:v>Far left-wall relief</x:v>
+      </x:c>
+      <x:c r="C10" s="35" t="str">
+        <x:v>Barberini Ivory</x:v>
+      </x:c>
+      <x:c r="D10" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E10" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F10" s="35" t="str">
+        <x:v>gallery_wall_02_2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="34" customHeight="1">
+      <x:c r="A11" s="35" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="B11" s="35" t="str">
+        <x:v>Front glass case</x:v>
+      </x:c>
+      <x:c r="C11" s="35" t="str">
+        <x:v>Illustrated folding fan</x:v>
+      </x:c>
+      <x:c r="D11" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E11" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F11" s="35" t="str">
+        <x:v>gallery_case_01_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="34" customHeight="1">
+      <x:c r="A12" s="35" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="B12" s="35" t="str">
+        <x:v>Small rear-wall frame</x:v>
+      </x:c>
+      <x:c r="C12" s="35" t="str">
+        <x:v>Roman Wall Sconce</x:v>
+      </x:c>
+      <x:c r="D12" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E12" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F12" s="35" t="str">
+        <x:v>gallery_wall_03_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="34" customHeight="1">
+      <x:c r="A13" s="35" t="str">
+        <x:v>conservation_lab</x:v>
+      </x:c>
+      <x:c r="B13" s="35" t="str">
+        <x:v>Central ivories collection</x:v>
+      </x:c>
+      <x:c r="C13" s="35" t="str">
+        <x:v>IU Eskenazi Museum Ivories</x:v>
+      </x:c>
+      <x:c r="D13" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E13" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F13" s="35" t="str">
+        <x:v>conservation_lab_table_01_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="34" customHeight="1">
+      <x:c r="A14" s="35" t="str">
+        <x:v>conservation_lab</x:v>
+      </x:c>
+      <x:c r="B14" s="35" t="str">
+        <x:v>Ivory Through the Ages</x:v>
+      </x:c>
+      <x:c r="C14" s="35" t="str">
+        <x:v>ivory_ages</x:v>
+      </x:c>
+      <x:c r="D14" s="35" t="str">
+        <x:v>timeline</x:v>
+      </x:c>
+      <x:c r="E14" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F14" s="35" t="str">
+        <x:v>conservation_lab_timeline_01_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="34" customHeight="1">
+      <x:c r="A15" s="35" t="str">
+        <x:v>conservation_lab</x:v>
+      </x:c>
+      <x:c r="B15" s="35" t="str">
+        <x:v>Rear analysis workbench</x:v>
+      </x:c>
+      <x:c r="C15" s="35" t="str">
+        <x:v>Analysis workbench</x:v>
+      </x:c>
+      <x:c r="D15" s="35" t="str">
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="E15" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F15" s="35" t="str">
+        <x:v>conservation_lab_media_01_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="34" customHeight="1">
+      <x:c r="A16" s="35" t="str">
+        <x:v>historical_society</x:v>
+      </x:c>
+      <x:c r="B16" s="35" t="str">
+        <x:v>Local Lives</x:v>
+      </x:c>
+      <x:c r="C16" s="35" t="str">
+        <x:v>local_lives</x:v>
+      </x:c>
+      <x:c r="D16" s="35" t="str">
+        <x:v>timeline</x:v>
+      </x:c>
+      <x:c r="E16" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F16" s="35" t="str">
+        <x:v>historical_society_timeline_01_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="34" customHeight="1">
+      <x:c r="A17" s="35" t="str">
+        <x:v>historical_society</x:v>
+      </x:c>
+      <x:c r="B17" s="35" t="str">
+        <x:v>Piano</x:v>
+      </x:c>
+      <x:c r="C17" s="35" t="str">
+        <x:v>Piano</x:v>
+      </x:c>
+      <x:c r="D17" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E17" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F17" s="35" t="str">
+        <x:v>historical_society_piano_01_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="34" customHeight="1">
+      <x:c r="A18" s="35" t="str">
+        <x:v>historical_society</x:v>
+      </x:c>
+      <x:c r="B18" s="35" t="str">
+        <x:v>Billiards table</x:v>
+      </x:c>
+      <x:c r="C18" s="35" t="str">
+        <x:v>Billiards table</x:v>
+      </x:c>
+      <x:c r="D18" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E18" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F18" s="35" t="str">
+        <x:v>historical_society_table_01_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="34" customHeight="1">
+      <x:c r="A19" s="35" t="str">
+        <x:v>attic</x:v>
+      </x:c>
+      <x:c r="B19" s="35" t="str">
+        <x:v>Family Traces</x:v>
+      </x:c>
+      <x:c r="C19" s="35" t="str">
+        <x:v>family_traces</x:v>
+      </x:c>
+      <x:c r="D19" s="35" t="str">
+        <x:v>timeline</x:v>
+      </x:c>
+      <x:c r="E19" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F19" s="35" t="str">
+        <x:v>attic_timeline_01_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="34" customHeight="1">
+      <x:c r="A20" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B20" s="35" t="str">
+        <x:v>Tusk specimen</x:v>
+      </x:c>
+      <x:c r="C20" s="35" t="str">
+        <x:v>Elephant tusk</x:v>
+      </x:c>
+      <x:c r="D20" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E20" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F20" s="35" t="str">
+        <x:v>natural_history_specimen_01_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="34" customHeight="1">
+      <x:c r="A21" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B21" s="35" t="str">
+        <x:v>Specimen label</x:v>
+      </x:c>
+      <x:c r="C21" s="35" t="str">
+        <x:v>Elephant tusk</x:v>
+      </x:c>
+      <x:c r="D21" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E21" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F21" s="35" t="str">
+        <x:v>natural_history_specimen_01_label_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="34" customHeight="1">
+      <x:c r="A22" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B22" s="35" t="str">
+        <x:v>Elephant interpretation panel</x:v>
+      </x:c>
+      <x:c r="C22" s="35" t="str">
+        <x:v>Natural History Intro</x:v>
+      </x:c>
+      <x:c r="D22" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E22" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F22" s="35" t="str">
+        <x:v>natural_history_panel_01_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="34" customHeight="1">
+      <x:c r="A23" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B23" s="35" t="str">
+        <x:v>Wall map</x:v>
+      </x:c>
+      <x:c r="C23" s="35" t="str">
+        <x:v>World map</x:v>
+      </x:c>
+      <x:c r="D23" s="35" t="str">
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="E23" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F23" s="35" t="str">
+        <x:v>natural_history_map_01_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="34" customHeight="1">
+      <x:c r="A24" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B24" s="35" t="str">
+        <x:v>Ivory Through Time poster</x:v>
+      </x:c>
+      <x:c r="C24" s="35" t="str">
+        <x:v>Ivory Through Time</x:v>
+      </x:c>
+      <x:c r="D24" s="35" t="str">
+        <x:v>timeline</x:v>
+      </x:c>
+      <x:c r="E24" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F24" s="35" t="str">
+        <x:v>natural_history_timeline_01_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="34" customHeight="1">
+      <x:c r="A25" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B25" s="35" t="str">
+        <x:v>Habitation map within explorer</x:v>
+      </x:c>
+      <x:c r="C25" s="35" t="str">
+        <x:v>Habitation map</x:v>
+      </x:c>
+      <x:c r="D25" s="35" t="str">
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="E25" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F25" s="35" t="str">
+        <x:v>natural_history_map_02_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="34" customHeight="1">
+      <x:c r="A26" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B26" s="35" t="str">
+        <x:v>Ivory inquiry</x:v>
+      </x:c>
+      <x:c r="C26" s="35" t="str">
+        <x:v>Ivory Inquiry Terminal</x:v>
+      </x:c>
+      <x:c r="D26" s="35" t="str">
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="E26" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F26" s="35" t="str">
+        <x:v>natural_history_inquiry_01_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="34" customHeight="1">
+      <x:c r="A27" s="35" t="str">
+        <x:v>conservators_office</x:v>
+      </x:c>
+      <x:c r="B27" s="35" t="str">
+        <x:v>Desk terminal</x:v>
+      </x:c>
+      <x:c r="C27" s="35" t="str">
+        <x:v>Curation terminal</x:v>
+      </x:c>
+      <x:c r="D27" s="35" t="str">
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="E27" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F27" s="35" t="str">
+        <x:v>conservators_office_terminal_01_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="34" customHeight="1">
+      <x:c r="A28" s="35" t="str">
+        <x:v>conservators_office</x:v>
+      </x:c>
+      <x:c r="B28" s="35" t="str">
+        <x:v>Elephant wall panel</x:v>
+      </x:c>
+      <x:c r="C28" s="35" t="str">
+        <x:v>Conservators Office Intro</x:v>
+      </x:c>
+      <x:c r="D28" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E28" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F28" s="35" t="str">
+        <x:v>conservators_office_panel_01_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="34" customHeight="1">
+      <x:c r="A29" s="35" t="str">
+        <x:v>lab</x:v>
+      </x:c>
+      <x:c r="B29" s="35" t="str">
+        <x:v>Attic access context</x:v>
+      </x:c>
+      <x:c r="C29" s="35" t="str">
+        <x:v>Attic investigations</x:v>
+      </x:c>
+      <x:c r="D29" s="35" t="str">
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="E29" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F29" s="35" t="str">
+        <x:v>lab_attic_context_01_1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="34" customHeight="1">
+      <x:c r="A30" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B30" s="35" t="str">
+        <x:v>Central recessed panel</x:v>
+      </x:c>
+      <x:c r="C30" s="35" t="str">
+        <x:v>Geib Flute</x:v>
+      </x:c>
+      <x:c r="D30" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E30" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F30" s="35" t="str">
+        <x:v>geib-flute</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="34" customHeight="1">
+      <x:c r="A31" s="35" t="str">
+        <x:v>historical_society</x:v>
+      </x:c>
+      <x:c r="B31" s="35" t="str">
+        <x:v>Historical Society introduction</x:v>
+      </x:c>
+      <x:c r="C31" s="35" t="str"/>
+      <x:c r="D31" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E31" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F31" s="35" t="str">
+        <x:v>draft_historical_society_intro</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="34" customHeight="1">
+      <x:c r="A32" s="35" t="str">
+        <x:v>attic</x:v>
+      </x:c>
+      <x:c r="B32" s="35" t="str">
+        <x:v>Attic introduction</x:v>
+      </x:c>
+      <x:c r="C32" s="35" t="str"/>
+      <x:c r="D32" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E32" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F32" s="35" t="str">
+        <x:v>draft_attic_intro</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="34" customHeight="1">
+      <x:c r="A33" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B33" s="35" t="str">
+        <x:v>Natural History Museum introduction</x:v>
+      </x:c>
+      <x:c r="C33" s="35" t="str"/>
+      <x:c r="D33" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E33" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F33" s="35" t="str">
+        <x:v>draft_natural_history_intro</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="34" customHeight="1">
+      <x:c r="A34" s="35" t="str">
+        <x:v>conservators_office</x:v>
+      </x:c>
+      <x:c r="B34" s="35" t="str">
+        <x:v>Conservator's Office introduction</x:v>
+      </x:c>
+      <x:c r="C34" s="35" t="str"/>
+      <x:c r="D34" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E34" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F34" s="35" t="str">
+        <x:v>draft_conservators_office_intro</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="34" customHeight="1">
+      <x:c r="A35" s="35" t="str">
+        <x:v>lab</x:v>
+      </x:c>
+      <x:c r="B35" s="35" t="str">
+        <x:v>Lab introduction</x:v>
+      </x:c>
+      <x:c r="C35" s="35" t="str"/>
+      <x:c r="D35" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E35" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F35" s="35" t="str">
+        <x:v>draft_lab_intro</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="34" customHeight="1">
+      <x:c r="A36" s="35" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="B36" s="35" t="str">
+        <x:v>Rear round display</x:v>
+      </x:c>
+      <x:c r="C36" s="35" t="str"/>
+      <x:c r="D36" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E36" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F36" s="35" t="str">
+        <x:v>draft_gallery_case_02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="34" customHeight="1">
+      <x:c r="A37" s="35" t="str">
+        <x:v>historical_society</x:v>
+      </x:c>
+      <x:c r="B37" s="35" t="str">
+        <x:v>Window-side case</x:v>
+      </x:c>
+      <x:c r="C37" s="35" t="str"/>
+      <x:c r="D37" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E37" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F37" s="35" t="str">
+        <x:v>draft_historical_society_case_01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="34" customHeight="1">
+      <x:c r="A38" s="35" t="str">
+        <x:v>historical_society</x:v>
+      </x:c>
+      <x:c r="B38" s="35" t="str">
+        <x:v>Foreground-right case</x:v>
+      </x:c>
+      <x:c r="C38" s="35" t="str"/>
+      <x:c r="D38" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E38" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F38" s="35" t="str">
+        <x:v>draft_historical_society_case_02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="34" customHeight="1">
+      <x:c r="A39" s="35" t="str">
+        <x:v>attic</x:v>
+      </x:c>
+      <x:c r="B39" s="35" t="str">
+        <x:v>Left open trunk</x:v>
+      </x:c>
+      <x:c r="C39" s="35" t="str"/>
+      <x:c r="D39" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E39" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F39" s="35" t="str">
+        <x:v>draft_attic_trunk_01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="34" customHeight="1">
+      <x:c r="A40" s="35" t="str">
+        <x:v>attic</x:v>
+      </x:c>
+      <x:c r="B40" s="35" t="str">
+        <x:v>Right open trunk</x:v>
+      </x:c>
+      <x:c r="C40" s="35" t="str"/>
+      <x:c r="D40" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E40" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F40" s="35" t="str">
+        <x:v>draft_attic_trunk_02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="34" customHeight="1">
+      <x:c r="A41" s="35" t="str">
+        <x:v>attic</x:v>
+      </x:c>
+      <x:c r="B41" s="35" t="str">
+        <x:v>Shelving</x:v>
+      </x:c>
+      <x:c r="C41" s="35" t="str"/>
+      <x:c r="D41" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E41" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F41" s="35" t="str">
+        <x:v>draft_attic_shelves_01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="34" customHeight="1">
+      <x:c r="A42" s="35" t="str">
+        <x:v>attic</x:v>
+      </x:c>
+      <x:c r="B42" s="35" t="str">
+        <x:v>Research table</x:v>
+      </x:c>
+      <x:c r="C42" s="35" t="str"/>
+      <x:c r="D42" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E42" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F42" s="35" t="str">
+        <x:v>draft_attic_table_01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="34" customHeight="1">
+      <x:c r="A43" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B43" s="35" t="str">
+        <x:v>Background wall curator mount</x:v>
+      </x:c>
+      <x:c r="C43" s="35" t="str"/>
+      <x:c r="D43" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E43" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F43" s="35" t="str">
+        <x:v>draft_natural_history_timeline_02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="34" customHeight="1">
+      <x:c r="A44" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B44" s="35" t="str">
+        <x:v>Foreground table left</x:v>
+      </x:c>
+      <x:c r="C44" s="35" t="str"/>
+      <x:c r="D44" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E44" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F44" s="35" t="str">
+        <x:v>draft_natural_history_table_01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="34" customHeight="1">
+      <x:c r="A45" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B45" s="35" t="str">
+        <x:v>Foreground table right</x:v>
+      </x:c>
+      <x:c r="C45" s="35" t="str"/>
+      <x:c r="D45" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E45" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F45" s="35" t="str">
+        <x:v>draft_natural_history_table_02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="34" customHeight="1">
+      <x:c r="A46" s="35" t="str">
+        <x:v>conservators_office</x:v>
+      </x:c>
+      <x:c r="B46" s="35" t="str">
+        <x:v>Left shelving</x:v>
+      </x:c>
+      <x:c r="C46" s="35" t="str"/>
+      <x:c r="D46" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E46" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F46" s="35" t="str">
+        <x:v>draft_conservators_office_shelves_01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="34" customHeight="1">
+      <x:c r="A47" s="35" t="str">
+        <x:v>conservators_office</x:v>
+      </x:c>
+      <x:c r="B47" s="35" t="str">
+        <x:v>Rear shelving</x:v>
+      </x:c>
+      <x:c r="C47" s="35" t="str"/>
+      <x:c r="D47" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E47" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F47" s="35" t="str">
+        <x:v>draft_conservators_office_shelves_02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="34" customHeight="1">
+      <x:c r="A48" s="35" t="str">
+        <x:v>conservators_office</x:v>
+      </x:c>
+      <x:c r="B48" s="35" t="str">
+        <x:v>Right shelving</x:v>
+      </x:c>
+      <x:c r="C48" s="35" t="str"/>
+      <x:c r="D48" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E48" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F48" s="35" t="str">
+        <x:v>draft_conservators_office_shelves_03</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="34" customHeight="1">
+      <x:c r="A49" s="35" t="str">
+        <x:v>lab</x:v>
+      </x:c>
+      <x:c r="B49" s="35" t="str">
+        <x:v>Analysis bench</x:v>
+      </x:c>
+      <x:c r="C49" s="35" t="str"/>
+      <x:c r="D49" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E49" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F49" s="35" t="str">
+        <x:v>draft_lab_bench_01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="34" customHeight="1">
+      <x:c r="A50" s="35" t="str">
+        <x:v>lab</x:v>
+      </x:c>
+      <x:c r="B50" s="35" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
+      <x:c r="C50" s="35" t="str"/>
+      <x:c r="D50" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E50" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F50" s="35" t="str">
+        <x:v>draft_lab_equipment_01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="34" customHeight="1">
+      <x:c r="A51" s="35" t="str">
+        <x:v>lab</x:v>
+      </x:c>
+      <x:c r="B51" s="35" t="str">
+        <x:v>Left cabinet</x:v>
+      </x:c>
+      <x:c r="C51" s="35" t="str"/>
+      <x:c r="D51" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E51" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F51" s="35" t="str">
+        <x:v>draft_lab_cabinet_01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="34" customHeight="1">
+      <x:c r="A52" s="35" t="str">
+        <x:v>lab</x:v>
+      </x:c>
+      <x:c r="B52" s="35" t="str">
+        <x:v>Right cabinet</x:v>
+      </x:c>
+      <x:c r="C52" s="35" t="str"/>
+      <x:c r="D52" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E52" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F52" s="35" t="str">
+        <x:v>draft_lab_cabinet_02</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
@@ -3525,7 +5975,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ccf8dbe9e9c427c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re25c2d70ea974e2c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3543,6 +5993,9 @@
     <x:col min="7" max="7" width="56" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="66" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="76" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="28" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="28" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
@@ -3573,6 +6026,15 @@
       <x:c r="I1" s="10" t="str">
         <x:v>extendedExplanation</x:v>
       </x:c>
+      <x:c r="J1" s="10" t="str">
+        <x:v>revealText</x:v>
+      </x:c>
+      <x:c r="K1" s="10" t="str">
+        <x:v>promptText</x:v>
+      </x:c>
+      <x:c r="L1" s="10" t="str">
+        <x:v>published</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="44" customHeight="1">
       <x:c r="A2" s="12" t="str">
@@ -3600,6 +6062,9 @@
       <x:c r="I2" s="12" t="str">
         <x:v>An inventory lists an unnamed carved object.</x:v>
       </x:c>
+      <x:c r="J2" s="12" t="str"/>
+      <x:c r="K2" s="12" t="str"/>
+      <x:c r="L2" s="12" t="str"/>
     </x:row>
     <x:row r="3" ht="44" customHeight="1">
       <x:c r="A3" s="12" t="str">
@@ -3627,6 +6092,9 @@
       <x:c r="I3" s="12" t="str">
         <x:v>A letter proposes a gift; intention is not a completed transfer.</x:v>
       </x:c>
+      <x:c r="J3" s="12" t="str"/>
+      <x:c r="K3" s="12" t="str"/>
+      <x:c r="L3" s="12" t="str"/>
     </x:row>
     <x:row r="4" ht="44" customHeight="1">
       <x:c r="A4" s="12" t="str">
@@ -3654,6 +6122,9 @@
       <x:c r="I4" s="12" t="str">
         <x:v>An accession entry records receipt by a local institution.</x:v>
       </x:c>
+      <x:c r="J4" s="12" t="str"/>
+      <x:c r="K4" s="12" t="str"/>
+      <x:c r="L4" s="12" t="str"/>
     </x:row>
     <x:row r="5" ht="44" customHeight="1">
       <x:c r="A5" s="12" t="str">
@@ -3681,6 +6152,9 @@
       <x:c r="I5" s="12" t="str">
         <x:v>A new label changes the interpretation of the object.</x:v>
       </x:c>
+      <x:c r="J5" s="12" t="str"/>
+      <x:c r="K5" s="12" t="str"/>
+      <x:c r="L5" s="12" t="str"/>
     </x:row>
     <x:row r="6" ht="44" customHeight="1">
       <x:c r="A6" s="12" t="str">
@@ -3708,6 +6182,9 @@
       <x:c r="I6" s="12" t="str">
         <x:v>A teaching sample introduces carving as a material practice.</x:v>
       </x:c>
+      <x:c r="J6" s="12" t="str"/>
+      <x:c r="K6" s="12" t="str"/>
+      <x:c r="L6" s="12" t="str"/>
     </x:row>
     <x:row r="7" ht="44" customHeight="1">
       <x:c r="A7" s="12" t="str">
@@ -3735,6 +6212,9 @@
       <x:c r="I7" s="12" t="str">
         <x:v>A later teaching sample explores relief technique.</x:v>
       </x:c>
+      <x:c r="J7" s="12" t="str"/>
+      <x:c r="K7" s="12" t="str"/>
+      <x:c r="L7" s="12" t="str"/>
     </x:row>
     <x:row r="8" ht="44" customHeight="1">
       <x:c r="A8" s="12" t="str">
@@ -3762,6 +6242,9 @@
       <x:c r="I8" s="12" t="str">
         <x:v>A teaching sample asks how construction and display relate.</x:v>
       </x:c>
+      <x:c r="J8" s="12" t="str"/>
+      <x:c r="K8" s="12" t="str"/>
+      <x:c r="L8" s="12" t="str"/>
     </x:row>
     <x:row r="9" ht="44" customHeight="1">
       <x:c r="A9" s="12" t="str">
@@ -3789,6 +6272,9 @@
       <x:c r="I9" s="12" t="str">
         <x:v>A teaching sample introduces another way to work the material.</x:v>
       </x:c>
+      <x:c r="J9" s="12" t="str"/>
+      <x:c r="K9" s="12" t="str"/>
+      <x:c r="L9" s="12" t="str"/>
     </x:row>
     <x:row r="10" ht="44" customHeight="1">
       <x:c r="A10" s="12" t="str">
@@ -3816,6 +6302,9 @@
       <x:c r="I10" s="12" t="str">
         <x:v>A household inventory survives.</x:v>
       </x:c>
+      <x:c r="J10" s="12" t="str"/>
+      <x:c r="K10" s="12" t="str"/>
+      <x:c r="L10" s="12" t="str"/>
     </x:row>
     <x:row r="11" ht="44" customHeight="1">
       <x:c r="A11" s="12" t="str">
@@ -3843,6 +6332,9 @@
       <x:c r="I11" s="12" t="str">
         <x:v>Equivalent to the envelope: either order is accepted. The image does not prove ownership.</x:v>
       </x:c>
+      <x:c r="J11" s="12" t="str"/>
+      <x:c r="K11" s="12" t="str"/>
+      <x:c r="L11" s="12" t="str"/>
     </x:row>
     <x:row r="12" ht="44" customHeight="1">
       <x:c r="A12" s="12" t="str">
@@ -3870,6 +6362,9 @@
       <x:c r="I12" s="12" t="str">
         <x:v>Equivalent to the photograph: there is no evidence to order them within the decade.</x:v>
       </x:c>
+      <x:c r="J12" s="12" t="str"/>
+      <x:c r="K12" s="12" t="str"/>
+      <x:c r="L12" s="12" t="str"/>
     </x:row>
     <x:row r="13" ht="44" customHeight="1">
       <x:c r="A13" s="12" t="str">
@@ -3897,6 +6392,9 @@
       <x:c r="I13" s="12" t="str">
         <x:v>The missing years do not establish who kept the object or how it moved.</x:v>
       </x:c>
+      <x:c r="J13" s="12" t="str"/>
+      <x:c r="K13" s="12" t="str"/>
+      <x:c r="L13" s="12" t="str"/>
     </x:row>
     <x:row r="14" ht="76" customHeight="1">
       <x:c r="A14" s="12" t="str">
@@ -3924,6 +6422,15 @@
       <x:c r="I14" s="12" t="str">
         <x:v>This state emphasizes origin and diversification. Visitors should distinguish the broader proboscidean order from the much later appearance of modern elephants. Broad interval ordering uses onset groups; not a precise date for every occurrence.</x:v>
       </x:c>
+      <x:c r="J14" s="12" t="str">
+        <x:v>The earliest part of the axis represents long ecological change before modern elephants or human ivory trade.</x:v>
+      </x:c>
+      <x:c r="K14" s="12" t="str">
+        <x:v>What evidence can show environmental change across this much time?</x:v>
+      </x:c>
+      <x:c r="L14" s="12" t="str">
+        <x:v>true</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="76" customHeight="1">
       <x:c r="A15" s="12" t="str">
@@ -3951,8 +6458,17 @@
       <x:c r="I15" s="12" t="str">
         <x:v>Movement across continents makes geography part of evolutionary history. Range maps should be treated as reconstructions based on fossil localities, not perfectly known boundaries. Broad interval ordering uses onset groups; not a precise date for every occurrence.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="16" ht="60" customHeight="1">
+      <x:c r="J15" s="12" t="str">
+        <x:v>Dispersal links fossil evidence to changing habitats and migration routes rather than a single fixed homeland.</x:v>
+      </x:c>
+      <x:c r="K15" s="12" t="str">
+        <x:v>How might movement across regions change the materials and stories available to people?</x:v>
+      </x:c>
+      <x:c r="L15" s="12" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="76" customHeight="1">
       <x:c r="A16" s="12" t="str">
         <x:v>deep_time_evidence</x:v>
       </x:c>
@@ -3978,8 +6494,17 @@
       <x:c r="I16" s="12" t="str">
         <x:v>The late Pleistocene shows that recent proboscidean diversity was once much greater than the three living elephant species suggest. Broad interval ordering uses onset groups; not a precise date for every occurrence.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="17" ht="76" customHeight="1">
+      <x:c r="J16" s="12" t="str">
+        <x:v>The compressed late band still covers millions of years of diverse proboscidean lives and environments.</x:v>
+      </x:c>
+      <x:c r="K16" s="12" t="str">
+        <x:v>What is lost when a long period is treated as a single moment?</x:v>
+      </x:c>
+      <x:c r="L16" s="12" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="92" customHeight="1">
       <x:c r="A17" s="12" t="str">
         <x:v>deep_time_evidence</x:v>
       </x:c>
@@ -4004,6 +6529,15 @@
       </x:c>
       <x:c r="I17" s="12" t="str">
         <x:v>Extinction should not be presented as monocausal. Climate, habitat change, human pressure, and regional variation must be weighed against one another. Broad interval ordering uses onset groups; not a precise date for every occurrence.</x:v>
+      </x:c>
+      <x:c r="J17" s="12" t="str">
+        <x:v>Late extinctions bring ecological pressures and human action into the same interpretive frame without reducing either to one cause.</x:v>
+      </x:c>
+      <x:c r="K17" s="12" t="str">
+        <x:v>How should uncertainty shape the stories we tell about extinction and extraction?</x:v>
+      </x:c>
+      <x:c r="L17" s="12" t="str">
+        <x:v>true</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="32" customHeight="1">
@@ -4016,6 +6550,9 @@
       <x:c r="G18" s="12"/>
       <x:c r="H18" s="12"/>
       <x:c r="I18" s="12"/>
+      <x:c r="J18" s="12"/>
+      <x:c r="K18" s="12"/>
+      <x:c r="L18" s="12"/>
     </x:row>
     <x:row r="19" ht="32" customHeight="1">
       <x:c r="A19" s="12"/>
@@ -4027,6 +6564,9 @@
       <x:c r="G19" s="12"/>
       <x:c r="H19" s="12"/>
       <x:c r="I19" s="12"/>
+      <x:c r="J19" s="12"/>
+      <x:c r="K19" s="12"/>
+      <x:c r="L19" s="12"/>
     </x:row>
     <x:row r="20" ht="32" customHeight="1">
       <x:c r="A20" s="12"/>
@@ -4038,6 +6578,9 @@
       <x:c r="G20" s="12"/>
       <x:c r="H20" s="12"/>
       <x:c r="I20" s="12"/>
+      <x:c r="J20" s="12"/>
+      <x:c r="K20" s="12"/>
+      <x:c r="L20" s="12"/>
     </x:row>
     <x:row r="21" ht="32" customHeight="1">
       <x:c r="A21" s="12"/>
@@ -4049,6 +6592,9 @@
       <x:c r="G21" s="12"/>
       <x:c r="H21" s="12"/>
       <x:c r="I21" s="12"/>
+      <x:c r="J21" s="12"/>
+      <x:c r="K21" s="12"/>
+      <x:c r="L21" s="12"/>
     </x:row>
     <x:row r="22" ht="32" customHeight="1">
       <x:c r="A22" s="12"/>
@@ -4060,6 +6606,9 @@
       <x:c r="G22" s="12"/>
       <x:c r="H22" s="12"/>
       <x:c r="I22" s="12"/>
+      <x:c r="J22" s="12"/>
+      <x:c r="K22" s="12"/>
+      <x:c r="L22" s="12"/>
     </x:row>
     <x:row r="23" ht="32" customHeight="1">
       <x:c r="A23" s="12"/>
@@ -4071,6 +6620,9 @@
       <x:c r="G23" s="12"/>
       <x:c r="H23" s="12"/>
       <x:c r="I23" s="12"/>
+      <x:c r="J23" s="12"/>
+      <x:c r="K23" s="12"/>
+      <x:c r="L23" s="12"/>
     </x:row>
     <x:row r="24" ht="32" customHeight="1">
       <x:c r="A24" s="12"/>
@@ -4082,6 +6634,9 @@
       <x:c r="G24" s="12"/>
       <x:c r="H24" s="12"/>
       <x:c r="I24" s="12"/>
+      <x:c r="J24" s="12"/>
+      <x:c r="K24" s="12"/>
+      <x:c r="L24" s="12"/>
     </x:row>
     <x:row r="25" ht="32" customHeight="1">
       <x:c r="A25" s="12"/>
@@ -4093,6 +6648,9 @@
       <x:c r="G25" s="12"/>
       <x:c r="H25" s="12"/>
       <x:c r="I25" s="12"/>
+      <x:c r="J25" s="12"/>
+      <x:c r="K25" s="12"/>
+      <x:c r="L25" s="12"/>
     </x:row>
     <x:row r="26" ht="32" customHeight="1">
       <x:c r="A26" s="12"/>
@@ -4104,6 +6662,9 @@
       <x:c r="G26" s="12"/>
       <x:c r="H26" s="12"/>
       <x:c r="I26" s="12"/>
+      <x:c r="J26" s="12"/>
+      <x:c r="K26" s="12"/>
+      <x:c r="L26" s="12"/>
     </x:row>
     <x:row r="27" ht="32" customHeight="1">
       <x:c r="A27" s="12"/>
@@ -4115,6 +6676,9 @@
       <x:c r="G27" s="12"/>
       <x:c r="H27" s="12"/>
       <x:c r="I27" s="12"/>
+      <x:c r="J27" s="12"/>
+      <x:c r="K27" s="12"/>
+      <x:c r="L27" s="12"/>
     </x:row>
     <x:row r="28" ht="32" customHeight="1">
       <x:c r="A28" s="12"/>
@@ -4126,6 +6690,9 @@
       <x:c r="G28" s="12"/>
       <x:c r="H28" s="12"/>
       <x:c r="I28" s="12"/>
+      <x:c r="J28" s="12"/>
+      <x:c r="K28" s="12"/>
+      <x:c r="L28" s="12"/>
     </x:row>
     <x:row r="29" ht="32" customHeight="1">
       <x:c r="A29" s="12"/>
@@ -4137,6 +6704,9 @@
       <x:c r="G29" s="12"/>
       <x:c r="H29" s="12"/>
       <x:c r="I29" s="12"/>
+      <x:c r="J29" s="12"/>
+      <x:c r="K29" s="12"/>
+      <x:c r="L29" s="12"/>
     </x:row>
     <x:row r="30" ht="32" customHeight="1">
       <x:c r="A30" s="12"/>
@@ -4148,6 +6718,9 @@
       <x:c r="G30" s="12"/>
       <x:c r="H30" s="12"/>
       <x:c r="I30" s="12"/>
+      <x:c r="J30" s="12"/>
+      <x:c r="K30" s="12"/>
+      <x:c r="L30" s="12"/>
     </x:row>
     <x:row r="31" ht="32" customHeight="1">
       <x:c r="A31" s="12"/>
@@ -4159,6 +6732,9 @@
       <x:c r="G31" s="12"/>
       <x:c r="H31" s="12"/>
       <x:c r="I31" s="12"/>
+      <x:c r="J31" s="12"/>
+      <x:c r="K31" s="12"/>
+      <x:c r="L31" s="12"/>
     </x:row>
     <x:row r="32" ht="32" customHeight="1">
       <x:c r="A32" s="12"/>
@@ -4170,16 +6746,22 @@
       <x:c r="G32" s="12"/>
       <x:c r="H32" s="12"/>
       <x:c r="I32" s="12"/>
+      <x:c r="J32" s="12"/>
+      <x:c r="K32" s="12"/>
+      <x:c r="L32" s="12"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="1">
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="L2:L501">
+      <x:formula1>"true,false"</x:formula1>
+    </x:dataValidation>
     <x:dataValidation type="list" sqref="A2:A501">
       <x:formula1>'Timelines'!$A$2:$A$501</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b375df68ac14d4a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb93538e37f484e7f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4194,6 +6776,16 @@
     <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="76" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="76" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="38" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="28" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="28" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="28" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="28" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="28" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="28" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="28" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="28" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
@@ -4215,6 +6807,36 @@
       <x:c r="F1" s="10" t="str">
         <x:v>successText</x:v>
       </x:c>
+      <x:c r="G1" s="10" t="str">
+        <x:v>title</x:v>
+      </x:c>
+      <x:c r="H1" s="10" t="str">
+        <x:v>subtitle</x:v>
+      </x:c>
+      <x:c r="I1" s="10" t="str">
+        <x:v>deep_question</x:v>
+      </x:c>
+      <x:c r="J1" s="10" t="str">
+        <x:v>intro_text</x:v>
+      </x:c>
+      <x:c r="K1" s="11" t="str">
+        <x:v>start_date</x:v>
+      </x:c>
+      <x:c r="L1" s="11" t="str">
+        <x:v>end_date</x:v>
+      </x:c>
+      <x:c r="M1" s="10" t="str">
+        <x:v>scale_mode</x:v>
+      </x:c>
+      <x:c r="N1" s="10" t="str">
+        <x:v>scale_config</x:v>
+      </x:c>
+      <x:c r="O1" s="10" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="P1" s="10" t="str">
+        <x:v>completion_reflection</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="60" customHeight="1">
       <x:c r="A2" s="12" t="str">
@@ -4235,6 +6857,16 @@
       <x:c r="F2" s="12" t="str">
         <x:v>At the scale of years and decades, an individual decision or an accession can redirect an object’s history. A gap between documents remains a gap; it does not prove continuous ownership.</x:v>
       </x:c>
+      <x:c r="G2" s="12" t="str"/>
+      <x:c r="H2" s="12" t="str"/>
+      <x:c r="I2" s="12" t="str"/>
+      <x:c r="J2" s="12" t="str"/>
+      <x:c r="K2" s="13" t="str"/>
+      <x:c r="L2" s="13" t="str"/>
+      <x:c r="M2" s="12" t="str"/>
+      <x:c r="N2" s="12" t="str"/>
+      <x:c r="O2" s="12" t="str"/>
+      <x:c r="P2" s="12" t="str"/>
     </x:row>
     <x:row r="3" ht="60" customHeight="1">
       <x:c r="A3" s="12" t="str">
@@ -4255,6 +6887,16 @@
       <x:c r="F3" s="12" t="str">
         <x:v>Across centuries and millennia, related materials can support changing techniques and meanings. A broad period comparison reveals artistic traditions, while obscuring the individual transfers visible at a shorter scale.</x:v>
       </x:c>
+      <x:c r="G3" s="12" t="str"/>
+      <x:c r="H3" s="12" t="str"/>
+      <x:c r="I3" s="12" t="str"/>
+      <x:c r="J3" s="12" t="str"/>
+      <x:c r="K3" s="13" t="str"/>
+      <x:c r="L3" s="13" t="str"/>
+      <x:c r="M3" s="12" t="str"/>
+      <x:c r="N3" s="12" t="str"/>
+      <x:c r="O3" s="12" t="str"/>
+      <x:c r="P3" s="12" t="str"/>
     </x:row>
     <x:row r="4" ht="60" customHeight="1">
       <x:c r="A4" s="12" t="str">
@@ -4275,8 +6917,18 @@
       <x:c r="F4" s="12" t="str">
         <x:v>Fragmented family records show what survives, not everything that happened. The two 1920s papers remain unordered within that decade, and the gap before rediscovery cannot establish an inheritance chain.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="5" ht="60" customHeight="1">
+      <x:c r="G4" s="12" t="str"/>
+      <x:c r="H4" s="12" t="str"/>
+      <x:c r="I4" s="12" t="str"/>
+      <x:c r="J4" s="12" t="str"/>
+      <x:c r="K4" s="13" t="str"/>
+      <x:c r="L4" s="13" t="str"/>
+      <x:c r="M4" s="12" t="str"/>
+      <x:c r="N4" s="12" t="str"/>
+      <x:c r="O4" s="12" t="str"/>
+      <x:c r="P4" s="12" t="str"/>
+    </x:row>
+    <x:row r="5" ht="92" customHeight="1">
       <x:c r="A5" s="12" t="str">
         <x:v>deep_time_evidence</x:v>
       </x:c>
@@ -4294,6 +6946,36 @@
       </x:c>
       <x:c r="F5" s="12" t="str">
         <x:v>Millions of years reveal evolution, dispersal and environmental change rather than a single owner’s story. The late intervals overlap: this order compares their beginnings and does not imply that every region changed at once.</x:v>
+      </x:c>
+      <x:c r="G5" s="12" t="str">
+        <x:v>Ivory Through Time</x:v>
+      </x:c>
+      <x:c r="H5" s="12" t="str">
+        <x:v>Proboscidean change across deep time</x:v>
+      </x:c>
+      <x:c r="I5" s="12" t="str">
+        <x:v>How do changing environments and human relationships reshape the meaning of ivory as a material?</x:v>
+      </x:c>
+      <x:c r="J5" s="12" t="str">
+        <x:v>Place each period, then use the expanding scale to consider the ecological and social changes that make ivory possible.</x:v>
+      </x:c>
+      <x:c r="K5" s="13" t="n">
+        <x:v>-60000000</x:v>
+      </x:c>
+      <x:c r="L5" s="13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M5" s="12" t="str">
+        <x:v>guided</x:v>
+      </x:c>
+      <x:c r="N5" s="12" t="str">
+        <x:v>{"segments":[{"start":-60000000,"end":-2600000,"weight":0.72},{"start":-2600000,"end":0,"weight":0.28}]}</x:v>
+      </x:c>
+      <x:c r="O5" s="12" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="P5" s="12" t="str">
+        <x:v>With the full scale visible, return to the question: whose lives and environments made each later use of ivory possible?</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="32" customHeight="1">
@@ -4303,6 +6985,16 @@
       <x:c r="D6" s="12"/>
       <x:c r="E6" s="12"/>
       <x:c r="F6" s="12"/>
+      <x:c r="G6" s="12"/>
+      <x:c r="H6" s="12"/>
+      <x:c r="I6" s="12"/>
+      <x:c r="J6" s="12"/>
+      <x:c r="K6" s="13"/>
+      <x:c r="L6" s="13"/>
+      <x:c r="M6" s="12"/>
+      <x:c r="N6" s="12"/>
+      <x:c r="O6" s="12"/>
+      <x:c r="P6" s="12"/>
     </x:row>
     <x:row r="7" ht="32" customHeight="1">
       <x:c r="A7" s="12"/>
@@ -4311,6 +7003,16 @@
       <x:c r="D7" s="12"/>
       <x:c r="E7" s="12"/>
       <x:c r="F7" s="12"/>
+      <x:c r="G7" s="12"/>
+      <x:c r="H7" s="12"/>
+      <x:c r="I7" s="12"/>
+      <x:c r="J7" s="12"/>
+      <x:c r="K7" s="13"/>
+      <x:c r="L7" s="13"/>
+      <x:c r="M7" s="12"/>
+      <x:c r="N7" s="12"/>
+      <x:c r="O7" s="12"/>
+      <x:c r="P7" s="12"/>
     </x:row>
     <x:row r="8" ht="32" customHeight="1">
       <x:c r="A8" s="12"/>
@@ -4319,6 +7021,16 @@
       <x:c r="D8" s="12"/>
       <x:c r="E8" s="12"/>
       <x:c r="F8" s="12"/>
+      <x:c r="G8" s="12"/>
+      <x:c r="H8" s="12"/>
+      <x:c r="I8" s="12"/>
+      <x:c r="J8" s="12"/>
+      <x:c r="K8" s="13"/>
+      <x:c r="L8" s="13"/>
+      <x:c r="M8" s="12"/>
+      <x:c r="N8" s="12"/>
+      <x:c r="O8" s="12"/>
+      <x:c r="P8" s="12"/>
     </x:row>
     <x:row r="9" ht="32" customHeight="1">
       <x:c r="A9" s="12"/>
@@ -4327,6 +7039,16 @@
       <x:c r="D9" s="12"/>
       <x:c r="E9" s="12"/>
       <x:c r="F9" s="12"/>
+      <x:c r="G9" s="12"/>
+      <x:c r="H9" s="12"/>
+      <x:c r="I9" s="12"/>
+      <x:c r="J9" s="12"/>
+      <x:c r="K9" s="13"/>
+      <x:c r="L9" s="13"/>
+      <x:c r="M9" s="12"/>
+      <x:c r="N9" s="12"/>
+      <x:c r="O9" s="12"/>
+      <x:c r="P9" s="12"/>
     </x:row>
     <x:row r="10" ht="32" customHeight="1">
       <x:c r="A10" s="12"/>
@@ -4335,6 +7057,16 @@
       <x:c r="D10" s="12"/>
       <x:c r="E10" s="12"/>
       <x:c r="F10" s="12"/>
+      <x:c r="G10" s="12"/>
+      <x:c r="H10" s="12"/>
+      <x:c r="I10" s="12"/>
+      <x:c r="J10" s="12"/>
+      <x:c r="K10" s="13"/>
+      <x:c r="L10" s="13"/>
+      <x:c r="M10" s="12"/>
+      <x:c r="N10" s="12"/>
+      <x:c r="O10" s="12"/>
+      <x:c r="P10" s="12"/>
     </x:row>
     <x:row r="11" ht="32" customHeight="1">
       <x:c r="A11" s="12"/>
@@ -4343,6 +7075,16 @@
       <x:c r="D11" s="12"/>
       <x:c r="E11" s="12"/>
       <x:c r="F11" s="12"/>
+      <x:c r="G11" s="12"/>
+      <x:c r="H11" s="12"/>
+      <x:c r="I11" s="12"/>
+      <x:c r="J11" s="12"/>
+      <x:c r="K11" s="13"/>
+      <x:c r="L11" s="13"/>
+      <x:c r="M11" s="12"/>
+      <x:c r="N11" s="12"/>
+      <x:c r="O11" s="12"/>
+      <x:c r="P11" s="12"/>
     </x:row>
     <x:row r="12" ht="32" customHeight="1">
       <x:c r="A12" s="12"/>
@@ -4351,6 +7093,16 @@
       <x:c r="D12" s="12"/>
       <x:c r="E12" s="12"/>
       <x:c r="F12" s="12"/>
+      <x:c r="G12" s="12"/>
+      <x:c r="H12" s="12"/>
+      <x:c r="I12" s="12"/>
+      <x:c r="J12" s="12"/>
+      <x:c r="K12" s="13"/>
+      <x:c r="L12" s="13"/>
+      <x:c r="M12" s="12"/>
+      <x:c r="N12" s="12"/>
+      <x:c r="O12" s="12"/>
+      <x:c r="P12" s="12"/>
     </x:row>
     <x:row r="13" ht="32" customHeight="1">
       <x:c r="A13" s="12"/>
@@ -4359,6 +7111,16 @@
       <x:c r="D13" s="12"/>
       <x:c r="E13" s="12"/>
       <x:c r="F13" s="12"/>
+      <x:c r="G13" s="12"/>
+      <x:c r="H13" s="12"/>
+      <x:c r="I13" s="12"/>
+      <x:c r="J13" s="12"/>
+      <x:c r="K13" s="13"/>
+      <x:c r="L13" s="13"/>
+      <x:c r="M13" s="12"/>
+      <x:c r="N13" s="12"/>
+      <x:c r="O13" s="12"/>
+      <x:c r="P13" s="12"/>
     </x:row>
     <x:row r="14" ht="32" customHeight="1">
       <x:c r="A14" s="12"/>
@@ -4367,6 +7129,16 @@
       <x:c r="D14" s="12"/>
       <x:c r="E14" s="12"/>
       <x:c r="F14" s="12"/>
+      <x:c r="G14" s="12"/>
+      <x:c r="H14" s="12"/>
+      <x:c r="I14" s="12"/>
+      <x:c r="J14" s="12"/>
+      <x:c r="K14" s="13"/>
+      <x:c r="L14" s="13"/>
+      <x:c r="M14" s="12"/>
+      <x:c r="N14" s="12"/>
+      <x:c r="O14" s="12"/>
+      <x:c r="P14" s="12"/>
     </x:row>
     <x:row r="15" ht="32" customHeight="1">
       <x:c r="A15" s="12"/>
@@ -4375,6 +7147,16 @@
       <x:c r="D15" s="12"/>
       <x:c r="E15" s="12"/>
       <x:c r="F15" s="12"/>
+      <x:c r="G15" s="12"/>
+      <x:c r="H15" s="12"/>
+      <x:c r="I15" s="12"/>
+      <x:c r="J15" s="12"/>
+      <x:c r="K15" s="13"/>
+      <x:c r="L15" s="13"/>
+      <x:c r="M15" s="12"/>
+      <x:c r="N15" s="12"/>
+      <x:c r="O15" s="12"/>
+      <x:c r="P15" s="12"/>
     </x:row>
     <x:row r="16" ht="32" customHeight="1">
       <x:c r="A16" s="12"/>
@@ -4383,6 +7165,16 @@
       <x:c r="D16" s="12"/>
       <x:c r="E16" s="12"/>
       <x:c r="F16" s="12"/>
+      <x:c r="G16" s="12"/>
+      <x:c r="H16" s="12"/>
+      <x:c r="I16" s="12"/>
+      <x:c r="J16" s="12"/>
+      <x:c r="K16" s="13"/>
+      <x:c r="L16" s="13"/>
+      <x:c r="M16" s="12"/>
+      <x:c r="N16" s="12"/>
+      <x:c r="O16" s="12"/>
+      <x:c r="P16" s="12"/>
     </x:row>
     <x:row r="17" ht="32" customHeight="1">
       <x:c r="A17" s="12"/>
@@ -4391,6 +7183,16 @@
       <x:c r="D17" s="12"/>
       <x:c r="E17" s="12"/>
       <x:c r="F17" s="12"/>
+      <x:c r="G17" s="12"/>
+      <x:c r="H17" s="12"/>
+      <x:c r="I17" s="12"/>
+      <x:c r="J17" s="12"/>
+      <x:c r="K17" s="13"/>
+      <x:c r="L17" s="13"/>
+      <x:c r="M17" s="12"/>
+      <x:c r="N17" s="12"/>
+      <x:c r="O17" s="12"/>
+      <x:c r="P17" s="12"/>
     </x:row>
     <x:row r="18" ht="32" customHeight="1">
       <x:c r="A18" s="12"/>
@@ -4399,6 +7201,16 @@
       <x:c r="D18" s="12"/>
       <x:c r="E18" s="12"/>
       <x:c r="F18" s="12"/>
+      <x:c r="G18" s="12"/>
+      <x:c r="H18" s="12"/>
+      <x:c r="I18" s="12"/>
+      <x:c r="J18" s="12"/>
+      <x:c r="K18" s="13"/>
+      <x:c r="L18" s="13"/>
+      <x:c r="M18" s="12"/>
+      <x:c r="N18" s="12"/>
+      <x:c r="O18" s="12"/>
+      <x:c r="P18" s="12"/>
     </x:row>
     <x:row r="19" ht="32" customHeight="1">
       <x:c r="A19" s="12"/>
@@ -4407,6 +7219,16 @@
       <x:c r="D19" s="12"/>
       <x:c r="E19" s="12"/>
       <x:c r="F19" s="12"/>
+      <x:c r="G19" s="12"/>
+      <x:c r="H19" s="12"/>
+      <x:c r="I19" s="12"/>
+      <x:c r="J19" s="12"/>
+      <x:c r="K19" s="13"/>
+      <x:c r="L19" s="13"/>
+      <x:c r="M19" s="12"/>
+      <x:c r="N19" s="12"/>
+      <x:c r="O19" s="12"/>
+      <x:c r="P19" s="12"/>
     </x:row>
     <x:row r="20" ht="32" customHeight="1">
       <x:c r="A20" s="12"/>
@@ -4415,11 +7237,26 @@
       <x:c r="D20" s="12"/>
       <x:c r="E20" s="12"/>
       <x:c r="F20" s="12"/>
+      <x:c r="G20" s="12"/>
+      <x:c r="H20" s="12"/>
+      <x:c r="I20" s="12"/>
+      <x:c r="J20" s="12"/>
+      <x:c r="K20" s="13"/>
+      <x:c r="L20" s="13"/>
+      <x:c r="M20" s="12"/>
+      <x:c r="N20" s="12"/>
+      <x:c r="O20" s="12"/>
+      <x:c r="P20" s="12"/>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="O2:O501">
+      <x:formula1>"true,false"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb080e66598cf433b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Recbdb6cd90804a88"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4699,7 +7536,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc701a1079022438c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea9ce6e4169d4f4f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6313,7 +9150,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R663e447f57e34a87"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f6460e6264d4f39"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6853,7 +9690,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b3b285d709e46e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R631134c8ec0848d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6970,7 +9807,7 @@
         <x:v>Prepared locations</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
-        <x:v>Slots lists all 45 validated access points with a human-readable editor_label, room, capacity, type, physical notes, and anchor reference. Keep IDs, anchors, routes, and assets stable. New physical locations require matching geometry and are outside this workbook workflow.</x:v>
+        <x:v>Slots lists all 47 validated access points with a human-readable editor_label, room, capacity, type, physical notes, and anchor reference. Keep IDs, anchors, routes, and assets stable. New physical locations require matching geometry and are outside this workbook workflow.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="58" customHeight="1">
@@ -7066,7 +9903,7 @@
         <x:v>_data/timeline_events.csv</x:v>
       </x:c>
       <x:c r="B25" s="24" t="str">
-        <x:v>1e783da63ae487794669258fcdc30342bf647796258d2fdd28d134c54f88f722</x:v>
+        <x:v>19c1f01cb9670f6a4a655334f02c9d44855dc5b8de7211e3581e2e2dafeda668</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="58" customHeight="1">
@@ -7074,7 +9911,7 @@
         <x:v>_data/room_timelines.csv</x:v>
       </x:c>
       <x:c r="B26" s="24" t="str">
-        <x:v>24dc2020209d20195d39ff7fd7497d560db9f86e846752d8d3ccbd90c428722c</x:v>
+        <x:v>40056f3e546ffaef9c49a9d9ccdaee40eef4607bcafb6c65a3efd536a610e438</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="58" customHeight="1">
@@ -7104,4 +9941,718 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="32" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="46" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="38" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="32" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="38" customHeight="1">
+      <x:c r="A1" s="28" t="str">
+        <x:v>Add or update visitor-facing exhibit items. Use this view to understand the current content; make website changes in the backend Content and Placements sheets until the guided import workflow is introduced.</x:v>
+      </x:c>
+      <x:c r="B1" t="str"/>
+      <x:c r="C1" t="str"/>
+      <x:c r="D1" t="str"/>
+      <x:c r="E1" t="str"/>
+      <x:c r="F1" t="str"/>
+      <x:c r="G1" t="str"/>
+      <x:c r="H1" t="str"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str"/>
+      <x:c r="B2" t="str"/>
+      <x:c r="C2" t="str"/>
+      <x:c r="D2" t="str"/>
+      <x:c r="E2" t="str"/>
+      <x:c r="F2" t="str"/>
+      <x:c r="G2" t="str"/>
+      <x:c r="H2" t="str"/>
+    </x:row>
+    <x:row r="3" ht="32" customHeight="1">
+      <x:c r="A3" s="31" t="str">
+        <x:v>Room</x:v>
+      </x:c>
+      <x:c r="B3" s="31" t="str">
+        <x:v>Where should it appear?</x:v>
+      </x:c>
+      <x:c r="C3" s="31" t="str">
+        <x:v>Item title</x:v>
+      </x:c>
+      <x:c r="D3" s="31" t="str">
+        <x:v>Description</x:v>
+      </x:c>
+      <x:c r="E3" s="31" t="str">
+        <x:v>Image</x:v>
+      </x:c>
+      <x:c r="F3" s="31" t="str">
+        <x:v>Display type</x:v>
+      </x:c>
+      <x:c r="G3" s="31" t="str">
+        <x:v>Show to visitors?</x:v>
+      </x:c>
+      <x:c r="H3" s="31" t="str">
+        <x:v>Item Name / ID</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="34" customHeight="1">
+      <x:c r="A4" s="35" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="B4" s="35" t="str">
+        <x:v>Gallery introduction</x:v>
+      </x:c>
+      <x:c r="C4" s="35" t="str">
+        <x:v>Gallery Intro</x:v>
+      </x:c>
+      <x:c r="D4" s="35" t="str">
+        <x:v>Featured research: Barberini Ivory, Roman Wall Sconce, and Susanna and the Elders. The illustrated reliefs and fan remain fixed scenery until their identities are confirmed.</x:v>
+      </x:c>
+      <x:c r="E4" s="35" t="str"/>
+      <x:c r="F4" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="G4" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H4" s="35" t="str">
+        <x:v>gallery_intro</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="34" customHeight="1">
+      <x:c r="A5" s="35" t="str">
+        <x:v>conservation_lab</x:v>
+      </x:c>
+      <x:c r="B5" s="35" t="str">
+        <x:v>Conservation Lab introduction</x:v>
+      </x:c>
+      <x:c r="C5" s="35" t="str">
+        <x:v>Conservation Lab Intro</x:v>
+      </x:c>
+      <x:c r="D5" s="35" t="str">
+        <x:v>Ivory as a medium: workmanship, materials, artistic traditions, and conservation evidence. Compare the collection on the central table with histories across centuries.</x:v>
+      </x:c>
+      <x:c r="E5" s="35" t="str"/>
+      <x:c r="F5" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="G5" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H5" s="35" t="str">
+        <x:v>conservation_lab_intro</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="34" customHeight="1">
+      <x:c r="A6" s="35" t="str">
+        <x:v>vestibule</x:v>
+      </x:c>
+      <x:c r="B6" s="35" t="str">
+        <x:v>Welcome and check-in</x:v>
+      </x:c>
+      <x:c r="C6" s="35" t="str">
+        <x:v>Welcome to ArchIvory</x:v>
+      </x:c>
+      <x:c r="D6" s="35" t="str">
+        <x:v>Welcome and check-in.</x:v>
+      </x:c>
+      <x:c r="E6" s="35" t="str"/>
+      <x:c r="F6" s="35" t="str">
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="G6" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H6" s="35" t="str">
+        <x:v>welcome-sequence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="34" customHeight="1">
+      <x:c r="A7" s="35" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="B7" s="35" t="str">
+        <x:v>Near left-wall relief</x:v>
+      </x:c>
+      <x:c r="C7" s="35" t="str">
+        <x:v>Illustrated relief — identity unverified</x:v>
+      </x:c>
+      <x:c r="D7" s="35" t="str">
+        <x:v>This carving is part of the room illustration. Its identity has not been verified against a collection record. The research below is comparative, not a provenance claim.</x:v>
+      </x:c>
+      <x:c r="E7" s="35" t="str"/>
+      <x:c r="F7" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="G7" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H7" s="35" t="str">
+        <x:v>gallery-fixed-wall_01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="34" customHeight="1">
+      <x:c r="A8" s="35" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="B8" s="35" t="str">
+        <x:v>Near left-wall relief</x:v>
+      </x:c>
+      <x:c r="C8" s="35" t="str">
+        <x:v>Susanna and the Elders</x:v>
+      </x:c>
+      <x:c r="D8" s="35" t="str">
+        <x:v>Existing Gallery research on the carving by Van Bossuit.</x:v>
+      </x:c>
+      <x:c r="E8" s="35" t="str"/>
+      <x:c r="F8" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="G8" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H8" s="35" t="str">
+        <x:v>art-susanna-sequence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="34" customHeight="1">
+      <x:c r="A9" s="35" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="B9" s="35" t="str">
+        <x:v>Far left-wall relief</x:v>
+      </x:c>
+      <x:c r="C9" s="35" t="str">
+        <x:v>Illustrated relief — identity unverified</x:v>
+      </x:c>
+      <x:c r="D9" s="35" t="str">
+        <x:v>This carving is part of the room illustration. Its identity has not been verified against a collection record. The research below is comparative, not a provenance claim.</x:v>
+      </x:c>
+      <x:c r="E9" s="35" t="str"/>
+      <x:c r="F9" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="G9" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H9" s="35" t="str">
+        <x:v>gallery-fixed-wall_02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="34" customHeight="1">
+      <x:c r="A10" s="35" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="B10" s="35" t="str">
+        <x:v>Far left-wall relief</x:v>
+      </x:c>
+      <x:c r="C10" s="35" t="str">
+        <x:v>Barberini Ivory</x:v>
+      </x:c>
+      <x:c r="D10" s="35" t="str">
+        <x:v>Existing Gallery research: sixth-century relief.</x:v>
+      </x:c>
+      <x:c r="E10" s="35" t="str"/>
+      <x:c r="F10" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="G10" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H10" s="35" t="str">
+        <x:v>art-relief-sequence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="34" customHeight="1">
+      <x:c r="A11" s="35" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="B11" s="35" t="str">
+        <x:v>Front glass case</x:v>
+      </x:c>
+      <x:c r="C11" s="35" t="str">
+        <x:v>Illustrated folding fan</x:v>
+      </x:c>
+      <x:c r="D11" s="35" t="str">
+        <x:v>The fan is a fixed part of the room artwork. Its identity has not been verified; it is not assigned the New Harmony fan record.</x:v>
+      </x:c>
+      <x:c r="E11" s="35" t="str"/>
+      <x:c r="F11" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="G11" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H11" s="35" t="str">
+        <x:v>gallery-fixed-fan</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="34" customHeight="1">
+      <x:c r="A12" s="35" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="B12" s="35" t="str">
+        <x:v>Small rear-wall frame</x:v>
+      </x:c>
+      <x:c r="C12" s="35" t="str">
+        <x:v>Roman Wall Sconce</x:v>
+      </x:c>
+      <x:c r="D12" s="35" t="str">
+        <x:v>Existing evidence case at the Eskenazi Museum of Art.</x:v>
+      </x:c>
+      <x:c r="E12" s="35" t="str">
+        <x:v>/assets/img/RomanWallSconce - 03-06-2026 14-41-38.jpeg</x:v>
+      </x:c>
+      <x:c r="F12" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="G12" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H12" s="35" t="str">
+        <x:v>gallery-roman-wall-sconce</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="34" customHeight="1">
+      <x:c r="A13" s="35" t="str">
+        <x:v>conservation_lab</x:v>
+      </x:c>
+      <x:c r="B13" s="35" t="str">
+        <x:v>Central ivories collection</x:v>
+      </x:c>
+      <x:c r="C13" s="35" t="str">
+        <x:v>IU Eskenazi Museum Ivories</x:v>
+      </x:c>
+      <x:c r="D13" s="35" t="str">
+        <x:v>Existing conservation-table research.</x:v>
+      </x:c>
+      <x:c r="E13" s="35" t="str"/>
+      <x:c r="F13" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="G13" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H13" s="35" t="str">
+        <x:v>ChineseUVIvoryCollection</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="34" customHeight="1">
+      <x:c r="A14" s="35" t="str">
+        <x:v>conservation_lab</x:v>
+      </x:c>
+      <x:c r="B14" s="35" t="str">
+        <x:v>Ivory Through the Ages</x:v>
+      </x:c>
+      <x:c r="C14" s="35" t="str">
+        <x:v>ivory_ages</x:v>
+      </x:c>
+      <x:c r="D14" s="35" t="str"/>
+      <x:c r="E14" s="35" t="str"/>
+      <x:c r="F14" s="35" t="str">
+        <x:v>timeline</x:v>
+      </x:c>
+      <x:c r="G14" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H14" s="35" t="str">
+        <x:v>ivory_ages</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="34" customHeight="1">
+      <x:c r="A15" s="35" t="str">
+        <x:v>conservation_lab</x:v>
+      </x:c>
+      <x:c r="B15" s="35" t="str">
+        <x:v>Rear analysis workbench</x:v>
+      </x:c>
+      <x:c r="C15" s="35" t="str">
+        <x:v>Analysis workbench</x:v>
+      </x:c>
+      <x:c r="D15" s="35" t="str">
+        <x:v>The existing collection record reports DNA evidence from African and Asian elephants. Open the central ivories collection for the supplied research. No additional analysis media have been supplied.</x:v>
+      </x:c>
+      <x:c r="E15" s="35" t="str"/>
+      <x:c r="F15" s="35" t="str">
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="G15" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H15" s="35" t="str">
+        <x:v>conservation-methods</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="34" customHeight="1">
+      <x:c r="A16" s="35" t="str">
+        <x:v>historical_society</x:v>
+      </x:c>
+      <x:c r="B16" s="35" t="str">
+        <x:v>Local Lives</x:v>
+      </x:c>
+      <x:c r="C16" s="35" t="str">
+        <x:v>local_lives</x:v>
+      </x:c>
+      <x:c r="D16" s="35" t="str"/>
+      <x:c r="E16" s="35" t="str"/>
+      <x:c r="F16" s="35" t="str">
+        <x:v>timeline</x:v>
+      </x:c>
+      <x:c r="G16" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H16" s="35" t="str">
+        <x:v>local_lives</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="34" customHeight="1">
+      <x:c r="A17" s="35" t="str">
+        <x:v>historical_society</x:v>
+      </x:c>
+      <x:c r="B17" s="35" t="str">
+        <x:v>Piano</x:v>
+      </x:c>
+      <x:c r="C17" s="35" t="str">
+        <x:v>Piano</x:v>
+      </x:c>
+      <x:c r="D17" s="35" t="str">
+        <x:v>An illustrated piano anchors this room. Keyboard coverings can prompt questions about materials and manufacture, but the artwork does not establish the material, maker or provenance of this piano.</x:v>
+      </x:c>
+      <x:c r="E17" s="35" t="str"/>
+      <x:c r="F17" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="G17" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H17" s="35" t="str">
+        <x:v>historical_society_piano_01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="34" customHeight="1">
+      <x:c r="A18" s="35" t="str">
+        <x:v>historical_society</x:v>
+      </x:c>
+      <x:c r="B18" s="35" t="str">
+        <x:v>Billiards table</x:v>
+      </x:c>
+      <x:c r="C18" s="35" t="str">
+        <x:v>Billiards table</x:v>
+      </x:c>
+      <x:c r="D18" s="35" t="str">
+        <x:v>The billiards table connects leisure with the history of materials. No object record or material identification has been assigned to this illustrated furnishing.</x:v>
+      </x:c>
+      <x:c r="E18" s="35" t="str"/>
+      <x:c r="F18" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="G18" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H18" s="35" t="str">
+        <x:v>historical_society_table_01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="34" customHeight="1">
+      <x:c r="A19" s="35" t="str">
+        <x:v>attic</x:v>
+      </x:c>
+      <x:c r="B19" s="35" t="str">
+        <x:v>Family Traces</x:v>
+      </x:c>
+      <x:c r="C19" s="35" t="str">
+        <x:v>family_traces</x:v>
+      </x:c>
+      <x:c r="D19" s="35" t="str"/>
+      <x:c r="E19" s="35" t="str"/>
+      <x:c r="F19" s="35" t="str">
+        <x:v>timeline</x:v>
+      </x:c>
+      <x:c r="G19" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H19" s="35" t="str">
+        <x:v>family_traces</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="34" customHeight="1">
+      <x:c r="A20" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B20" s="35" t="str">
+        <x:v>Tusk specimen</x:v>
+      </x:c>
+      <x:c r="C20" s="35" t="str">
+        <x:v>Elephant tusk</x:v>
+      </x:c>
+      <x:c r="D20" s="35" t="str">
+        <x:v>The room illustration presents a tusk as a specimen. A specimen accession, individual animal, collecting locality and provenance have not been supplied. Use the inquiry terminal for evidence-based questions; do not infer an individual history from the scenery.</x:v>
+      </x:c>
+      <x:c r="E20" s="35" t="str"/>
+      <x:c r="F20" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="G20" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H20" s="35" t="str">
+        <x:v>natural-history-specimen</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="34" customHeight="1">
+      <x:c r="A21" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B21" s="35" t="str">
+        <x:v>Specimen label</x:v>
+      </x:c>
+      <x:c r="C21" s="35" t="str">
+        <x:v>Elephant tusk</x:v>
+      </x:c>
+      <x:c r="D21" s="35" t="str">
+        <x:v>The room illustration presents a tusk as a specimen. A specimen accession, individual animal, collecting locality and provenance have not been supplied. Use the inquiry terminal for evidence-based questions; do not infer an individual history from the scenery.</x:v>
+      </x:c>
+      <x:c r="E21" s="35" t="str"/>
+      <x:c r="F21" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="G21" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H21" s="35" t="str">
+        <x:v>natural-history-specimen</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="34" customHeight="1">
+      <x:c r="A22" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B22" s="35" t="str">
+        <x:v>Elephant interpretation panel</x:v>
+      </x:c>
+      <x:c r="C22" s="35" t="str">
+        <x:v>Natural History Intro</x:v>
+      </x:c>
+      <x:c r="D22" s="35" t="str">
+        <x:v>Elephants, ivory as material, and environmental history. Explore deep time, maps, specimen interpretation, and a separate evidence-ordering activity.</x:v>
+      </x:c>
+      <x:c r="E22" s="35" t="str"/>
+      <x:c r="F22" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="G22" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H22" s="35" t="str">
+        <x:v>natural_history_intro</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="34" customHeight="1">
+      <x:c r="A23" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B23" s="35" t="str">
+        <x:v>Wall map</x:v>
+      </x:c>
+      <x:c r="C23" s="35" t="str">
+        <x:v>World map</x:v>
+      </x:c>
+      <x:c r="D23" s="35" t="str">
+        <x:v>Existing collection geography map.</x:v>
+      </x:c>
+      <x:c r="E23" s="35" t="str"/>
+      <x:c r="F23" s="35" t="str">
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="G23" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H23" s="35" t="str">
+        <x:v>natural-history-map</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="34" customHeight="1">
+      <x:c r="A24" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B24" s="35" t="str">
+        <x:v>Ivory Through Time poster</x:v>
+      </x:c>
+      <x:c r="C24" s="35" t="str">
+        <x:v>deep_time_evidence</x:v>
+      </x:c>
+      <x:c r="D24" s="35" t="str"/>
+      <x:c r="E24" s="35" t="str"/>
+      <x:c r="F24" s="35" t="str">
+        <x:v>timeline</x:v>
+      </x:c>
+      <x:c r="G24" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H24" s="35" t="str">
+        <x:v>deep_time_evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="34" customHeight="1">
+      <x:c r="A25" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B25" s="35" t="str">
+        <x:v>Habitation map within explorer</x:v>
+      </x:c>
+      <x:c r="C25" s="35" t="str">
+        <x:v>Habitation map</x:v>
+      </x:c>
+      <x:c r="D25" s="35" t="str">
+        <x:v>Nested component of the deep-time explorer, not a second wall location.</x:v>
+      </x:c>
+      <x:c r="E25" s="35" t="str"/>
+      <x:c r="F25" s="35" t="str">
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="G25" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H25" s="35" t="str">
+        <x:v>habitation-map</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="34" customHeight="1">
+      <x:c r="A26" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B26" s="35" t="str">
+        <x:v>Ivory inquiry</x:v>
+      </x:c>
+      <x:c r="C26" s="35" t="str">
+        <x:v>Ivory Inquiry Terminal</x:v>
+      </x:c>
+      <x:c r="D26" s="35" t="str">
+        <x:v>Existing inquiry tool.</x:v>
+      </x:c>
+      <x:c r="E26" s="35" t="str"/>
+      <x:c r="F26" s="35" t="str">
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="G26" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H26" s="35" t="str">
+        <x:v>natural-history-tusk</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="34" customHeight="1">
+      <x:c r="A27" s="35" t="str">
+        <x:v>conservators_office</x:v>
+      </x:c>
+      <x:c r="B27" s="35" t="str">
+        <x:v>Desk terminal</x:v>
+      </x:c>
+      <x:c r="C27" s="35" t="str">
+        <x:v>Curation terminal</x:v>
+      </x:c>
+      <x:c r="D27" s="35" t="str">
+        <x:v>Exhibition assembly remains a planned feature.</x:v>
+      </x:c>
+      <x:c r="E27" s="35" t="str"/>
+      <x:c r="F27" s="35" t="str">
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="G27" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H27" s="35" t="str">
+        <x:v>conservator-terminal</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="34" customHeight="1">
+      <x:c r="A28" s="35" t="str">
+        <x:v>conservators_office</x:v>
+      </x:c>
+      <x:c r="B28" s="35" t="str">
+        <x:v>Elephant wall panel</x:v>
+      </x:c>
+      <x:c r="C28" s="35" t="str">
+        <x:v>Conservators Office Intro</x:v>
+      </x:c>
+      <x:c r="D28" s="35" t="str">
+        <x:v>Care, repair, research and preservation. Exhibition assembly at the terminal remains a future feature.</x:v>
+      </x:c>
+      <x:c r="E28" s="35" t="str"/>
+      <x:c r="F28" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="G28" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H28" s="35" t="str">
+        <x:v>conservators_office_intro</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="34" customHeight="1">
+      <x:c r="A29" s="35" t="str">
+        <x:v>lab</x:v>
+      </x:c>
+      <x:c r="B29" s="35" t="str">
+        <x:v>Attic access context</x:v>
+      </x:c>
+      <x:c r="C29" s="35" t="str">
+        <x:v>Attic investigations</x:v>
+      </x:c>
+      <x:c r="D29" s="35" t="str">
+        <x:v>Existing context and navigation.</x:v>
+      </x:c>
+      <x:c r="E29" s="35" t="str"/>
+      <x:c r="F29" s="35" t="str">
+        <x:v>tool</x:v>
+      </x:c>
+      <x:c r="G29" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H29" s="35" t="str">
+        <x:v>lab-attic-sequence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="34" customHeight="1">
+      <x:c r="A30" s="35" t="str">
+        <x:v>natural_history</x:v>
+      </x:c>
+      <x:c r="B30" s="35" t="str">
+        <x:v>Central recessed panel</x:v>
+      </x:c>
+      <x:c r="C30" s="35" t="str">
+        <x:v>Geib Flute</x:v>
+      </x:c>
+      <x:c r="D30" s="35" t="str">
+        <x:v>test</x:v>
+      </x:c>
+      <x:c r="E30" s="35" t="str">
+        <x:v>/assets/img/editorial/geib-flute-3ec90b3a3ce8.jpeg</x:v>
+      </x:c>
+      <x:c r="F30" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="G30" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H30" s="35" t="str">
+        <x:v>geib-flute</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Validate linear interpretive timeline in Conservation Lab
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/archivory-editorial/ArchIvory Editorial Workbook.xlsx
+++ b/outputs/archivory-editorial/ArchIvory Editorial Workbook.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Placements" sheetId="1" r:id="R0cf6673335704b3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content" sheetId="2" r:id="R1ba60e2bb612419a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="3" r:id="Rf83177706bc24d9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timelines" sheetId="4" r:id="Re33f1023b6364a91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rooms" sheetId="5" r:id="Rbd5db61eaa964efc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slots" sheetId="6" r:id="R20d23e67ab7d40d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection" sheetId="7" r:id="R7c1592b892834ca5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="Re4288a1cbadb4731"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edit Items" sheetId="9" r:id="Rb1c922022850484c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline Cards" sheetId="10" r:id="Rc28f0ab5e3bb42d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Room Overview" sheetId="11" r:id="R66b6e898cc664bbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing" sheetId="12" r:id="R12462e242c344dea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Placements" sheetId="1" r:id="Rb7457834bf56470f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content" sheetId="2" r:id="Rc74e5745fa4046ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="3" r:id="Rac68e6233d214a9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timelines" sheetId="4" r:id="R7edc30122bae4e82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rooms" sheetId="5" r:id="R48f2d5cede0c4cf1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slots" sheetId="6" r:id="R1e0d496664ab4e24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection" sheetId="7" r:id="Rd6c86cf7719f46f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="Ra0c51869802f4cbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edit Items" sheetId="9" r:id="R974be6918df74d5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline Cards" sheetId="10" r:id="R241f856729ad4a18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Room Overview" sheetId="11" r:id="Re14e39a493f54d45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing" sheetId="12" r:id="R8b339fa1a0294653"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2918,7 +2918,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45d9315a020e4989"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e1ff5259eee462e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3070,7 +3070,7 @@
         <x:v>conservation_lab</x:v>
       </x:c>
       <x:c r="B8" s="35" t="str">
-        <x:v>Conservation Lab</x:v>
+        <x:v>Ivory Through the Ages</x:v>
       </x:c>
       <x:c r="C8" s="35" t="str">
         <x:v>Early carved sample</x:v>
@@ -3078,8 +3078,12 @@
       <x:c r="D8" s="35" t="str">
         <x:v>2000 BCE (fictional sample)</x:v>
       </x:c>
-      <x:c r="E8" s="35" t="str"/>
-      <x:c r="F8" s="35" t="str"/>
+      <x:c r="E8" s="35" t="str">
+        <x:v>The earliest sample sits at the beginning of a long BCE-to-CE interval, making later workshop changes visibly closer together.</x:v>
+      </x:c>
+      <x:c r="F8" s="35" t="str">
+        <x:v>What changes when centuries of material practice are shown on one continuous scale?</x:v>
+      </x:c>
       <x:c r="G8" s="35" t="str"/>
       <x:c r="H8" s="35" t="str">
         <x:v>Yes</x:v>
@@ -3090,7 +3094,7 @@
         <x:v>conservation_lab</x:v>
       </x:c>
       <x:c r="B9" s="35" t="str">
-        <x:v>Conservation Lab</x:v>
+        <x:v>Ivory Through the Ages</x:v>
       </x:c>
       <x:c r="C9" s="35" t="str">
         <x:v>Relief workshop sample</x:v>
@@ -3098,8 +3102,12 @@
       <x:c r="D9" s="35" t="str">
         <x:v>500 CE (fictional sample)</x:v>
       </x:c>
-      <x:c r="E9" s="35" t="str"/>
-      <x:c r="F9" s="35" t="str"/>
+      <x:c r="E9" s="35" t="str">
+        <x:v>The move into the CE range is represented by a positive chronology value while the visitor-facing label remains historical rather than technical.</x:v>
+      </x:c>
+      <x:c r="F9" s="35" t="str">
+        <x:v>How can a shared material carry different meanings in different workshop settings?</x:v>
+      </x:c>
       <x:c r="G9" s="35" t="str"/>
       <x:c r="H9" s="35" t="str">
         <x:v>Yes</x:v>
@@ -3110,7 +3118,7 @@
         <x:v>conservation_lab</x:v>
       </x:c>
       <x:c r="B10" s="35" t="str">
-        <x:v>Conservation Lab</x:v>
+        <x:v>Ivory Through the Ages</x:v>
       </x:c>
       <x:c r="C10" s="35" t="str">
         <x:v>Joined-panel sample</x:v>
@@ -3118,8 +3126,12 @@
       <x:c r="D10" s="35" t="str">
         <x:v>1200 CE (fictional sample)</x:v>
       </x:c>
-      <x:c r="E10" s="35" t="str"/>
-      <x:c r="F10" s="35" t="str"/>
+      <x:c r="E10" s="35" t="str">
+        <x:v>This later sample is separated from 500 CE by far less time than the BCE-to-CE span at the start of the activity.</x:v>
+      </x:c>
+      <x:c r="F10" s="35" t="str">
+        <x:v>What might a proportional gap reveal that an equally spaced list would hide?</x:v>
+      </x:c>
       <x:c r="G10" s="35" t="str"/>
       <x:c r="H10" s="35" t="str">
         <x:v>Yes</x:v>
@@ -3130,7 +3142,7 @@
         <x:v>conservation_lab</x:v>
       </x:c>
       <x:c r="B11" s="35" t="str">
-        <x:v>Conservation Lab</x:v>
+        <x:v>Ivory Through the Ages</x:v>
       </x:c>
       <x:c r="C11" s="35" t="str">
         <x:v>Turned-object sample</x:v>
@@ -3138,8 +3150,12 @@
       <x:c r="D11" s="35" t="str">
         <x:v>1800 CE (fictional sample)</x:v>
       </x:c>
-      <x:c r="E11" s="35" t="str"/>
-      <x:c r="F11" s="35" t="str"/>
+      <x:c r="E11" s="35" t="str">
+        <x:v>The final card anchors the end of the linear scale and makes the relative distances among the four teaching samples visible.</x:v>
+      </x:c>
+      <x:c r="F11" s="35" t="str">
+        <x:v>When does a new technique change the social meaning of a material?</x:v>
+      </x:c>
       <x:c r="G11" s="35" t="str"/>
       <x:c r="H11" s="35" t="str">
         <x:v>Yes</x:v>
@@ -3676,7 +3692,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="F18" s="35" t="str">
-        <x:v>ivory_ages</x:v>
+        <x:v>Ivory Through the Ages</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="34" customHeight="1">
@@ -4585,7 +4601,7 @@
         <x:v>Ivory Through the Ages</x:v>
       </x:c>
       <x:c r="C14" s="35" t="str">
-        <x:v>ivory_ages</x:v>
+        <x:v>Ivory Through the Ages</x:v>
       </x:c>
       <x:c r="D14" s="35" t="str">
         <x:v>timeline</x:v>
@@ -5975,7 +5991,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re25c2d70ea974e2c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2da99640916b4759"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6156,7 +6172,7 @@
       <x:c r="K5" s="12" t="str"/>
       <x:c r="L5" s="12" t="str"/>
     </x:row>
-    <x:row r="6" ht="44" customHeight="1">
+    <x:row r="6" ht="92" customHeight="1">
       <x:c r="A6" s="12" t="str">
         <x:v>ivory_ages</x:v>
       </x:c>
@@ -6182,11 +6198,17 @@
       <x:c r="I6" s="12" t="str">
         <x:v>A teaching sample introduces carving as a material practice.</x:v>
       </x:c>
-      <x:c r="J6" s="12" t="str"/>
-      <x:c r="K6" s="12" t="str"/>
-      <x:c r="L6" s="12" t="str"/>
-    </x:row>
-    <x:row r="7" ht="44" customHeight="1">
+      <x:c r="J6" s="12" t="str">
+        <x:v>The earliest sample sits at the beginning of a long BCE-to-CE interval, making later workshop changes visibly closer together.</x:v>
+      </x:c>
+      <x:c r="K6" s="12" t="str">
+        <x:v>What changes when centuries of material practice are shown on one continuous scale?</x:v>
+      </x:c>
+      <x:c r="L6" s="12" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="108" customHeight="1">
       <x:c r="A7" s="12" t="str">
         <x:v>ivory_ages</x:v>
       </x:c>
@@ -6212,11 +6234,17 @@
       <x:c r="I7" s="12" t="str">
         <x:v>A later teaching sample explores relief technique.</x:v>
       </x:c>
-      <x:c r="J7" s="12" t="str"/>
-      <x:c r="K7" s="12" t="str"/>
-      <x:c r="L7" s="12" t="str"/>
-    </x:row>
-    <x:row r="8" ht="44" customHeight="1">
+      <x:c r="J7" s="12" t="str">
+        <x:v>The move into the CE range is represented by a positive chronology value while the visitor-facing label remains historical rather than technical.</x:v>
+      </x:c>
+      <x:c r="K7" s="12" t="str">
+        <x:v>How can a shared material carry different meanings in different workshop settings?</x:v>
+      </x:c>
+      <x:c r="L7" s="12" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="92" customHeight="1">
       <x:c r="A8" s="12" t="str">
         <x:v>ivory_ages</x:v>
       </x:c>
@@ -6242,11 +6270,17 @@
       <x:c r="I8" s="12" t="str">
         <x:v>A teaching sample asks how construction and display relate.</x:v>
       </x:c>
-      <x:c r="J8" s="12" t="str"/>
-      <x:c r="K8" s="12" t="str"/>
-      <x:c r="L8" s="12" t="str"/>
-    </x:row>
-    <x:row r="9" ht="44" customHeight="1">
+      <x:c r="J8" s="12" t="str">
+        <x:v>This later sample is separated from 500 CE by far less time than the BCE-to-CE span at the start of the activity.</x:v>
+      </x:c>
+      <x:c r="K8" s="12" t="str">
+        <x:v>What might a proportional gap reveal that an equally spaced list would hide?</x:v>
+      </x:c>
+      <x:c r="L8" s="12" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="92" customHeight="1">
       <x:c r="A9" s="12" t="str">
         <x:v>ivory_ages</x:v>
       </x:c>
@@ -6272,9 +6306,15 @@
       <x:c r="I9" s="12" t="str">
         <x:v>A teaching sample introduces another way to work the material.</x:v>
       </x:c>
-      <x:c r="J9" s="12" t="str"/>
-      <x:c r="K9" s="12" t="str"/>
-      <x:c r="L9" s="12" t="str"/>
+      <x:c r="J9" s="12" t="str">
+        <x:v>The final card anchors the end of the linear scale and makes the relative distances among the four teaching samples visible.</x:v>
+      </x:c>
+      <x:c r="K9" s="12" t="str">
+        <x:v>When does a new technique change the social meaning of a material?</x:v>
+      </x:c>
+      <x:c r="L9" s="12" t="str">
+        <x:v>true</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="44" customHeight="1">
       <x:c r="A10" s="12" t="str">
@@ -6761,7 +6801,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb93538e37f484e7f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64d5735699984ca9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6868,7 +6908,7 @@
       <x:c r="O2" s="12" t="str"/>
       <x:c r="P2" s="12" t="str"/>
     </x:row>
-    <x:row r="3" ht="60" customHeight="1">
+    <x:row r="3" ht="124" customHeight="1">
       <x:c r="A3" s="12" t="str">
         <x:v>ivory_ages</x:v>
       </x:c>
@@ -6887,16 +6927,34 @@
       <x:c r="F3" s="12" t="str">
         <x:v>Across centuries and millennia, related materials can support changing techniques and meanings. A broad period comparison reveals artistic traditions, while obscuring the individual transfers visible at a shorter scale.</x:v>
       </x:c>
-      <x:c r="G3" s="12" t="str"/>
-      <x:c r="H3" s="12" t="str"/>
-      <x:c r="I3" s="12" t="str"/>
-      <x:c r="J3" s="12" t="str"/>
-      <x:c r="K3" s="13" t="str"/>
-      <x:c r="L3" s="13" t="str"/>
-      <x:c r="M3" s="12" t="str"/>
+      <x:c r="G3" s="12" t="str">
+        <x:v>Ivory Through the Ages</x:v>
+      </x:c>
+      <x:c r="H3" s="12" t="str">
+        <x:v>Material practice across BCE and CE</x:v>
+      </x:c>
+      <x:c r="I3" s="12" t="str">
+        <x:v>How do changes in technique and display alter what ivory means across time?</x:v>
+      </x:c>
+      <x:c r="J3" s="12" t="str">
+        <x:v>Place the teaching samples on a continuous BCE-to-CE scale, then consider how material practice changes without assigning these histories to the illustrated room objects.</x:v>
+      </x:c>
+      <x:c r="K3" s="13" t="n">
+        <x:v>-2000</x:v>
+      </x:c>
+      <x:c r="L3" s="13" t="n">
+        <x:v>1800</x:v>
+      </x:c>
+      <x:c r="M3" s="12" t="str">
+        <x:v>linear</x:v>
+      </x:c>
       <x:c r="N3" s="12" t="str"/>
-      <x:c r="O3" s="12" t="str"/>
-      <x:c r="P3" s="12" t="str"/>
+      <x:c r="O3" s="12" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="P3" s="12" t="str">
+        <x:v>With the full scale visible, compare the long early interval with the later changes in workshop practice and display.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="60" customHeight="1">
       <x:c r="A4" s="12" t="str">
@@ -7256,7 +7314,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Recbdb6cd90804a88"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re146a52e7f424505"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7536,7 +7594,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea9ce6e4169d4f4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60d754df694f40a2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9150,7 +9208,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f6460e6264d4f39"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a08c94a148f485c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9690,7 +9748,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R631134c8ec0848d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reaed199754c84b3e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9903,7 +9961,7 @@
         <x:v>_data/timeline_events.csv</x:v>
       </x:c>
       <x:c r="B25" s="24" t="str">
-        <x:v>19c1f01cb9670f6a4a655334f02c9d44855dc5b8de7211e3581e2e2dafeda668</x:v>
+        <x:v>5d876d5c0dd733dea511a8025f7035cfb8c0c4c273daba531a7a87adbfce0a56</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="58" customHeight="1">
@@ -9911,7 +9969,7 @@
         <x:v>_data/room_timelines.csv</x:v>
       </x:c>
       <x:c r="B26" s="24" t="str">
-        <x:v>40056f3e546ffaef9c49a9d9ccdaee40eef4607bcafb6c65a3efd536a610e438</x:v>
+        <x:v>ba0aaf6126b0af0863e001f0dcdd4d66c0bb5ccfa0bdb44d6797024130fea539</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="58" customHeight="1">

</xml_diff>

<commit_message>
Add visual room access-point authoring
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/archivory-editorial/ArchIvory Editorial Workbook.xlsx
+++ b/outputs/archivory-editorial/ArchIvory Editorial Workbook.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Placements" sheetId="1" r:id="Rb7457834bf56470f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content" sheetId="2" r:id="Rc74e5745fa4046ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="3" r:id="Rac68e6233d214a9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timelines" sheetId="4" r:id="R7edc30122bae4e82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rooms" sheetId="5" r:id="R48f2d5cede0c4cf1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slots" sheetId="6" r:id="R1e0d496664ab4e24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection" sheetId="7" r:id="Rd6c86cf7719f46f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="Ra0c51869802f4cbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edit Items" sheetId="9" r:id="R974be6918df74d5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline Cards" sheetId="10" r:id="R241f856729ad4a18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Room Overview" sheetId="11" r:id="Re14e39a493f54d45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing" sheetId="12" r:id="R8b339fa1a0294653"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Placements" sheetId="1" r:id="Rce635eccc2294b74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content" sheetId="2" r:id="Ree1a7c86f3c145b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="3" r:id="R6e09b83a1bd74e83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timelines" sheetId="4" r:id="Rec883b2a242145f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rooms" sheetId="5" r:id="R1c24cd4245084470"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slots" sheetId="6" r:id="R9c3dcad3cdbe4404"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection" sheetId="7" r:id="Re9799fc4f9fe494a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="R441e68790cab4e1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edit Items" sheetId="9" r:id="R9bcae7e9267d425b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline Cards" sheetId="10" r:id="R525c412c544e4a0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Room Overview" sheetId="11" r:id="Re4747086bdf34ed6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing" sheetId="12" r:id="R9e447ab9dc764292"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -235,7 +235,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PlacementsTable" displayName="PlacementsTable" ref="A1:K65" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PlacementsTable" displayName="PlacementsTable" ref="A1:K66" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="placement_id"/>
     <x:tableColumn id="2" name="slot_id"/>
@@ -326,7 +326,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="SlotsTable" displayName="SlotsTable" ref="A1:J63" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="SlotsTable" displayName="SlotsTable" ref="A1:J64" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="slot_id"/>
     <x:tableColumn id="2" name="room_id"/>
@@ -2536,27 +2536,42 @@
         <x:v>8</x:v>
       </x:c>
     </x:row>
-    <x:row r="51" ht="32" customHeight="1">
-      <x:c r="A51" s="12"/>
-      <x:c r="B51" s="12"/>
-      <x:c r="C51" s="12"/>
-      <x:c r="D51" s="12"/>
-      <x:c r="E51" s="13"/>
-      <x:c r="F51" s="12"/>
+    <x:row r="51" ht="34" customHeight="1">
+      <x:c r="A51" s="12" t="str">
+        <x:v>draft_gallery_detail_01</x:v>
+      </x:c>
+      <x:c r="B51" s="12" t="str">
+        <x:v>gallery_detail_01</x:v>
+      </x:c>
+      <x:c r="C51" s="12" t="str"/>
+      <x:c r="D51" s="12" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E51" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F51" s="12" t="str">
+        <x:v>false</x:v>
+      </x:c>
       <x:c r="G51" s="15" t="str">
         <x:f>IF(B51="","",IFERROR(VLOOKUP(B51,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+        <x:v>gallery</x:v>
       </x:c>
       <x:c r="H51" s="15" t="str">
         <x:f>IF(G51="","",IFERROR(VLOOKUP(G51,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+        <x:v>Gallery</x:v>
       </x:c>
       <x:c r="I51" s="15" t="str">
         <x:f>IF(B51="","",IFERROR(VLOOKUP(B51,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+        <x:v>New access point</x:v>
       </x:c>
       <x:c r="J51" s="15" t="str">
         <x:f>IF(B51="","",IFERROR(VLOOKUP(B51,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
-      </x:c>
-      <x:c r="K51" s="15" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="K51" s="15" t="n">
         <x:f>IF(B51="","",IFERROR(VLOOKUP(B51,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="32" customHeight="1">
@@ -2881,23 +2896,46 @@
         <x:f>IF(B65="","",IFERROR(VLOOKUP(B65,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
       </x:c>
     </x:row>
+    <x:row r="66" ht="32" customHeight="1">
+      <x:c r="A66" s="12"/>
+      <x:c r="B66" s="12"/>
+      <x:c r="C66" s="12"/>
+      <x:c r="D66" s="12"/>
+      <x:c r="E66" s="13"/>
+      <x:c r="F66" s="12"/>
+      <x:c r="G66" s="15" t="str">
+        <x:f>IF(B66="","",IFERROR(VLOOKUP(B66,Slots!$A$2:$D$501,2,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="H66" s="15" t="str">
+        <x:f>IF(G66="","",IFERROR(VLOOKUP(G66,Rooms!$A$2:$B$501,2,FALSE),"Unknown room"))</x:f>
+      </x:c>
+      <x:c r="I66" s="15" t="str">
+        <x:f>IF(B66="","",IFERROR(VLOOKUP(B66,Slots!$A$2:$D$501,4,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="J66" s="15" t="str">
+        <x:f>IF(B66="","",IFERROR(VLOOKUP(B66,Slots!$A$2:$E$501,5,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+      <x:c r="K66" s="15" t="str">
+        <x:f>IF(B66="","",IFERROR(VLOOKUP(B66,Slots!$A$2:$F$501,6,FALSE),"Unknown slot"))</x:f>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="C2:C65">
+  <x:conditionalFormatting sqref="C2:C66">
     <x:cfRule type="expression" dxfId="0" priority="1">
       <x:formula>AND($A2&lt;&gt;"",$C2="")</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="B2:B65">
+  <x:conditionalFormatting sqref="B2:B66">
     <x:cfRule type="expression" dxfId="1" priority="2">
       <x:formula>AND($A2&lt;&gt;"",$B2&lt;&gt;"",COUNTIF(Slots!$A$2:$A$501,$B2)=0)</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="F2:F65">
+  <x:conditionalFormatting sqref="F2:F66">
     <x:cfRule type="expression" dxfId="2" priority="3">
       <x:formula>AND($A2&lt;&gt;"",$F2="true",COUNTIFS($B$2:$B$501,$B2,$E$2:$E$501,$E2,$F$2:$F$501,"true")&gt;1)</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="E2:E65">
+  <x:conditionalFormatting sqref="E2:E66">
     <x:cfRule type="expression" dxfId="3" priority="4">
       <x:formula>AND($A2&lt;&gt;"",$F2="true",$E2&lt;&gt;"",COUNTIFS($B$2:$B$501,$B2,$E$2:$E$501,$E2,$F$2:$F$501,"true")&gt;1)</x:formula>
     </x:cfRule>
@@ -2918,7 +2956,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e1ff5259eee462e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab40a55f13114671"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4335,6 +4373,26 @@
         <x:v>Attic investigations</x:v>
       </x:c>
     </x:row>
+    <x:row r="51" ht="34" customHeight="1">
+      <x:c r="A51" s="35" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="B51" s="35" t="str">
+        <x:v>New access point</x:v>
+      </x:c>
+      <x:c r="C51" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="D51" s="35" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E51" s="35" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F51" s="35" t="str">
+        <x:v>Reserved</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
@@ -5327,6 +5385,24 @@
       </x:c>
       <x:c r="F52" s="35" t="str">
         <x:v>draft_lab_cabinet_02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="34" customHeight="1">
+      <x:c r="A53" s="35" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="B53" s="35" t="str">
+        <x:v>New access point</x:v>
+      </x:c>
+      <x:c r="C53" s="35" t="str"/>
+      <x:c r="D53" s="35" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="E53" s="35" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F53" s="35" t="str">
+        <x:v>draft_gallery_detail_01</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5991,7 +6067,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2da99640916b4759"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d3b4212ef594f61"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6801,7 +6877,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64d5735699984ca9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8665164329249e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7314,7 +7390,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re146a52e7f424505"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9813f587aa324fd8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7594,7 +7670,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60d754df694f40a2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2314a63a042a4698"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9017,17 +9093,35 @@
       <x:c r="I48" s="17" t="str"/>
       <x:c r="J48" s="17" t="str"/>
     </x:row>
-    <x:row r="49" ht="32" customHeight="1">
-      <x:c r="A49" s="17"/>
-      <x:c r="B49" s="17"/>
-      <x:c r="C49" s="17"/>
-      <x:c r="D49" s="17"/>
-      <x:c r="E49" s="17"/>
-      <x:c r="F49" s="18"/>
-      <x:c r="G49" s="16"/>
-      <x:c r="H49" s="17"/>
-      <x:c r="I49" s="17"/>
-      <x:c r="J49" s="17"/>
+    <x:row r="49" ht="34" customHeight="1">
+      <x:c r="A49" s="17" t="str">
+        <x:v>gallery_detail_01</x:v>
+      </x:c>
+      <x:c r="B49" s="17" t="str">
+        <x:v>gallery</x:v>
+      </x:c>
+      <x:c r="C49" s="17" t="str">
+        <x:v>authoring</x:v>
+      </x:c>
+      <x:c r="D49" s="17" t="str">
+        <x:v>New access point</x:v>
+      </x:c>
+      <x:c r="E49" s="17" t="str">
+        <x:v>detail</x:v>
+      </x:c>
+      <x:c r="F49" s="18" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G49" s="16" t="str">
+        <x:v>gallery_detail_01_anchor</x:v>
+      </x:c>
+      <x:c r="H49" s="17" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="I49" s="17" t="str">
+        <x:v>Prepared by visual room authoring.</x:v>
+      </x:c>
+      <x:c r="J49" s="17" t="str"/>
     </x:row>
     <x:row r="50" ht="32" customHeight="1">
       <x:c r="A50" s="17"/>
@@ -9197,6 +9291,18 @@
       <x:c r="I63" s="17"/>
       <x:c r="J63" s="17"/>
     </x:row>
+    <x:row r="64" ht="32" customHeight="1">
+      <x:c r="A64" s="17"/>
+      <x:c r="B64" s="17"/>
+      <x:c r="C64" s="17"/>
+      <x:c r="D64" s="17"/>
+      <x:c r="E64" s="17"/>
+      <x:c r="F64" s="18"/>
+      <x:c r="G64" s="16"/>
+      <x:c r="H64" s="17"/>
+      <x:c r="I64" s="17"/>
+      <x:c r="J64" s="17"/>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="H2:H501">
@@ -9208,7 +9314,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a08c94a148f485c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1fae393b591d4665"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9748,7 +9854,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reaed199754c84b3e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R714ef859380e4d27"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9865,7 +9971,7 @@
         <x:v>Prepared locations</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
-        <x:v>Slots lists all 47 validated access points with a human-readable editor_label, room, capacity, type, physical notes, and anchor reference. Keep IDs, anchors, routes, and assets stable. New physical locations require matching geometry and are outside this workbook workflow.</x:v>
+        <x:v>Slots lists all 48 validated access points with a human-readable editor_label, room, capacity, type, physical notes, and anchor reference. Keep IDs, anchors, routes, and assets stable. New physical locations require matching geometry and are outside this workbook workflow.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="58" customHeight="1">
@@ -9985,7 +10091,7 @@
         <x:v>_data/exhibit_slots.csv</x:v>
       </x:c>
       <x:c r="B28" s="24" t="str">
-        <x:v>2d093b6723b5aa46864919db8329a560a6c36333435f1cf40e12018bd6aa4e77</x:v>
+        <x:v>b1168bb22dc797e86e07fea457d1e410e24b9789464eb5d4198025335e43a270</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="58" customHeight="1">

</xml_diff>